<commit_message>
Atualizando planilha de tasks da sprint 2
</commit_message>
<xml_diff>
--- a/DOCS/sprints/sprint-02/TasksSprint2.xlsx
+++ b/DOCS/sprints/sprint-02/TasksSprint2.xlsx
@@ -17,7 +17,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="178" uniqueCount="178">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="176" uniqueCount="176">
   <si>
     <t>ID</t>
   </si>
@@ -196,19 +196,13 @@
     <t xml:space="preserve">Implementar Frontend</t>
   </si>
   <si>
-    <t xml:space="preserve">Desenvolver frontend da página de email.</t>
-  </si>
-  <si>
     <t>DW08.1.3</t>
   </si>
   <si>
-    <t xml:space="preserve">Implementar Backend </t>
+    <t xml:space="preserve">Implementar Backend</t>
   </si>
   <si>
     <t>Validação</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Desenvolver backend da página de email.</t>
   </si>
   <si>
     <t>ES01.1</t>
@@ -734,7 +728,7 @@
   <cellStyleXfs count="1">
     <xf fontId="0" fillId="0" borderId="0" numFmtId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
   </cellStyleXfs>
-  <cellXfs count="48">
+  <cellXfs count="47">
     <xf fontId="0" fillId="0" borderId="0" numFmtId="0" xfId="0"/>
     <xf fontId="0" fillId="0" borderId="0" numFmtId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -772,19 +766,16 @@
     <xf fontId="8" fillId="5" borderId="1" numFmtId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf fontId="5" fillId="2" borderId="0" numFmtId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf fontId="0" fillId="0" borderId="1" numFmtId="0" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf fontId="1" fillId="0" borderId="0" numFmtId="164" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+    <xf fontId="1" fillId="0" borderId="1" numFmtId="164" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf fontId="6" fillId="0" borderId="1" numFmtId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf fontId="1" fillId="0" borderId="0" numFmtId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+    <xf fontId="1" fillId="0" borderId="1" numFmtId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf fontId="6" fillId="6" borderId="1" numFmtId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -832,8 +823,9 @@
       <alignment horizontal="center" vertical="center"/>
       <protection hidden="0" locked="1"/>
     </xf>
-    <xf fontId="1" fillId="7" borderId="1" numFmtId="16" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf fontId="1" fillId="6" borderId="1" numFmtId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
+      <protection hidden="0" locked="1"/>
     </xf>
     <xf fontId="6" fillId="8" borderId="1" numFmtId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -895,6 +887,1265 @@
     </ext>
   </extLst>
 </styleSheet>
+</file>
+
+<file path=xl/charts/chart1.xml><?xml version="1.0" encoding="utf-8"?>
+<c:chartSpace xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart" xmlns:c14="http://schemas.microsoft.com/office/drawing/2007/8/2/chart" xmlns:c16r2="http://schemas.microsoft.com/office/drawing/2015/06/chart">
+  <c:date1904 val="0"/>
+  <c:lang val="en-US"/>
+  <c:roundedCorners val="0"/>
+  <mc:AlternateContent>
+    <mc:Choice Requires="c14">
+      <c14:style val="102"/>
+    </mc:Choice>
+    <mc:Fallback>
+      <c:style val="2"/>
+    </mc:Fallback>
+  </mc:AlternateContent>
+  <c:chart>
+    <c:title>
+      <c:tx>
+        <c:rich>
+          <a:bodyPr/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr sz="1400" b="0" spc="0">
+                <a:solidFill>
+                  <a:schemeClr val="tx1">
+                    <a:lumMod val="65000"/>
+                    <a:lumOff val="35000"/>
+                  </a:schemeClr>
+                </a:solidFill>
+                <a:latin typeface="+mn-lt"/>
+                <a:ea typeface="+mn-ea"/>
+                <a:cs typeface="+mn-cs"/>
+              </a:defRPr>
+            </a:pPr>
+            <a:r>
+              <a:rPr/>
+              <a:t>Sprint 2</a:t>
+            </a:r>
+            <a:endParaRPr/>
+          </a:p>
+        </c:rich>
+      </c:tx>
+      <c:layout/>
+      <c:overlay val="0"/>
+      <c:spPr bwMode="auto">
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:noFill/>
+        <a:ln>
+          <a:noFill/>
+        </a:ln>
+      </c:spPr>
+      <c:txPr>
+        <a:bodyPr/>
+        <a:p>
+          <a:pPr>
+            <a:defRPr sz="1400" b="0" spc="0">
+              <a:solidFill>
+                <a:schemeClr val="tx1">
+                  <a:lumMod val="65000"/>
+                  <a:lumOff val="35000"/>
+                </a:schemeClr>
+              </a:solidFill>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:defRPr>
+          </a:pPr>
+          <a:endParaRPr/>
+        </a:p>
+      </c:txPr>
+    </c:title>
+    <c:autoTitleDeleted val="0"/>
+    <c:plotArea>
+      <c:layout>
+        <c:manualLayout/>
+      </c:layout>
+      <c:lineChart>
+        <c:grouping val="standard"/>
+        <c:varyColors val="0"/>
+        <c:ser>
+          <c:idx val="0"/>
+          <c:order val="0"/>
+          <c:tx>
+            <c:strRef>
+              <c:f>'Sprint 2'!$K$3</c:f>
+              <c:strCache>
+                <c:ptCount val="1"/>
+                <c:pt idx="0">
+                  <c:v>Esforço Ideal</c:v>
+                </c:pt>
+              </c:strCache>
+            </c:strRef>
+          </c:tx>
+          <c:spPr bwMode="auto">
+            <a:prstGeom prst="rect">
+              <a:avLst/>
+            </a:prstGeom>
+            <a:solidFill>
+              <a:schemeClr val="accent1"/>
+            </a:solidFill>
+            <a:ln w="28575" cap="rnd">
+              <a:solidFill>
+                <a:schemeClr val="accent1"/>
+              </a:solidFill>
+              <a:round/>
+            </a:ln>
+          </c:spPr>
+          <c:marker>
+            <c:symbol val="circle"/>
+            <c:size val="5"/>
+            <c:spPr bwMode="auto">
+              <a:prstGeom prst="rect">
+                <a:avLst/>
+              </a:prstGeom>
+              <a:solidFill>
+                <a:schemeClr val="accent1"/>
+              </a:solidFill>
+              <a:ln/>
+            </c:spPr>
+          </c:marker>
+          <c:cat>
+            <c:numRef>
+              <c:f>'Sprint 2'!$J$4:$J$22</c:f>
+              <c:numCache>
+                <c:formatCode>dd/mm;@</c:formatCode>
+                <c:ptCount val="19"/>
+                <c:pt idx="0">
+                  <c:v>46148</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>46149</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>46150</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>46151</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>46152</c:v>
+                </c:pt>
+                <c:pt idx="5">
+                  <c:v>46153</c:v>
+                </c:pt>
+                <c:pt idx="6">
+                  <c:v>46154</c:v>
+                </c:pt>
+                <c:pt idx="7">
+                  <c:v>46155</c:v>
+                </c:pt>
+                <c:pt idx="8">
+                  <c:v>46156</c:v>
+                </c:pt>
+                <c:pt idx="9">
+                  <c:v>46157</c:v>
+                </c:pt>
+                <c:pt idx="10">
+                  <c:v>46158</c:v>
+                </c:pt>
+                <c:pt idx="11">
+                  <c:v>46159</c:v>
+                </c:pt>
+                <c:pt idx="12">
+                  <c:v>46160</c:v>
+                </c:pt>
+                <c:pt idx="13">
+                  <c:v>46161</c:v>
+                </c:pt>
+                <c:pt idx="14">
+                  <c:v>46162</c:v>
+                </c:pt>
+                <c:pt idx="15">
+                  <c:v>46163</c:v>
+                </c:pt>
+                <c:pt idx="16">
+                  <c:v>46164</c:v>
+                </c:pt>
+                <c:pt idx="17">
+                  <c:v>46165</c:v>
+                </c:pt>
+                <c:pt idx="18">
+                  <c:v>46166</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:cat>
+          <c:val>
+            <c:numRef>
+              <c:f>'Sprint 2'!$K$4:$K$22</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="19"/>
+                <c:pt idx="0" formatCode="General">
+                  <c:v>508</c:v>
+                </c:pt>
+                <c:pt idx="1" formatCode="0.00">
+                  <c:v>479.778</c:v>
+                </c:pt>
+                <c:pt idx="2" formatCode="0.00">
+                  <c:v>451.55600000000004</c:v>
+                </c:pt>
+                <c:pt idx="3" formatCode="0.00">
+                  <c:v>423.33400000000006</c:v>
+                </c:pt>
+                <c:pt idx="4" formatCode="0.00">
+                  <c:v>395.1120000000001</c:v>
+                </c:pt>
+                <c:pt idx="5" formatCode="0.00">
+                  <c:v>366.8900000000001</c:v>
+                </c:pt>
+                <c:pt idx="6" formatCode="0.00">
+                  <c:v>338.6680000000001</c:v>
+                </c:pt>
+                <c:pt idx="7" formatCode="0.00">
+                  <c:v>310.44600000000014</c:v>
+                </c:pt>
+                <c:pt idx="8" formatCode="0.00">
+                  <c:v>282.22400000000016</c:v>
+                </c:pt>
+                <c:pt idx="9" formatCode="0.00">
+                  <c:v>254.00200000000015</c:v>
+                </c:pt>
+                <c:pt idx="10" formatCode="0.00">
+                  <c:v>225.78000000000014</c:v>
+                </c:pt>
+                <c:pt idx="11" formatCode="0.00">
+                  <c:v>197.55800000000013</c:v>
+                </c:pt>
+                <c:pt idx="12" formatCode="0.00">
+                  <c:v>169.33600000000013</c:v>
+                </c:pt>
+                <c:pt idx="13" formatCode="0.00">
+                  <c:v>141.11400000000012</c:v>
+                </c:pt>
+                <c:pt idx="14" formatCode="0.00">
+                  <c:v>112.89200000000011</c:v>
+                </c:pt>
+                <c:pt idx="15" formatCode="0.00">
+                  <c:v>84.6700000000001</c:v>
+                </c:pt>
+                <c:pt idx="16" formatCode="0.00">
+                  <c:v>56.4480000000001</c:v>
+                </c:pt>
+                <c:pt idx="17" formatCode="0.00">
+                  <c:v>28.2260000000001</c:v>
+                </c:pt>
+                <c:pt idx="18" formatCode="0.00">
+                  <c:v>0.004000000000097259</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:val>
+          <c:smooth val="0"/>
+        </c:ser>
+        <c:ser>
+          <c:idx val="1"/>
+          <c:order val="1"/>
+          <c:tx>
+            <c:strRef>
+              <c:f>'Sprint 2'!$L$3</c:f>
+              <c:strCache>
+                <c:ptCount val="1"/>
+                <c:pt idx="0">
+                  <c:v>Esforço Real</c:v>
+                </c:pt>
+              </c:strCache>
+            </c:strRef>
+          </c:tx>
+          <c:spPr bwMode="auto">
+            <a:prstGeom prst="rect">
+              <a:avLst/>
+            </a:prstGeom>
+            <a:solidFill>
+              <a:schemeClr val="accent2"/>
+            </a:solidFill>
+            <a:ln w="28575" cap="rnd">
+              <a:solidFill>
+                <a:schemeClr val="accent2"/>
+              </a:solidFill>
+              <a:round/>
+            </a:ln>
+          </c:spPr>
+          <c:marker>
+            <c:symbol val="circle"/>
+            <c:size val="5"/>
+            <c:spPr bwMode="auto">
+              <a:prstGeom prst="rect">
+                <a:avLst/>
+              </a:prstGeom>
+              <a:solidFill>
+                <a:schemeClr val="accent2"/>
+              </a:solidFill>
+              <a:ln/>
+            </c:spPr>
+          </c:marker>
+          <c:cat>
+            <c:numRef>
+              <c:f>'Sprint 2'!$J$4:$J$22</c:f>
+              <c:numCache>
+                <c:formatCode>dd/mm;@</c:formatCode>
+                <c:ptCount val="19"/>
+                <c:pt idx="0">
+                  <c:v>46148</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>46149</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>46150</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>46151</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>46152</c:v>
+                </c:pt>
+                <c:pt idx="5">
+                  <c:v>46153</c:v>
+                </c:pt>
+                <c:pt idx="6">
+                  <c:v>46154</c:v>
+                </c:pt>
+                <c:pt idx="7">
+                  <c:v>46155</c:v>
+                </c:pt>
+                <c:pt idx="8">
+                  <c:v>46156</c:v>
+                </c:pt>
+                <c:pt idx="9">
+                  <c:v>46157</c:v>
+                </c:pt>
+                <c:pt idx="10">
+                  <c:v>46158</c:v>
+                </c:pt>
+                <c:pt idx="11">
+                  <c:v>46159</c:v>
+                </c:pt>
+                <c:pt idx="12">
+                  <c:v>46160</c:v>
+                </c:pt>
+                <c:pt idx="13">
+                  <c:v>46161</c:v>
+                </c:pt>
+                <c:pt idx="14">
+                  <c:v>46162</c:v>
+                </c:pt>
+                <c:pt idx="15">
+                  <c:v>46163</c:v>
+                </c:pt>
+                <c:pt idx="16">
+                  <c:v>46164</c:v>
+                </c:pt>
+                <c:pt idx="17">
+                  <c:v>46165</c:v>
+                </c:pt>
+                <c:pt idx="18">
+                  <c:v>46166</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:cat>
+          <c:val>
+            <c:numRef>
+              <c:f>'Sprint 2'!$L$4:$L$22</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="19"/>
+                <c:pt idx="0">
+                  <c:v>508</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>508</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>508</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>508</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>508</c:v>
+                </c:pt>
+                <c:pt idx="5">
+                  <c:v>508</c:v>
+                </c:pt>
+                <c:pt idx="6">
+                  <c:v>508</c:v>
+                </c:pt>
+                <c:pt idx="7">
+                  <c:v>508</c:v>
+                </c:pt>
+                <c:pt idx="8">
+                  <c:v>508</c:v>
+                </c:pt>
+                <c:pt idx="9">
+                  <c:v>508</c:v>
+                </c:pt>
+                <c:pt idx="10">
+                  <c:v>508</c:v>
+                </c:pt>
+                <c:pt idx="11">
+                  <c:v>508</c:v>
+                </c:pt>
+                <c:pt idx="12">
+                  <c:v>494</c:v>
+                </c:pt>
+                <c:pt idx="13">
+                  <c:v>477</c:v>
+                </c:pt>
+                <c:pt idx="14">
+                  <c:v>477</c:v>
+                </c:pt>
+                <c:pt idx="15">
+                  <c:v>477</c:v>
+                </c:pt>
+                <c:pt idx="18">
+                  <c:v>0</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:val>
+          <c:smooth val="0"/>
+        </c:ser>
+        <c:marker val="1"/>
+        <c:smooth val="0"/>
+        <c:axId val="2140841537"/>
+        <c:axId val="2140841538"/>
+      </c:lineChart>
+      <c:catAx>
+        <c:axId val="2140841537"/>
+        <c:scaling>
+          <c:orientation val="minMax"/>
+        </c:scaling>
+        <c:delete val="0"/>
+        <c:axPos val="b"/>
+        <c:numFmt formatCode="dd/mm;@" sourceLinked="1"/>
+        <c:majorTickMark val="none"/>
+        <c:minorTickMark val="out"/>
+        <c:tickLblPos val="nextTo"/>
+        <c:spPr bwMode="auto">
+          <a:prstGeom prst="rect">
+            <a:avLst/>
+          </a:prstGeom>
+          <a:noFill/>
+          <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+            <a:solidFill>
+              <a:schemeClr val="tx1">
+                <a:lumMod val="15000"/>
+                <a:lumOff val="85000"/>
+              </a:schemeClr>
+            </a:solidFill>
+            <a:round/>
+          </a:ln>
+        </c:spPr>
+        <c:txPr>
+          <a:bodyPr/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr sz="900">
+                <a:solidFill>
+                  <a:schemeClr val="tx1">
+                    <a:lumMod val="65000"/>
+                    <a:lumOff val="35000"/>
+                  </a:schemeClr>
+                </a:solidFill>
+                <a:latin typeface="Calibri"/>
+                <a:ea typeface="Arial"/>
+                <a:cs typeface="Arial"/>
+              </a:defRPr>
+            </a:pPr>
+            <a:endParaRPr/>
+          </a:p>
+        </c:txPr>
+        <c:crossAx val="2140841538"/>
+        <c:crosses val="autoZero"/>
+        <c:auto val="1"/>
+        <c:lblAlgn val="ctr"/>
+        <c:lblOffset val="100"/>
+        <c:noMultiLvlLbl val="0"/>
+      </c:catAx>
+      <c:valAx>
+        <c:axId val="2140841538"/>
+        <c:scaling>
+          <c:orientation val="minMax"/>
+        </c:scaling>
+        <c:delete val="0"/>
+        <c:axPos val="l"/>
+        <c:majorGridlines>
+          <c:spPr bwMode="auto">
+            <a:prstGeom prst="rect">
+              <a:avLst/>
+            </a:prstGeom>
+            <a:noFill/>
+            <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+              <a:solidFill>
+                <a:schemeClr val="tx1">
+                  <a:lumMod val="15000"/>
+                  <a:lumOff val="85000"/>
+                </a:schemeClr>
+              </a:solidFill>
+              <a:round/>
+            </a:ln>
+          </c:spPr>
+        </c:majorGridlines>
+        <c:numFmt formatCode="General" sourceLinked="1"/>
+        <c:majorTickMark val="none"/>
+        <c:minorTickMark val="none"/>
+        <c:tickLblPos val="nextTo"/>
+        <c:spPr bwMode="auto">
+          <a:prstGeom prst="rect">
+            <a:avLst/>
+          </a:prstGeom>
+          <a:noFill/>
+          <a:ln>
+            <a:noFill/>
+          </a:ln>
+        </c:spPr>
+        <c:txPr>
+          <a:bodyPr/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr sz="900">
+                <a:solidFill>
+                  <a:schemeClr val="tx1">
+                    <a:lumMod val="65000"/>
+                    <a:lumOff val="35000"/>
+                  </a:schemeClr>
+                </a:solidFill>
+                <a:latin typeface="Calibri"/>
+                <a:ea typeface="Arial"/>
+                <a:cs typeface="Arial"/>
+              </a:defRPr>
+            </a:pPr>
+            <a:endParaRPr/>
+          </a:p>
+        </c:txPr>
+        <c:crossAx val="2140841537"/>
+        <c:crosses val="autoZero"/>
+        <c:crossBetween val="between"/>
+      </c:valAx>
+      <c:spPr bwMode="auto">
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:noFill/>
+        <a:ln>
+          <a:noFill/>
+        </a:ln>
+      </c:spPr>
+    </c:plotArea>
+    <c:legend>
+      <c:legendPos val="b"/>
+      <c:layout/>
+      <c:overlay val="0"/>
+      <c:spPr bwMode="auto">
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:noFill/>
+        <a:ln>
+          <a:noFill/>
+        </a:ln>
+        <a:effectLst/>
+      </c:spPr>
+      <c:txPr>
+        <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+        <a:lstStyle/>
+        <a:p>
+          <a:pPr>
+            <a:defRPr sz="900">
+              <a:solidFill>
+                <a:schemeClr val="tx1">
+                  <a:lumMod val="65000"/>
+                  <a:lumOff val="35000"/>
+                </a:schemeClr>
+              </a:solidFill>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:defRPr>
+          </a:pPr>
+          <a:endParaRPr lang="en-US"/>
+        </a:p>
+      </c:txPr>
+    </c:legend>
+    <c:plotVisOnly val="1"/>
+    <c:dispBlanksAs val="zero"/>
+    <c:showDLblsOverMax val="0"/>
+  </c:chart>
+  <c:spPr bwMode="auto">
+    <a:xfrm rot="0" flipH="0" flipV="0">
+      <a:off x="28908374" y="257174"/>
+      <a:ext cx="9315450" cy="4543424"/>
+    </a:xfrm>
+    <a:prstGeom prst="rect">
+      <a:avLst/>
+    </a:prstGeom>
+    <a:solidFill>
+      <a:schemeClr val="bg1"/>
+    </a:solidFill>
+    <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+      <a:solidFill>
+        <a:schemeClr val="tx1">
+          <a:lumMod val="15000"/>
+          <a:lumOff val="85000"/>
+        </a:schemeClr>
+      </a:solidFill>
+      <a:round/>
+    </a:ln>
+  </c:spPr>
+  <c:txPr>
+    <a:bodyPr/>
+    <a:p>
+      <a:pPr>
+        <a:defRPr sz="1000">
+          <a:solidFill>
+            <a:schemeClr val="tx1"/>
+          </a:solidFill>
+          <a:latin typeface="+mn-lt"/>
+          <a:ea typeface="+mn-ea"/>
+          <a:cs typeface="+mn-cs"/>
+        </a:defRPr>
+      </a:pPr>
+      <a:endParaRPr/>
+    </a:p>
+  </c:txPr>
+  <c:printSettings>
+    <c:headerFooter/>
+    <c:pageMargins l="0.69999999999999996" r="0.69999999999999996" t="0.75" b="0.75" header="0.29999999999999999" footer="0.29999999999999999"/>
+    <c:pageSetup/>
+  </c:printSettings>
+</c:chartSpace>
+</file>
+
+<file path=xl/charts/colors1.xml><?xml version="1.0" encoding="utf-8"?>
+<cs:colorStyle xmlns:cs="http://schemas.microsoft.com/office/drawing/2012/chartStyle" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" meth="cycle" id="10">
+  <a:schemeClr val="accent1"/>
+  <a:schemeClr val="accent2"/>
+  <a:schemeClr val="accent3"/>
+  <a:schemeClr val="accent4"/>
+  <a:schemeClr val="accent5"/>
+  <a:schemeClr val="accent6"/>
+  <cs:variation/>
+  <cs:variation>
+    <a:lumMod val="60000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="80000"/>
+    <a:lumOff val="20000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="80000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="60000"/>
+    <a:lumOff val="40000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="50000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="70000"/>
+    <a:lumOff val="30000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="70000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="50000"/>
+    <a:lumOff val="50000"/>
+  </cs:variation>
+</cs:colorStyle>
+</file>
+
+<file path=xl/charts/style1.xml><?xml version="1.0" encoding="utf-8"?>
+<cs:chartStyle xmlns:cs="http://schemas.microsoft.com/office/drawing/2012/chartStyle" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" id="227">
+  <cs:axisTitle>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="1000"/>
+  </cs:axisTitle>
+  <cs:categoryAxis>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:spPr bwMode="auto">
+      <a:prstGeom prst="rect">
+        <a:avLst/>
+      </a:prstGeom>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900"/>
+  </cs:categoryAxis>
+  <cs:chartArea>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr bwMode="auto">
+      <a:prstGeom prst="rect">
+        <a:avLst/>
+      </a:prstGeom>
+      <a:solidFill>
+        <a:schemeClr val="bg1"/>
+      </a:solidFill>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="1000"/>
+  </cs:chartArea>
+  <cs:dataLabel>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="75000"/>
+        <a:lumOff val="25000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900"/>
+  </cs:dataLabel>
+  <cs:dataPoint>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="1">
+      <cs:styleClr val="auto"/>
+    </cs:fillRef>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr bwMode="auto">
+      <a:prstGeom prst="rect">
+        <a:avLst/>
+      </a:prstGeom>
+      <a:solidFill>
+        <a:schemeClr val="phClr"/>
+      </a:solidFill>
+    </cs:spPr>
+  </cs:dataPoint>
+  <cs:dataPoint3D>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="1">
+      <cs:styleClr val="auto"/>
+    </cs:fillRef>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr bwMode="auto">
+      <a:prstGeom prst="rect">
+        <a:avLst/>
+      </a:prstGeom>
+      <a:solidFill>
+        <a:schemeClr val="phClr"/>
+      </a:solidFill>
+    </cs:spPr>
+  </cs:dataPoint3D>
+  <cs:dataPointLine>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="1"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr bwMode="auto">
+      <a:prstGeom prst="rect">
+        <a:avLst/>
+      </a:prstGeom>
+      <a:ln w="28575" cap="rnd">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:dataPointLine>
+  <cs:dataPointMarker>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="1">
+      <cs:styleClr val="auto"/>
+    </cs:fillRef>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr bwMode="auto">
+      <a:prstGeom prst="rect">
+        <a:avLst/>
+      </a:prstGeom>
+      <a:solidFill>
+        <a:schemeClr val="phClr"/>
+      </a:solidFill>
+      <a:ln w="9525">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+      </a:ln>
+    </cs:spPr>
+  </cs:dataPointMarker>
+  <cs:dataPointWireframe>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="1"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr bwMode="auto">
+      <a:prstGeom prst="rect">
+        <a:avLst/>
+      </a:prstGeom>
+      <a:ln w="9525" cap="rnd">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:dataPointWireframe>
+  <cs:dataTable>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:spPr bwMode="auto">
+      <a:prstGeom prst="rect">
+        <a:avLst/>
+      </a:prstGeom>
+      <a:noFill/>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900"/>
+  </cs:dataTable>
+  <cs:downBar>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="dk1"/>
+    </cs:fontRef>
+    <cs:spPr bwMode="auto">
+      <a:prstGeom prst="rect">
+        <a:avLst/>
+      </a:prstGeom>
+      <a:solidFill>
+        <a:schemeClr val="dk1">
+          <a:lumMod val="65000"/>
+          <a:lumOff val="35000"/>
+        </a:schemeClr>
+      </a:solidFill>
+      <a:ln w="9525">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="65000"/>
+            <a:lumOff val="35000"/>
+          </a:schemeClr>
+        </a:solidFill>
+      </a:ln>
+    </cs:spPr>
+  </cs:downBar>
+  <cs:dropLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr bwMode="auto">
+      <a:prstGeom prst="rect">
+        <a:avLst/>
+      </a:prstGeom>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="35000"/>
+            <a:lumOff val="65000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:dropLine>
+  <cs:errorBar>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr bwMode="auto">
+      <a:prstGeom prst="rect">
+        <a:avLst/>
+      </a:prstGeom>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="65000"/>
+            <a:lumOff val="35000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:errorBar>
+  <cs:floor>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr bwMode="auto">
+      <a:prstGeom prst="rect">
+        <a:avLst/>
+      </a:prstGeom>
+      <a:noFill/>
+      <a:ln>
+        <a:noFill/>
+      </a:ln>
+    </cs:spPr>
+  </cs:floor>
+  <cs:gridlineMajor>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr bwMode="auto">
+      <a:prstGeom prst="rect">
+        <a:avLst/>
+      </a:prstGeom>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:gridlineMajor>
+  <cs:gridlineMinor>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr bwMode="auto">
+      <a:prstGeom prst="rect">
+        <a:avLst/>
+      </a:prstGeom>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="5000"/>
+            <a:lumOff val="95000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:gridlineMinor>
+  <cs:hiLoLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr bwMode="auto">
+      <a:prstGeom prst="rect">
+        <a:avLst/>
+      </a:prstGeom>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="75000"/>
+            <a:lumOff val="25000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:hiLoLine>
+  <cs:leaderLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr bwMode="auto">
+      <a:prstGeom prst="rect">
+        <a:avLst/>
+      </a:prstGeom>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="35000"/>
+            <a:lumOff val="65000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:leaderLine>
+  <cs:legend>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900"/>
+  </cs:legend>
+  <cs:plotArea>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+  </cs:plotArea>
+  <cs:plotArea3D>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+  </cs:plotArea3D>
+  <cs:seriesAxis>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900"/>
+  </cs:seriesAxis>
+  <cs:seriesLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr bwMode="auto">
+      <a:prstGeom prst="rect">
+        <a:avLst/>
+      </a:prstGeom>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="35000"/>
+            <a:lumOff val="65000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:seriesLine>
+  <cs:title>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="1400" b="0" spc="0"/>
+  </cs:title>
+  <cs:trendline>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr bwMode="auto">
+      <a:prstGeom prst="rect">
+        <a:avLst/>
+      </a:prstGeom>
+      <a:ln w="19050" cap="rnd">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:prstDash val="sysDot"/>
+      </a:ln>
+    </cs:spPr>
+  </cs:trendline>
+  <cs:trendlineLabel>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900"/>
+  </cs:trendlineLabel>
+  <cs:upBar>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="dk1"/>
+    </cs:fontRef>
+    <cs:spPr bwMode="auto">
+      <a:prstGeom prst="rect">
+        <a:avLst/>
+      </a:prstGeom>
+      <a:solidFill>
+        <a:schemeClr val="lt1"/>
+      </a:solidFill>
+      <a:ln w="9525">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+      </a:ln>
+    </cs:spPr>
+  </cs:upBar>
+  <cs:valueAxis>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900"/>
+  </cs:valueAxis>
+  <cs:wall>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr bwMode="auto">
+      <a:prstGeom prst="rect">
+        <a:avLst/>
+      </a:prstGeom>
+      <a:noFill/>
+      <a:ln>
+        <a:noFill/>
+      </a:ln>
+    </cs:spPr>
+  </cs:wall>
+  <cs:dataPointMarkerLayout symbol="circle" size="5"/>
+</cs:chartStyle>
+</file>
+
+<file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
+<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:m="http://schemas.openxmlformats.org/officeDocument/2006/math" xmlns:w="http://schemas.openxmlformats.org/wordprocessingml/2006/main">
+  <xdr:twoCellAnchor editAs="twoCell">
+    <xdr:from>
+      <xdr:col>12</xdr:col>
+      <xdr:colOff>323849</xdr:colOff>
+      <xdr:row>1</xdr:row>
+      <xdr:rowOff>9524</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>27</xdr:col>
+      <xdr:colOff>495299</xdr:colOff>
+      <xdr:row>19</xdr:row>
+      <xdr:rowOff>95249</xdr:rowOff>
+    </xdr:to>
+    <xdr:graphicFrame>
+      <xdr:nvGraphicFramePr>
+        <xdr:cNvPr id="879650156" name=""/>
+        <xdr:cNvGraphicFramePr>
+          <a:graphicFrameLocks xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+        </xdr:cNvGraphicFramePr>
+      </xdr:nvGraphicFramePr>
+      <xdr:xfrm rot="0" flipH="0" flipV="0">
+        <a:off x="28908374" y="257174"/>
+        <a:ext cx="9315450" cy="4543424"/>
+      </xdr:xfrm>
+      <a:graphic>
+        <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
+          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
+        </a:graphicData>
+      </a:graphic>
+    </xdr:graphicFrame>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+</xdr:wsDr>
 </file>
 
 <file path=xl/theme/theme.xml><?xml version="1.0" encoding="utf-8"?>
@@ -1473,33 +2724,33 @@
         <v>28</v>
       </c>
       <c r="H3" s="11"/>
-      <c r="J3" s="13" t="s">
+      <c r="J3" s="7" t="s">
         <v>17</v>
       </c>
-      <c r="K3" s="13" t="s">
+      <c r="K3" s="7" t="s">
         <v>18</v>
       </c>
-      <c r="L3" s="13" t="s">
+      <c r="L3" s="7" t="s">
         <v>19</v>
       </c>
     </row>
     <row r="4" ht="19.5" customHeight="1">
       <c r="A4" s="8"/>
-      <c r="B4" s="14"/>
-      <c r="C4" s="14"/>
-      <c r="D4" s="14"/>
-      <c r="E4" s="14"/>
-      <c r="F4" s="14"/>
-      <c r="G4" s="14"/>
+      <c r="B4" s="13"/>
+      <c r="C4" s="13"/>
+      <c r="D4" s="13"/>
+      <c r="E4" s="13"/>
+      <c r="F4" s="13"/>
+      <c r="G4" s="13"/>
       <c r="H4" s="11"/>
-      <c r="J4" s="15">
+      <c r="J4" s="14">
         <v>46148</v>
       </c>
-      <c r="K4" s="2">
+      <c r="K4" s="11">
         <f>G67</f>
         <v>508</v>
       </c>
-      <c r="L4" s="2">
+      <c r="L4" s="11">
         <f>G67</f>
         <v>508</v>
       </c>
@@ -1523,19 +2774,19 @@
       <c r="F5" s="9" t="s">
         <v>23</v>
       </c>
-      <c r="G5" s="16">
+      <c r="G5" s="15">
         <v>27</v>
       </c>
       <c r="H5" s="11"/>
       <c r="I5" s="1"/>
-      <c r="J5" s="15">
+      <c r="J5" s="14">
         <v>46149</v>
       </c>
-      <c r="K5" s="17">
-        <f>K4-28.222</f>
+      <c r="K5" s="16">
+        <f t="shared" ref="K5:K10" si="0">K4-28.222</f>
         <v>479.77800000000002</v>
       </c>
-      <c r="L5" s="2">
+      <c r="L5" s="11">
         <v>508</v>
       </c>
     </row>
@@ -1563,14 +2814,14 @@
       </c>
       <c r="H6" s="11"/>
       <c r="I6" s="1"/>
-      <c r="J6" s="15">
+      <c r="J6" s="14">
         <v>46150</v>
       </c>
-      <c r="K6" s="17">
-        <f>K5-28.222</f>
+      <c r="K6" s="16">
+        <f t="shared" si="0"/>
         <v>451.55600000000004</v>
       </c>
-      <c r="L6" s="2">
+      <c r="L6" s="11">
         <v>508</v>
       </c>
     </row>
@@ -1584,195 +2835,195 @@
       <c r="G7" s="11"/>
       <c r="H7" s="11"/>
       <c r="I7" s="1"/>
-      <c r="J7" s="15">
+      <c r="J7" s="14">
         <v>46151</v>
       </c>
-      <c r="K7" s="17">
-        <f>K6-28.222</f>
+      <c r="K7" s="16">
+        <f t="shared" si="0"/>
         <v>423.33400000000006</v>
       </c>
-      <c r="L7" s="2">
+      <c r="L7" s="11">
         <v>508</v>
       </c>
     </row>
     <row r="8" ht="19.5" customHeight="1">
-      <c r="A8" s="18" t="s">
+      <c r="A8" s="17" t="s">
         <v>28</v>
       </c>
-      <c r="B8" s="18" t="s">
+      <c r="B8" s="17" t="s">
         <v>29</v>
       </c>
-      <c r="C8" s="18" t="s">
+      <c r="C8" s="17" t="s">
         <v>30</v>
       </c>
-      <c r="D8" s="19" t="s">
+      <c r="D8" s="18" t="s">
         <v>31</v>
       </c>
-      <c r="E8" s="20" t="s">
+      <c r="E8" s="19" t="s">
         <v>32</v>
       </c>
-      <c r="F8" s="18" t="s">
+      <c r="F8" s="17" t="s">
         <v>30</v>
       </c>
-      <c r="G8" s="19">
+      <c r="G8" s="18">
         <v>21</v>
       </c>
-      <c r="H8" s="19"/>
+      <c r="H8" s="18"/>
       <c r="I8" s="1"/>
-      <c r="J8" s="15">
+      <c r="J8" s="14">
         <v>46152</v>
       </c>
-      <c r="K8" s="17">
-        <f>K7-28.222</f>
+      <c r="K8" s="16">
+        <f t="shared" si="0"/>
         <v>395.11200000000008</v>
       </c>
-      <c r="L8" s="2">
+      <c r="L8" s="11">
         <v>508</v>
       </c>
     </row>
     <row r="9" ht="19.5" customHeight="1">
-      <c r="A9" s="21" t="s">
+      <c r="A9" s="20" t="s">
         <v>33</v>
       </c>
-      <c r="B9" s="21" t="s">
+      <c r="B9" s="20" t="s">
         <v>29</v>
       </c>
-      <c r="C9" s="21" t="s">
+      <c r="C9" s="20" t="s">
         <v>34</v>
       </c>
-      <c r="D9" s="22" t="s">
+      <c r="D9" s="21" t="s">
         <v>31</v>
       </c>
-      <c r="E9" s="23" t="s">
+      <c r="E9" s="22" t="s">
         <v>35</v>
       </c>
-      <c r="F9" s="21" t="s">
+      <c r="F9" s="20" t="s">
         <v>30</v>
       </c>
-      <c r="G9" s="22">
+      <c r="G9" s="21">
         <v>5</v>
       </c>
-      <c r="H9" s="24">
+      <c r="H9" s="23">
         <v>46161</v>
       </c>
       <c r="I9" s="1"/>
-      <c r="J9" s="15">
+      <c r="J9" s="14">
         <v>46153</v>
       </c>
-      <c r="K9" s="17">
-        <f>K8-28.222</f>
+      <c r="K9" s="16">
+        <f t="shared" si="0"/>
         <v>366.8900000000001</v>
       </c>
-      <c r="L9" s="2">
+      <c r="L9" s="11">
         <v>508</v>
       </c>
     </row>
     <row r="10" ht="19.5" customHeight="1">
-      <c r="A10" s="21" t="s">
+      <c r="A10" s="20" t="s">
         <v>36</v>
       </c>
-      <c r="B10" s="21" t="s">
+      <c r="B10" s="20" t="s">
         <v>29</v>
       </c>
-      <c r="C10" s="21" t="s">
+      <c r="C10" s="20" t="s">
         <v>37</v>
       </c>
-      <c r="D10" s="22" t="s">
+      <c r="D10" s="21" t="s">
         <v>31</v>
       </c>
-      <c r="E10" s="23" t="s">
+      <c r="E10" s="22" t="s">
         <v>35</v>
       </c>
-      <c r="F10" s="21" t="s">
+      <c r="F10" s="20" t="s">
         <v>30</v>
       </c>
-      <c r="G10" s="22">
+      <c r="G10" s="21">
         <v>5</v>
       </c>
-      <c r="H10" s="24">
+      <c r="H10" s="23">
         <v>46161</v>
       </c>
       <c r="I10" s="1"/>
-      <c r="J10" s="15">
+      <c r="J10" s="14">
         <v>46154</v>
       </c>
-      <c r="K10" s="17">
-        <f>K9-28.222</f>
+      <c r="K10" s="16">
+        <f t="shared" si="0"/>
         <v>338.66800000000012</v>
       </c>
-      <c r="L10" s="2">
+      <c r="L10" s="11">
         <v>508</v>
       </c>
     </row>
     <row r="11" ht="19.5" customHeight="1">
-      <c r="A11" s="18" t="s">
+      <c r="A11" s="17" t="s">
         <v>38</v>
       </c>
-      <c r="B11" s="18" t="s">
+      <c r="B11" s="17" t="s">
         <v>29</v>
       </c>
-      <c r="C11" s="18" t="s">
+      <c r="C11" s="17" t="s">
         <v>39</v>
       </c>
-      <c r="D11" s="19" t="s">
+      <c r="D11" s="18" t="s">
         <v>31</v>
       </c>
-      <c r="E11" s="20" t="s">
+      <c r="E11" s="19" t="s">
         <v>32</v>
       </c>
-      <c r="F11" s="18" t="s">
+      <c r="F11" s="17" t="s">
         <v>30</v>
       </c>
-      <c r="G11" s="19">
+      <c r="G11" s="18">
         <v>6</v>
       </c>
-      <c r="H11" s="19"/>
+      <c r="H11" s="18"/>
       <c r="I11" s="1"/>
-      <c r="J11" s="15">
+      <c r="J11" s="14">
         <v>46155</v>
       </c>
-      <c r="K11" s="17">
-        <f>K10-28.222</f>
+      <c r="K11" s="16">
+        <f t="shared" ref="K11:K22" si="1">K10-28.222</f>
         <v>310.44600000000014</v>
       </c>
-      <c r="L11" s="2">
+      <c r="L11" s="11">
         <v>508</v>
       </c>
     </row>
     <row r="12" ht="19.5" customHeight="1">
-      <c r="A12" s="21" t="s">
+      <c r="A12" s="20" t="s">
         <v>40</v>
       </c>
-      <c r="B12" s="21" t="s">
+      <c r="B12" s="20" t="s">
         <v>29</v>
       </c>
-      <c r="C12" s="21" t="s">
+      <c r="C12" s="20" t="s">
         <v>41</v>
       </c>
-      <c r="D12" s="22" t="s">
+      <c r="D12" s="21" t="s">
         <v>31</v>
       </c>
-      <c r="E12" s="23" t="s">
+      <c r="E12" s="22" t="s">
         <v>35</v>
       </c>
-      <c r="F12" s="21" t="s">
+      <c r="F12" s="20" t="s">
         <v>30</v>
       </c>
-      <c r="G12" s="22">
+      <c r="G12" s="21">
         <v>5</v>
       </c>
-      <c r="H12" s="24">
+      <c r="H12" s="23">
         <v>46161</v>
       </c>
       <c r="I12" s="1"/>
-      <c r="J12" s="15">
+      <c r="J12" s="14">
         <v>46156</v>
       </c>
-      <c r="K12" s="17">
-        <f>K11-28.222</f>
+      <c r="K12" s="16">
+        <f t="shared" si="1"/>
         <v>282.22400000000016</v>
       </c>
-      <c r="L12" s="2">
+      <c r="L12" s="11">
         <v>508</v>
       </c>
     </row>
@@ -1786,49 +3037,49 @@
       <c r="G13" s="11"/>
       <c r="H13" s="11"/>
       <c r="I13" s="1"/>
-      <c r="J13" s="15">
+      <c r="J13" s="14">
         <v>46157</v>
       </c>
-      <c r="K13" s="17">
-        <f>K12-28.222</f>
+      <c r="K13" s="16">
+        <f t="shared" si="1"/>
         <v>254.00200000000015</v>
       </c>
-      <c r="L13" s="2">
+      <c r="L13" s="11">
         <v>508</v>
       </c>
     </row>
     <row r="14" ht="19.5" customHeight="1">
-      <c r="A14" s="20" t="s">
+      <c r="A14" s="19" t="s">
         <v>42</v>
       </c>
-      <c r="B14" s="20" t="s">
+      <c r="B14" s="19" t="s">
         <v>42</v>
       </c>
-      <c r="C14" s="20" t="s">
+      <c r="C14" s="19" t="s">
         <v>43</v>
       </c>
-      <c r="D14" s="20" t="s">
+      <c r="D14" s="19" t="s">
         <v>44</v>
       </c>
-      <c r="E14" s="20" t="s">
+      <c r="E14" s="19" t="s">
         <v>32</v>
       </c>
-      <c r="F14" s="20" t="s">
+      <c r="F14" s="19" t="s">
         <v>45</v>
       </c>
-      <c r="G14" s="19">
+      <c r="G14" s="18">
         <v>34</v>
       </c>
-      <c r="H14" s="19"/>
+      <c r="H14" s="18"/>
       <c r="I14" s="1"/>
-      <c r="J14" s="15">
+      <c r="J14" s="14">
         <v>46158</v>
       </c>
-      <c r="K14" s="17">
-        <f>K13-28.222</f>
+      <c r="K14" s="16">
+        <f t="shared" si="1"/>
         <v>225.78000000000014</v>
       </c>
-      <c r="L14" s="2">
+      <c r="L14" s="11">
         <v>508</v>
       </c>
       <c r="M14" s="1"/>
@@ -1843,14 +3094,14 @@
       <c r="G15" s="11"/>
       <c r="H15" s="11"/>
       <c r="I15" s="1"/>
-      <c r="J15" s="15">
+      <c r="J15" s="14">
         <v>46159</v>
       </c>
-      <c r="K15" s="17">
-        <f>K14-28.222</f>
+      <c r="K15" s="16">
+        <f t="shared" si="1"/>
         <v>197.55800000000013</v>
       </c>
-      <c r="L15" s="2">
+      <c r="L15" s="11">
         <v>508</v>
       </c>
       <c r="M15" s="1"/>
@@ -1879,14 +3130,14 @@
       </c>
       <c r="H16" s="11"/>
       <c r="I16" s="1"/>
-      <c r="J16" s="15">
+      <c r="J16" s="14">
         <v>46160</v>
       </c>
-      <c r="K16" s="17">
-        <f>K15-28.222</f>
+      <c r="K16" s="16">
+        <f t="shared" si="1"/>
         <v>169.33600000000013</v>
       </c>
-      <c r="L16" s="2">
+      <c r="L16" s="11">
         <f>L15-14</f>
         <v>494</v>
       </c>
@@ -1902,51 +3153,51 @@
       <c r="G17" s="11"/>
       <c r="H17" s="11"/>
       <c r="I17" s="1"/>
-      <c r="J17" s="15">
+      <c r="J17" s="14">
         <v>46161</v>
       </c>
-      <c r="K17" s="17">
-        <f>K16-28.222</f>
+      <c r="K17" s="16">
+        <f t="shared" si="1"/>
         <v>141.11400000000012</v>
       </c>
-      <c r="L17" s="2">
+      <c r="L17" s="11">
         <f>L16-17</f>
         <v>477</v>
       </c>
       <c r="M17" s="1"/>
     </row>
     <row r="18" ht="19.5" customHeight="1">
-      <c r="A18" s="20" t="s">
+      <c r="A18" s="19" t="s">
         <v>49</v>
       </c>
-      <c r="B18" s="20" t="s">
+      <c r="B18" s="19" t="s">
         <v>49</v>
       </c>
-      <c r="C18" s="20" t="s">
+      <c r="C18" s="19" t="s">
         <v>50</v>
       </c>
-      <c r="D18" s="20" t="s">
+      <c r="D18" s="19" t="s">
         <v>51</v>
       </c>
-      <c r="E18" s="20" t="s">
+      <c r="E18" s="19" t="s">
         <v>32</v>
       </c>
-      <c r="F18" s="20" t="s">
+      <c r="F18" s="19" t="s">
         <v>52</v>
       </c>
-      <c r="G18" s="19">
+      <c r="G18" s="18">
         <v>55</v>
       </c>
-      <c r="H18" s="19"/>
+      <c r="H18" s="18"/>
       <c r="I18" s="1"/>
-      <c r="J18" s="15">
+      <c r="J18" s="14">
         <v>46162</v>
       </c>
-      <c r="K18" s="17">
-        <f>K17-28.222</f>
+      <c r="K18" s="16">
+        <f t="shared" si="1"/>
         <v>112.89200000000011</v>
       </c>
-      <c r="L18" s="2">
+      <c r="L18" s="11">
         <v>477</v>
       </c>
       <c r="M18" s="1"/>
@@ -1961,116 +3212,118 @@
       <c r="G19" s="11"/>
       <c r="H19" s="11"/>
       <c r="I19" s="1"/>
-      <c r="J19" s="15">
+      <c r="J19" s="14">
         <v>46163</v>
       </c>
-      <c r="K19" s="17">
-        <f>K18-28.222</f>
+      <c r="K19" s="16">
+        <f t="shared" si="1"/>
         <v>84.670000000000101</v>
       </c>
-      <c r="L19" s="2"/>
+      <c r="L19" s="11">
+        <v>477</v>
+      </c>
       <c r="M19" s="1"/>
     </row>
     <row r="20" ht="19.5" customHeight="1">
-      <c r="A20" s="20" t="s">
+      <c r="A20" s="19" t="s">
         <v>53</v>
       </c>
-      <c r="B20" s="20" t="s">
+      <c r="B20" s="19" t="s">
         <v>54</v>
       </c>
-      <c r="C20" s="19" t="s">
+      <c r="C20" s="18" t="s">
         <v>55</v>
       </c>
-      <c r="D20" s="20" t="s">
+      <c r="D20" s="19" t="s">
         <v>44</v>
       </c>
-      <c r="E20" s="20" t="s">
+      <c r="E20" s="19" t="s">
         <v>32</v>
       </c>
-      <c r="F20" s="25" t="s">
+      <c r="F20" s="24" t="s">
         <v>56</v>
       </c>
-      <c r="G20" s="19">
+      <c r="G20" s="18">
         <v>21</v>
       </c>
-      <c r="H20" s="19"/>
+      <c r="H20" s="18"/>
       <c r="I20" s="1"/>
-      <c r="J20" s="15">
+      <c r="J20" s="14">
         <v>46164</v>
       </c>
-      <c r="K20" s="17">
-        <f>K19-28.222</f>
+      <c r="K20" s="16">
+        <f t="shared" si="1"/>
         <v>56.4480000000001</v>
       </c>
-      <c r="L20" s="2"/>
+      <c r="L20" s="11"/>
       <c r="M20" s="1"/>
     </row>
     <row r="21" ht="19.5" customHeight="1">
-      <c r="A21" s="20" t="s">
+      <c r="A21" s="19" t="s">
         <v>57</v>
       </c>
-      <c r="B21" s="20" t="s">
+      <c r="B21" s="19" t="s">
         <v>54</v>
       </c>
-      <c r="C21" s="19" t="s">
+      <c r="C21" s="18" t="s">
         <v>58</v>
       </c>
-      <c r="D21" s="20" t="s">
+      <c r="D21" s="19" t="s">
         <v>51</v>
       </c>
-      <c r="E21" s="20" t="s">
+      <c r="E21" s="19" t="s">
         <v>32</v>
       </c>
-      <c r="F21" s="19" t="s">
+      <c r="F21" s="18" t="s">
+        <v>56</v>
+      </c>
+      <c r="G21" s="18">
+        <v>10</v>
+      </c>
+      <c r="H21" s="18"/>
+      <c r="I21" s="1"/>
+      <c r="J21" s="14">
+        <v>46165</v>
+      </c>
+      <c r="K21" s="16">
+        <f t="shared" si="1"/>
+        <v>28.226000000000099</v>
+      </c>
+      <c r="L21" s="11"/>
+      <c r="M21" s="1"/>
+    </row>
+    <row r="22" ht="19.5" customHeight="1">
+      <c r="A22" s="25" t="s">
         <v>59</v>
       </c>
-      <c r="G21" s="19">
-        <v>10</v>
-      </c>
-      <c r="H21" s="19"/>
-      <c r="I21" s="1"/>
-      <c r="J21" s="15">
-        <v>46165</v>
-      </c>
-      <c r="K21" s="17">
-        <f>K20-28.222</f>
-        <v>28.226000000000099</v>
-      </c>
-      <c r="L21" s="2"/>
-      <c r="M21" s="1"/>
-    </row>
-    <row r="22" ht="19.5" customHeight="1">
-      <c r="A22" s="26" t="s">
+      <c r="B22" s="25" t="s">
+        <v>54</v>
+      </c>
+      <c r="C22" s="26" t="s">
         <v>60</v>
       </c>
-      <c r="B22" s="26" t="s">
-        <v>54</v>
-      </c>
-      <c r="C22" s="27" t="s">
+      <c r="D22" s="25" t="s">
+        <v>26</v>
+      </c>
+      <c r="E22" s="25" t="s">
         <v>61</v>
       </c>
-      <c r="D22" s="26" t="s">
-        <v>26</v>
-      </c>
-      <c r="E22" s="26" t="s">
-        <v>62</v>
-      </c>
-      <c r="F22" s="27" t="s">
-        <v>63</v>
-      </c>
-      <c r="G22" s="27">
+      <c r="F22" s="26" t="s">
+        <v>56</v>
+      </c>
+      <c r="G22" s="26">
         <v>11</v>
       </c>
-      <c r="H22" s="27"/>
+      <c r="H22" s="26"/>
       <c r="I22" s="1"/>
-      <c r="J22" s="15">
+      <c r="J22" s="14">
         <v>46166</v>
       </c>
-      <c r="K22" s="17">
-        <f>K21-28.222</f>
+      <c r="K22" s="16">
+        <f t="shared" si="1"/>
         <v>0.0040000000000972591</v>
       </c>
-      <c r="L22" s="2">
+      <c r="L22" s="11">
         <v>0</v>
       </c>
       <c r="M22" s="1"/>
@@ -2081,7 +3334,7 @@
       <c r="C23" s="11"/>
       <c r="D23" s="9"/>
       <c r="E23" s="9"/>
-      <c r="F23" s="14"/>
+      <c r="F23" s="13"/>
       <c r="G23" s="11"/>
       <c r="H23" s="11"/>
       <c r="I23" s="1"/>
@@ -2091,28 +3344,28 @@
       <c r="M23" s="1"/>
     </row>
     <row r="24" ht="19.5" customHeight="1">
-      <c r="A24" s="23" t="s">
+      <c r="A24" s="22" t="s">
+        <v>62</v>
+      </c>
+      <c r="B24" s="22" t="s">
+        <v>63</v>
+      </c>
+      <c r="C24" s="22" t="s">
         <v>64</v>
       </c>
-      <c r="B24" s="23" t="s">
+      <c r="D24" s="22" t="s">
         <v>65</v>
       </c>
-      <c r="C24" s="23" t="s">
+      <c r="E24" s="22" t="s">
+        <v>35</v>
+      </c>
+      <c r="F24" s="22" t="s">
         <v>66</v>
       </c>
-      <c r="D24" s="23" t="s">
-        <v>67</v>
-      </c>
-      <c r="E24" s="23" t="s">
-        <v>35</v>
-      </c>
-      <c r="F24" s="23" t="s">
-        <v>68</v>
-      </c>
-      <c r="G24" s="22">
+      <c r="G24" s="21">
         <v>2</v>
       </c>
-      <c r="H24" s="28">
+      <c r="H24" s="27">
         <v>46160</v>
       </c>
       <c r="I24" s="1"/>
@@ -2122,28 +3375,28 @@
       <c r="M24" s="1"/>
     </row>
     <row r="25" ht="19.5" customHeight="1">
-      <c r="A25" s="23" t="s">
+      <c r="A25" s="22" t="s">
+        <v>67</v>
+      </c>
+      <c r="B25" s="22" t="s">
+        <v>63</v>
+      </c>
+      <c r="C25" s="22" t="s">
+        <v>68</v>
+      </c>
+      <c r="D25" s="22" t="s">
+        <v>65</v>
+      </c>
+      <c r="E25" s="22" t="s">
+        <v>35</v>
+      </c>
+      <c r="F25" s="22" t="s">
         <v>69</v>
       </c>
-      <c r="B25" s="23" t="s">
-        <v>65</v>
-      </c>
-      <c r="C25" s="23" t="s">
-        <v>70</v>
-      </c>
-      <c r="D25" s="23" t="s">
-        <v>67</v>
-      </c>
-      <c r="E25" s="23" t="s">
-        <v>35</v>
-      </c>
-      <c r="F25" s="23" t="s">
-        <v>71</v>
-      </c>
-      <c r="G25" s="22">
+      <c r="G25" s="21">
         <v>2</v>
       </c>
-      <c r="H25" s="24">
+      <c r="H25" s="23">
         <v>46160</v>
       </c>
       <c r="I25" s="1"/>
@@ -2153,28 +3406,28 @@
       <c r="M25" s="1"/>
     </row>
     <row r="26" ht="19.5" customHeight="1">
-      <c r="A26" s="23" t="s">
+      <c r="A26" s="22" t="s">
+        <v>70</v>
+      </c>
+      <c r="B26" s="22" t="s">
+        <v>63</v>
+      </c>
+      <c r="C26" s="22" t="s">
+        <v>71</v>
+      </c>
+      <c r="D26" s="22" t="s">
+        <v>65</v>
+      </c>
+      <c r="E26" s="22" t="s">
+        <v>35</v>
+      </c>
+      <c r="F26" s="22" t="s">
         <v>72</v>
       </c>
-      <c r="B26" s="23" t="s">
-        <v>65</v>
-      </c>
-      <c r="C26" s="23" t="s">
-        <v>73</v>
-      </c>
-      <c r="D26" s="23" t="s">
-        <v>67</v>
-      </c>
-      <c r="E26" s="23" t="s">
-        <v>35</v>
-      </c>
-      <c r="F26" s="23" t="s">
-        <v>74</v>
-      </c>
-      <c r="G26" s="22">
+      <c r="G26" s="21">
         <v>2</v>
       </c>
-      <c r="H26" s="24">
+      <c r="H26" s="23">
         <v>46160</v>
       </c>
       <c r="I26" s="1"/>
@@ -2184,28 +3437,28 @@
       <c r="M26" s="1"/>
     </row>
     <row r="27" ht="19.5" customHeight="1">
-      <c r="A27" s="26" t="s">
+      <c r="A27" s="25" t="s">
+        <v>73</v>
+      </c>
+      <c r="B27" s="25" t="s">
+        <v>63</v>
+      </c>
+      <c r="C27" s="25" t="s">
+        <v>74</v>
+      </c>
+      <c r="D27" s="25" t="s">
+        <v>65</v>
+      </c>
+      <c r="E27" s="25" t="s">
+        <v>61</v>
+      </c>
+      <c r="F27" s="25" t="s">
         <v>75</v>
       </c>
-      <c r="B27" s="26" t="s">
-        <v>65</v>
-      </c>
-      <c r="C27" s="26" t="s">
-        <v>76</v>
-      </c>
-      <c r="D27" s="26" t="s">
-        <v>67</v>
-      </c>
-      <c r="E27" s="26" t="s">
-        <v>62</v>
-      </c>
-      <c r="F27" s="26" t="s">
-        <v>77</v>
-      </c>
-      <c r="G27" s="27">
+      <c r="G27" s="26">
         <v>2</v>
       </c>
-      <c r="H27" s="27"/>
+      <c r="H27" s="26"/>
       <c r="I27" s="1"/>
       <c r="J27" s="1"/>
       <c r="K27" s="1"/>
@@ -2213,28 +3466,28 @@
       <c r="M27" s="1"/>
     </row>
     <row r="28" ht="19.5" customHeight="1">
-      <c r="A28" s="26" t="s">
+      <c r="A28" s="25" t="s">
+        <v>76</v>
+      </c>
+      <c r="B28" s="28" t="s">
+        <v>63</v>
+      </c>
+      <c r="C28" s="25" t="s">
+        <v>77</v>
+      </c>
+      <c r="D28" s="25" t="s">
+        <v>65</v>
+      </c>
+      <c r="E28" s="25" t="s">
+        <v>61</v>
+      </c>
+      <c r="F28" s="25" t="s">
         <v>78</v>
       </c>
-      <c r="B28" s="29" t="s">
-        <v>65</v>
-      </c>
-      <c r="C28" s="26" t="s">
-        <v>79</v>
-      </c>
-      <c r="D28" s="26" t="s">
-        <v>67</v>
-      </c>
-      <c r="E28" s="26" t="s">
-        <v>62</v>
-      </c>
-      <c r="F28" s="26" t="s">
-        <v>80</v>
-      </c>
-      <c r="G28" s="27">
+      <c r="G28" s="26">
         <v>2</v>
       </c>
-      <c r="H28" s="27"/>
+      <c r="H28" s="26"/>
       <c r="I28" s="1"/>
       <c r="J28" s="1"/>
       <c r="K28" s="1"/>
@@ -2242,28 +3495,28 @@
       <c r="M28" s="1"/>
     </row>
     <row r="29" ht="19.5" customHeight="1">
-      <c r="A29" s="26" t="s">
+      <c r="A29" s="25" t="s">
+        <v>79</v>
+      </c>
+      <c r="B29" s="28" t="s">
+        <v>63</v>
+      </c>
+      <c r="C29" s="25" t="s">
+        <v>80</v>
+      </c>
+      <c r="D29" s="25" t="s">
+        <v>65</v>
+      </c>
+      <c r="E29" s="25" t="s">
+        <v>61</v>
+      </c>
+      <c r="F29" s="25" t="s">
         <v>81</v>
       </c>
-      <c r="B29" s="29" t="s">
-        <v>65</v>
-      </c>
-      <c r="C29" s="26" t="s">
-        <v>82</v>
-      </c>
-      <c r="D29" s="26" t="s">
-        <v>67</v>
-      </c>
-      <c r="E29" s="26" t="s">
-        <v>62</v>
-      </c>
-      <c r="F29" s="26" t="s">
-        <v>83</v>
-      </c>
-      <c r="G29" s="27">
+      <c r="G29" s="26">
         <v>2</v>
       </c>
-      <c r="H29" s="27"/>
+      <c r="H29" s="26"/>
       <c r="I29" s="1"/>
       <c r="J29" s="1"/>
       <c r="K29" s="1"/>
@@ -2271,28 +3524,28 @@
       <c r="M29" s="1"/>
     </row>
     <row r="30" ht="19.5" customHeight="1">
-      <c r="A30" s="26" t="s">
+      <c r="A30" s="25" t="s">
+        <v>82</v>
+      </c>
+      <c r="B30" s="28" t="s">
+        <v>63</v>
+      </c>
+      <c r="C30" s="25" t="s">
+        <v>83</v>
+      </c>
+      <c r="D30" s="25" t="s">
+        <v>65</v>
+      </c>
+      <c r="E30" s="25" t="s">
+        <v>61</v>
+      </c>
+      <c r="F30" s="25" t="s">
         <v>84</v>
       </c>
-      <c r="B30" s="29" t="s">
-        <v>65</v>
-      </c>
-      <c r="C30" s="26" t="s">
-        <v>85</v>
-      </c>
-      <c r="D30" s="26" t="s">
-        <v>67</v>
-      </c>
-      <c r="E30" s="26" t="s">
-        <v>62</v>
-      </c>
-      <c r="F30" s="26" t="s">
-        <v>86</v>
-      </c>
-      <c r="G30" s="27">
+      <c r="G30" s="26">
         <v>2</v>
       </c>
-      <c r="H30" s="27"/>
+      <c r="H30" s="26"/>
       <c r="I30" s="1"/>
       <c r="J30" s="1"/>
       <c r="K30" s="1"/>
@@ -2300,28 +3553,28 @@
       <c r="M30" s="1"/>
     </row>
     <row r="31" ht="19.5" customHeight="1">
-      <c r="A31" s="23" t="s">
+      <c r="A31" s="22" t="s">
+        <v>85</v>
+      </c>
+      <c r="B31" s="29" t="s">
+        <v>63</v>
+      </c>
+      <c r="C31" s="22" t="s">
+        <v>86</v>
+      </c>
+      <c r="D31" s="22" t="s">
+        <v>65</v>
+      </c>
+      <c r="E31" s="22" t="s">
+        <v>35</v>
+      </c>
+      <c r="F31" s="22" t="s">
         <v>87</v>
       </c>
-      <c r="B31" s="30" t="s">
-        <v>65</v>
-      </c>
-      <c r="C31" s="23" t="s">
-        <v>88</v>
-      </c>
-      <c r="D31" s="23" t="s">
-        <v>67</v>
-      </c>
-      <c r="E31" s="23" t="s">
-        <v>35</v>
-      </c>
-      <c r="F31" s="23" t="s">
-        <v>89</v>
-      </c>
-      <c r="G31" s="22">
+      <c r="G31" s="21">
         <v>2</v>
       </c>
-      <c r="H31" s="24">
+      <c r="H31" s="23">
         <v>46160</v>
       </c>
       <c r="I31" s="1"/>
@@ -2331,28 +3584,28 @@
       <c r="M31" s="1"/>
     </row>
     <row r="32" ht="19.5" customHeight="1">
-      <c r="A32" s="23" t="s">
+      <c r="A32" s="22" t="s">
+        <v>88</v>
+      </c>
+      <c r="B32" s="29" t="s">
+        <v>63</v>
+      </c>
+      <c r="C32" s="22" t="s">
+        <v>89</v>
+      </c>
+      <c r="D32" s="22" t="s">
+        <v>65</v>
+      </c>
+      <c r="E32" s="22" t="s">
+        <v>35</v>
+      </c>
+      <c r="F32" s="22" t="s">
         <v>90</v>
       </c>
-      <c r="B32" s="30" t="s">
-        <v>65</v>
-      </c>
-      <c r="C32" s="23" t="s">
-        <v>91</v>
-      </c>
-      <c r="D32" s="23" t="s">
-        <v>67</v>
-      </c>
-      <c r="E32" s="23" t="s">
-        <v>35</v>
-      </c>
-      <c r="F32" s="23" t="s">
-        <v>92</v>
-      </c>
-      <c r="G32" s="22">
+      <c r="G32" s="21">
         <v>2</v>
       </c>
-      <c r="H32" s="24">
+      <c r="H32" s="23">
         <v>46160</v>
       </c>
       <c r="I32" s="1"/>
@@ -2362,28 +3615,28 @@
       <c r="M32" s="1"/>
     </row>
     <row r="33" ht="19.5" customHeight="1">
-      <c r="A33" s="23" t="s">
+      <c r="A33" s="22" t="s">
+        <v>91</v>
+      </c>
+      <c r="B33" s="29" t="s">
+        <v>63</v>
+      </c>
+      <c r="C33" s="22" t="s">
+        <v>92</v>
+      </c>
+      <c r="D33" s="22" t="s">
+        <v>65</v>
+      </c>
+      <c r="E33" s="22" t="s">
+        <v>35</v>
+      </c>
+      <c r="F33" s="22" t="s">
         <v>93</v>
       </c>
-      <c r="B33" s="30" t="s">
-        <v>65</v>
-      </c>
-      <c r="C33" s="23" t="s">
-        <v>94</v>
-      </c>
-      <c r="D33" s="23" t="s">
-        <v>67</v>
-      </c>
-      <c r="E33" s="23" t="s">
-        <v>35</v>
-      </c>
-      <c r="F33" s="23" t="s">
-        <v>95</v>
-      </c>
-      <c r="G33" s="22">
+      <c r="G33" s="21">
         <v>2</v>
       </c>
-      <c r="H33" s="24">
+      <c r="H33" s="23">
         <v>46160</v>
       </c>
       <c r="I33" s="1"/>
@@ -2393,28 +3646,28 @@
       <c r="M33" s="1"/>
     </row>
     <row r="34" ht="19.5" customHeight="1">
-      <c r="A34" s="23" t="s">
+      <c r="A34" s="22" t="s">
+        <v>94</v>
+      </c>
+      <c r="B34" s="22" t="s">
+        <v>63</v>
+      </c>
+      <c r="C34" s="22" t="s">
+        <v>95</v>
+      </c>
+      <c r="D34" s="22" t="s">
+        <v>65</v>
+      </c>
+      <c r="E34" s="22" t="s">
+        <v>35</v>
+      </c>
+      <c r="F34" s="22" t="s">
         <v>96</v>
       </c>
-      <c r="B34" s="23" t="s">
-        <v>65</v>
-      </c>
-      <c r="C34" s="23" t="s">
-        <v>97</v>
-      </c>
-      <c r="D34" s="23" t="s">
-        <v>67</v>
-      </c>
-      <c r="E34" s="23" t="s">
-        <v>35</v>
-      </c>
-      <c r="F34" s="23" t="s">
-        <v>98</v>
-      </c>
-      <c r="G34" s="22">
+      <c r="G34" s="21">
         <v>2</v>
       </c>
-      <c r="H34" s="28">
+      <c r="H34" s="27">
         <v>46160</v>
       </c>
       <c r="I34" s="1"/>
@@ -2425,22 +3678,22 @@
     </row>
     <row r="35" ht="19.5" customHeight="1">
       <c r="A35" s="9" t="s">
+        <v>97</v>
+      </c>
+      <c r="B35" s="30" t="s">
+        <v>63</v>
+      </c>
+      <c r="C35" s="9" t="s">
+        <v>98</v>
+      </c>
+      <c r="D35" s="9" t="s">
         <v>99</v>
-      </c>
-      <c r="B35" s="31" t="s">
-        <v>65</v>
-      </c>
-      <c r="C35" s="9" t="s">
-        <v>100</v>
-      </c>
-      <c r="D35" s="9" t="s">
-        <v>101</v>
       </c>
       <c r="E35" s="10" t="s">
         <v>12</v>
       </c>
       <c r="F35" s="9" t="s">
-        <v>102</v>
+        <v>100</v>
       </c>
       <c r="G35" s="11">
         <v>2</v>
@@ -2453,28 +3706,28 @@
       <c r="M35" s="1"/>
     </row>
     <row r="36" ht="19.5" customHeight="1">
-      <c r="A36" s="23" t="s">
+      <c r="A36" s="22" t="s">
+        <v>101</v>
+      </c>
+      <c r="B36" s="29" t="s">
+        <v>63</v>
+      </c>
+      <c r="C36" s="22" t="s">
+        <v>102</v>
+      </c>
+      <c r="D36" s="22" t="s">
+        <v>99</v>
+      </c>
+      <c r="E36" s="22" t="s">
+        <v>35</v>
+      </c>
+      <c r="F36" s="22" t="s">
         <v>103</v>
       </c>
-      <c r="B36" s="30" t="s">
-        <v>65</v>
-      </c>
-      <c r="C36" s="23" t="s">
-        <v>104</v>
-      </c>
-      <c r="D36" s="23" t="s">
-        <v>101</v>
-      </c>
-      <c r="E36" s="23" t="s">
-        <v>35</v>
-      </c>
-      <c r="F36" s="23" t="s">
-        <v>105</v>
-      </c>
-      <c r="G36" s="22">
+      <c r="G36" s="21">
         <v>2</v>
       </c>
-      <c r="H36" s="32">
+      <c r="H36" s="27">
         <v>46161</v>
       </c>
       <c r="I36" s="1"/>
@@ -2484,28 +3737,28 @@
       <c r="M36" s="1"/>
     </row>
     <row r="37" ht="19.5" customHeight="1">
-      <c r="A37" s="9" t="s">
+      <c r="A37" s="19" t="s">
+        <v>104</v>
+      </c>
+      <c r="B37" s="31" t="s">
+        <v>63</v>
+      </c>
+      <c r="C37" s="19" t="s">
+        <v>105</v>
+      </c>
+      <c r="D37" s="19" t="s">
+        <v>99</v>
+      </c>
+      <c r="E37" s="19" t="s">
+        <v>32</v>
+      </c>
+      <c r="F37" s="19" t="s">
         <v>106</v>
       </c>
-      <c r="B37" s="31" t="s">
-        <v>65</v>
-      </c>
-      <c r="C37" s="9" t="s">
-        <v>107</v>
-      </c>
-      <c r="D37" s="9" t="s">
-        <v>101</v>
-      </c>
-      <c r="E37" s="10" t="s">
-        <v>12</v>
-      </c>
-      <c r="F37" s="9" t="s">
-        <v>108</v>
-      </c>
-      <c r="G37" s="11">
+      <c r="G37" s="18">
         <v>2</v>
       </c>
-      <c r="H37" s="11"/>
+      <c r="H37" s="18"/>
       <c r="I37" s="1"/>
       <c r="J37" s="1"/>
       <c r="K37" s="1"/>
@@ -2514,22 +3767,22 @@
     </row>
     <row r="38" ht="19.5" customHeight="1">
       <c r="A38" s="9" t="s">
+        <v>107</v>
+      </c>
+      <c r="B38" s="30" t="s">
+        <v>63</v>
+      </c>
+      <c r="C38" s="9" t="s">
+        <v>108</v>
+      </c>
+      <c r="D38" s="9" t="s">
         <v>109</v>
-      </c>
-      <c r="B38" s="31" t="s">
-        <v>65</v>
-      </c>
-      <c r="C38" s="9" t="s">
-        <v>110</v>
-      </c>
-      <c r="D38" s="9" t="s">
-        <v>111</v>
       </c>
       <c r="E38" s="10" t="s">
         <v>12</v>
       </c>
       <c r="F38" s="9" t="s">
-        <v>112</v>
+        <v>110</v>
       </c>
       <c r="G38" s="11">
         <v>2</v>
@@ -2542,28 +3795,28 @@
       <c r="M38" s="1"/>
     </row>
     <row r="39" ht="19.5" customHeight="1">
-      <c r="A39" s="26" t="s">
+      <c r="A39" s="25" t="s">
+        <v>111</v>
+      </c>
+      <c r="B39" s="25" t="s">
+        <v>63</v>
+      </c>
+      <c r="C39" s="25" t="s">
+        <v>112</v>
+      </c>
+      <c r="D39" s="25" t="s">
         <v>113</v>
       </c>
-      <c r="B39" s="26" t="s">
-        <v>65</v>
-      </c>
-      <c r="C39" s="26" t="s">
+      <c r="E39" s="25" t="s">
+        <v>61</v>
+      </c>
+      <c r="F39" s="25" t="s">
         <v>114</v>
       </c>
-      <c r="D39" s="26" t="s">
-        <v>115</v>
-      </c>
-      <c r="E39" s="26" t="s">
-        <v>62</v>
-      </c>
-      <c r="F39" s="26" t="s">
-        <v>116</v>
-      </c>
-      <c r="G39" s="27">
+      <c r="G39" s="26">
         <v>2</v>
       </c>
-      <c r="H39" s="27"/>
+      <c r="H39" s="26"/>
       <c r="I39" s="1"/>
       <c r="J39" s="1"/>
       <c r="K39" s="1"/>
@@ -2586,28 +3839,28 @@
       <c r="M40" s="1"/>
     </row>
     <row r="41" ht="19.5" customHeight="1">
-      <c r="A41" s="9" t="s">
+      <c r="A41" s="19" t="s">
+        <v>115</v>
+      </c>
+      <c r="B41" s="19" t="s">
+        <v>63</v>
+      </c>
+      <c r="C41" s="18" t="s">
+        <v>116</v>
+      </c>
+      <c r="D41" s="19" t="s">
+        <v>113</v>
+      </c>
+      <c r="E41" s="19" t="s">
+        <v>32</v>
+      </c>
+      <c r="F41" s="18" t="s">
         <v>117</v>
       </c>
-      <c r="B41" s="9" t="s">
-        <v>65</v>
-      </c>
-      <c r="C41" s="11" t="s">
-        <v>118</v>
-      </c>
-      <c r="D41" s="9" t="s">
-        <v>115</v>
-      </c>
-      <c r="E41" s="10" t="s">
-        <v>12</v>
-      </c>
-      <c r="F41" s="11" t="s">
-        <v>119</v>
-      </c>
-      <c r="G41" s="11">
+      <c r="G41" s="18">
         <v>2</v>
       </c>
-      <c r="H41" s="11"/>
+      <c r="H41" s="18"/>
       <c r="I41" s="1"/>
       <c r="J41" s="1"/>
       <c r="K41" s="1"/>
@@ -2615,28 +3868,28 @@
       <c r="M41" s="1"/>
     </row>
     <row r="42" ht="19.5" customHeight="1">
-      <c r="A42" s="9" t="s">
+      <c r="A42" s="19" t="s">
+        <v>118</v>
+      </c>
+      <c r="B42" s="19" t="s">
+        <v>63</v>
+      </c>
+      <c r="C42" s="19" t="s">
+        <v>119</v>
+      </c>
+      <c r="D42" s="19" t="s">
+        <v>113</v>
+      </c>
+      <c r="E42" s="19" t="s">
+        <v>32</v>
+      </c>
+      <c r="F42" s="19" t="s">
         <v>120</v>
       </c>
-      <c r="B42" s="9" t="s">
-        <v>65</v>
-      </c>
-      <c r="C42" s="9" t="s">
-        <v>121</v>
-      </c>
-      <c r="D42" s="9" t="s">
-        <v>115</v>
-      </c>
-      <c r="E42" s="10" t="s">
-        <v>12</v>
-      </c>
-      <c r="F42" s="9" t="s">
-        <v>122</v>
-      </c>
-      <c r="G42" s="11">
+      <c r="G42" s="18">
         <v>0.69999999999999996</v>
       </c>
-      <c r="H42" s="11"/>
+      <c r="H42" s="18"/>
       <c r="I42" s="1"/>
       <c r="J42" s="1"/>
       <c r="K42" s="1"/>
@@ -2644,28 +3897,28 @@
       <c r="M42" s="1"/>
     </row>
     <row r="43" ht="19.5" customHeight="1">
-      <c r="A43" s="9" t="s">
+      <c r="A43" s="19" t="s">
+        <v>121</v>
+      </c>
+      <c r="B43" s="19" t="s">
+        <v>63</v>
+      </c>
+      <c r="C43" s="19" t="s">
+        <v>122</v>
+      </c>
+      <c r="D43" s="19" t="s">
+        <v>113</v>
+      </c>
+      <c r="E43" s="19" t="s">
+        <v>32</v>
+      </c>
+      <c r="F43" s="19" t="s">
         <v>123</v>
       </c>
-      <c r="B43" s="9" t="s">
-        <v>65</v>
-      </c>
-      <c r="C43" s="9" t="s">
-        <v>124</v>
-      </c>
-      <c r="D43" s="9" t="s">
-        <v>115</v>
-      </c>
-      <c r="E43" s="10" t="s">
-        <v>12</v>
-      </c>
-      <c r="F43" s="9" t="s">
-        <v>125</v>
-      </c>
-      <c r="G43" s="11">
+      <c r="G43" s="18">
         <v>0.69999999999999996</v>
       </c>
-      <c r="H43" s="11"/>
+      <c r="H43" s="18"/>
       <c r="I43" s="1"/>
       <c r="J43" s="1"/>
       <c r="K43" s="1"/>
@@ -2673,28 +3926,28 @@
       <c r="M43" s="1"/>
     </row>
     <row r="44" ht="19.5" customHeight="1">
-      <c r="A44" s="9" t="s">
+      <c r="A44" s="19" t="s">
+        <v>124</v>
+      </c>
+      <c r="B44" s="19" t="s">
+        <v>63</v>
+      </c>
+      <c r="C44" s="19" t="s">
+        <v>125</v>
+      </c>
+      <c r="D44" s="19" t="s">
+        <v>113</v>
+      </c>
+      <c r="E44" s="19" t="s">
+        <v>32</v>
+      </c>
+      <c r="F44" s="19" t="s">
         <v>126</v>
       </c>
-      <c r="B44" s="9" t="s">
-        <v>65</v>
-      </c>
-      <c r="C44" s="9" t="s">
-        <v>127</v>
-      </c>
-      <c r="D44" s="9" t="s">
-        <v>115</v>
-      </c>
-      <c r="E44" s="10" t="s">
-        <v>12</v>
-      </c>
-      <c r="F44" s="9" t="s">
-        <v>128</v>
-      </c>
-      <c r="G44" s="11">
+      <c r="G44" s="18">
         <v>0.59999999999999998</v>
       </c>
-      <c r="H44" s="11"/>
+      <c r="H44" s="18"/>
       <c r="I44" s="1"/>
       <c r="J44" s="1"/>
       <c r="K44" s="1"/>
@@ -2718,22 +3971,22 @@
     </row>
     <row r="46" ht="19.5" customHeight="1">
       <c r="A46" s="11" t="s">
+        <v>127</v>
+      </c>
+      <c r="B46" s="11" t="s">
+        <v>127</v>
+      </c>
+      <c r="C46" s="15" t="s">
+        <v>128</v>
+      </c>
+      <c r="D46" s="9" t="s">
         <v>129</v>
-      </c>
-      <c r="B46" s="11" t="s">
-        <v>129</v>
-      </c>
-      <c r="C46" s="16" t="s">
-        <v>130</v>
-      </c>
-      <c r="D46" s="9" t="s">
-        <v>131</v>
       </c>
       <c r="E46" s="10" t="s">
         <v>12</v>
       </c>
-      <c r="F46" s="16" t="s">
-        <v>132</v>
+      <c r="F46" s="15" t="s">
+        <v>130</v>
       </c>
       <c r="G46" s="11">
         <v>21</v>
@@ -2748,10 +4001,10 @@
     <row r="47" ht="19.5" customHeight="1">
       <c r="A47" s="11"/>
       <c r="B47" s="11"/>
-      <c r="C47" s="16"/>
+      <c r="C47" s="15"/>
       <c r="D47" s="11"/>
       <c r="E47" s="9"/>
-      <c r="F47" s="16"/>
+      <c r="F47" s="15"/>
       <c r="G47" s="11"/>
       <c r="H47" s="11"/>
       <c r="I47" s="1"/>
@@ -2762,13 +4015,13 @@
     </row>
     <row r="48" ht="19.5" customHeight="1">
       <c r="A48" s="9" t="s">
-        <v>133</v>
+        <v>131</v>
       </c>
       <c r="B48" s="9" t="s">
-        <v>133</v>
+        <v>131</v>
       </c>
       <c r="C48" s="9" t="s">
-        <v>134</v>
+        <v>132</v>
       </c>
       <c r="D48" s="9" t="s">
         <v>44</v>
@@ -2777,7 +4030,7 @@
         <v>12</v>
       </c>
       <c r="F48" s="9" t="s">
-        <v>135</v>
+        <v>133</v>
       </c>
       <c r="G48" s="11">
         <v>34</v>
@@ -2805,28 +4058,28 @@
       <c r="M49" s="1"/>
     </row>
     <row r="50" ht="19.5" customHeight="1">
-      <c r="A50" s="26" t="s">
+      <c r="A50" s="25" t="s">
+        <v>134</v>
+      </c>
+      <c r="B50" s="25" t="s">
+        <v>135</v>
+      </c>
+      <c r="C50" s="25" t="s">
         <v>136</v>
       </c>
-      <c r="B50" s="26" t="s">
+      <c r="D50" s="25" t="s">
+        <v>129</v>
+      </c>
+      <c r="E50" s="25" t="s">
+        <v>61</v>
+      </c>
+      <c r="F50" s="25" t="s">
         <v>137</v>
       </c>
-      <c r="C50" s="26" t="s">
-        <v>138</v>
-      </c>
-      <c r="D50" s="26" t="s">
-        <v>131</v>
-      </c>
-      <c r="E50" s="26" t="s">
-        <v>62</v>
-      </c>
-      <c r="F50" s="26" t="s">
-        <v>139</v>
-      </c>
-      <c r="G50" s="27">
+      <c r="G50" s="26">
         <v>17</v>
       </c>
-      <c r="H50" s="27"/>
+      <c r="H50" s="26"/>
       <c r="I50" s="1"/>
       <c r="J50" s="1"/>
       <c r="K50" s="1"/>
@@ -2834,28 +4087,28 @@
       <c r="M50" s="1"/>
     </row>
     <row r="51" ht="19.5" customHeight="1">
-      <c r="A51" s="26" t="s">
+      <c r="A51" s="25" t="s">
+        <v>138</v>
+      </c>
+      <c r="B51" s="25" t="s">
+        <v>135</v>
+      </c>
+      <c r="C51" s="25" t="s">
+        <v>139</v>
+      </c>
+      <c r="D51" s="25" t="s">
+        <v>129</v>
+      </c>
+      <c r="E51" s="25" t="s">
+        <v>61</v>
+      </c>
+      <c r="F51" s="25" t="s">
         <v>140</v>
       </c>
-      <c r="B51" s="26" t="s">
-        <v>137</v>
-      </c>
-      <c r="C51" s="26" t="s">
-        <v>141</v>
-      </c>
-      <c r="D51" s="26" t="s">
-        <v>131</v>
-      </c>
-      <c r="E51" s="26" t="s">
-        <v>62</v>
-      </c>
-      <c r="F51" s="26" t="s">
-        <v>142</v>
-      </c>
-      <c r="G51" s="27">
+      <c r="G51" s="26">
         <v>17</v>
       </c>
-      <c r="H51" s="27"/>
+      <c r="H51" s="26"/>
       <c r="I51" s="1"/>
       <c r="J51" s="1"/>
       <c r="K51" s="1"/>
@@ -2863,28 +4116,28 @@
       <c r="M51" s="1"/>
     </row>
     <row r="52" ht="19.5" customHeight="1">
-      <c r="A52" s="20" t="s">
+      <c r="A52" s="19" t="s">
+        <v>141</v>
+      </c>
+      <c r="B52" s="19" t="s">
+        <v>135</v>
+      </c>
+      <c r="C52" s="19" t="s">
+        <v>142</v>
+      </c>
+      <c r="D52" s="19" t="s">
+        <v>26</v>
+      </c>
+      <c r="E52" s="19" t="s">
+        <v>32</v>
+      </c>
+      <c r="F52" s="19" t="s">
         <v>143</v>
       </c>
-      <c r="B52" s="20" t="s">
-        <v>137</v>
-      </c>
-      <c r="C52" s="20" t="s">
-        <v>144</v>
-      </c>
-      <c r="D52" s="20" t="s">
-        <v>26</v>
-      </c>
-      <c r="E52" s="20" t="s">
-        <v>32</v>
-      </c>
-      <c r="F52" s="20" t="s">
-        <v>145</v>
-      </c>
-      <c r="G52" s="19">
+      <c r="G52" s="18">
         <v>17</v>
       </c>
-      <c r="H52" s="19"/>
+      <c r="H52" s="18"/>
       <c r="I52" s="1"/>
       <c r="J52" s="1"/>
       <c r="K52" s="1"/>
@@ -2902,76 +4155,76 @@
       <c r="H53" s="11"/>
     </row>
     <row r="54" ht="19.5" customHeight="1">
-      <c r="A54" s="33" t="s">
+      <c r="A54" s="32" t="s">
+        <v>144</v>
+      </c>
+      <c r="B54" s="25" t="s">
+        <v>145</v>
+      </c>
+      <c r="C54" s="25" t="s">
         <v>146</v>
       </c>
-      <c r="B54" s="26" t="s">
+      <c r="D54" s="25" t="s">
         <v>147</v>
       </c>
-      <c r="C54" s="26" t="s">
+      <c r="E54" s="25" t="s">
+        <v>61</v>
+      </c>
+      <c r="F54" s="25" t="s">
         <v>148</v>
       </c>
-      <c r="D54" s="26" t="s">
+      <c r="G54" s="26">
+        <v>28</v>
+      </c>
+      <c r="H54" s="26"/>
+    </row>
+    <row r="55" ht="19.5" customHeight="1">
+      <c r="A55" s="32" t="s">
         <v>149</v>
       </c>
-      <c r="E54" s="26" t="s">
-        <v>62</v>
-      </c>
-      <c r="F54" s="26" t="s">
+      <c r="B55" s="25" t="s">
+        <v>145</v>
+      </c>
+      <c r="C55" s="25" t="s">
         <v>150</v>
       </c>
-      <c r="G54" s="27">
-        <v>28</v>
-      </c>
-      <c r="H54" s="27"/>
-    </row>
-    <row r="55" ht="19.5" customHeight="1">
-      <c r="A55" s="33" t="s">
+      <c r="D55" s="25" t="s">
+        <v>129</v>
+      </c>
+      <c r="E55" s="25" t="s">
+        <v>61</v>
+      </c>
+      <c r="F55" s="25" t="s">
+        <v>148</v>
+      </c>
+      <c r="G55" s="26">
+        <v>10</v>
+      </c>
+      <c r="H55" s="26"/>
+    </row>
+    <row r="56" ht="19.5" customHeight="1">
+      <c r="A56" s="32" t="s">
         <v>151</v>
       </c>
-      <c r="B55" s="26" t="s">
-        <v>147</v>
-      </c>
-      <c r="C55" s="26" t="s">
+      <c r="B56" s="25" t="s">
+        <v>145</v>
+      </c>
+      <c r="C56" s="25" t="s">
         <v>152</v>
       </c>
-      <c r="D55" s="26" t="s">
-        <v>131</v>
-      </c>
-      <c r="E55" s="26" t="s">
-        <v>62</v>
-      </c>
-      <c r="F55" s="26" t="s">
-        <v>150</v>
-      </c>
-      <c r="G55" s="27">
-        <v>10</v>
-      </c>
-      <c r="H55" s="27"/>
-    </row>
-    <row r="56" ht="19.5" customHeight="1">
-      <c r="A56" s="33" t="s">
-        <v>153</v>
-      </c>
-      <c r="B56" s="26" t="s">
-        <v>147</v>
-      </c>
-      <c r="C56" s="26" t="s">
-        <v>154</v>
-      </c>
-      <c r="D56" s="26" t="s">
+      <c r="D56" s="25" t="s">
         <v>26</v>
       </c>
-      <c r="E56" s="26" t="s">
-        <v>62</v>
-      </c>
-      <c r="F56" s="26" t="s">
-        <v>150</v>
-      </c>
-      <c r="G56" s="27">
+      <c r="E56" s="25" t="s">
+        <v>61</v>
+      </c>
+      <c r="F56" s="25" t="s">
+        <v>148</v>
+      </c>
+      <c r="G56" s="26">
         <v>18</v>
       </c>
-      <c r="H56" s="27"/>
+      <c r="H56" s="26"/>
     </row>
     <row r="57" ht="19.5" customHeight="1">
       <c r="A57" s="8"/>
@@ -2984,76 +4237,76 @@
       <c r="H57" s="11"/>
     </row>
     <row r="58" ht="19.5" customHeight="1">
-      <c r="A58" s="18" t="s">
+      <c r="A58" s="17" t="s">
+        <v>153</v>
+      </c>
+      <c r="B58" s="19" t="s">
+        <v>145</v>
+      </c>
+      <c r="C58" s="19" t="s">
+        <v>154</v>
+      </c>
+      <c r="D58" s="19" t="s">
+        <v>147</v>
+      </c>
+      <c r="E58" s="33" t="s">
+        <v>32</v>
+      </c>
+      <c r="F58" s="19" t="s">
         <v>155</v>
       </c>
-      <c r="B58" s="20" t="s">
-        <v>147</v>
-      </c>
-      <c r="C58" s="20" t="s">
+      <c r="G58" s="18">
+        <v>27</v>
+      </c>
+      <c r="H58" s="18"/>
+    </row>
+    <row r="59" ht="19.5" customHeight="1">
+      <c r="A59" s="32" t="s">
         <v>156</v>
       </c>
-      <c r="D58" s="20" t="s">
-        <v>149</v>
-      </c>
-      <c r="E58" s="34" t="s">
+      <c r="B59" s="25" t="s">
+        <v>145</v>
+      </c>
+      <c r="C59" s="25" t="s">
+        <v>150</v>
+      </c>
+      <c r="D59" s="25" t="s">
+        <v>129</v>
+      </c>
+      <c r="E59" s="25" t="s">
+        <v>61</v>
+      </c>
+      <c r="F59" s="25" t="s">
+        <v>155</v>
+      </c>
+      <c r="G59" s="26">
+        <v>10</v>
+      </c>
+      <c r="H59" s="26"/>
+    </row>
+    <row r="60" ht="19.5" customHeight="1">
+      <c r="A60" s="17" t="s">
+        <v>157</v>
+      </c>
+      <c r="B60" s="19" t="s">
+        <v>145</v>
+      </c>
+      <c r="C60" s="19" t="s">
+        <v>152</v>
+      </c>
+      <c r="D60" s="19" t="s">
+        <v>26</v>
+      </c>
+      <c r="E60" s="19" t="s">
         <v>32</v>
       </c>
-      <c r="F58" s="20" t="s">
-        <v>157</v>
-      </c>
-      <c r="G58" s="19">
-        <v>27</v>
-      </c>
-      <c r="H58" s="19"/>
-    </row>
-    <row r="59" ht="19.5" customHeight="1">
-      <c r="A59" s="33" t="s">
-        <v>158</v>
-      </c>
-      <c r="B59" s="26" t="s">
-        <v>147</v>
-      </c>
-      <c r="C59" s="26" t="s">
-        <v>152</v>
-      </c>
-      <c r="D59" s="26" t="s">
-        <v>131</v>
-      </c>
-      <c r="E59" s="26" t="s">
-        <v>62</v>
-      </c>
-      <c r="F59" s="26" t="s">
-        <v>157</v>
-      </c>
-      <c r="G59" s="27">
-        <v>10</v>
-      </c>
-      <c r="H59" s="27"/>
-    </row>
-    <row r="60" ht="19.5" customHeight="1">
-      <c r="A60" s="18" t="s">
-        <v>159</v>
-      </c>
-      <c r="B60" s="20" t="s">
-        <v>147</v>
-      </c>
-      <c r="C60" s="20" t="s">
-        <v>154</v>
-      </c>
-      <c r="D60" s="20" t="s">
-        <v>26</v>
-      </c>
-      <c r="E60" s="20" t="s">
-        <v>32</v>
-      </c>
-      <c r="F60" s="20" t="s">
-        <v>157</v>
-      </c>
-      <c r="G60" s="19">
+      <c r="F60" s="19" t="s">
+        <v>155</v>
+      </c>
+      <c r="G60" s="18">
         <v>17</v>
       </c>
-      <c r="H60" s="19"/>
+      <c r="H60" s="18"/>
     </row>
     <row r="61" ht="19.5" customHeight="1">
       <c r="A61" s="11"/>
@@ -3066,71 +4319,71 @@
       <c r="H61" s="11"/>
     </row>
     <row r="62" ht="19.5" customHeight="1">
-      <c r="A62" s="9" t="s">
+      <c r="A62" s="19" t="s">
+        <v>158</v>
+      </c>
+      <c r="B62" s="19" t="s">
+        <v>159</v>
+      </c>
+      <c r="C62" s="19" t="s">
         <v>160</v>
       </c>
-      <c r="B62" s="9" t="s">
+      <c r="D62" s="19" t="s">
+        <v>26</v>
+      </c>
+      <c r="E62" s="19" t="s">
+        <v>32</v>
+      </c>
+      <c r="F62" s="19" t="s">
         <v>161</v>
       </c>
-      <c r="C62" s="9" t="s">
+      <c r="G62" s="18">
+        <v>11</v>
+      </c>
+      <c r="H62" s="18"/>
+    </row>
+    <row r="63" ht="19.5" customHeight="1">
+      <c r="A63" s="25" t="s">
         <v>162</v>
       </c>
-      <c r="D62" s="9" t="s">
-        <v>26</v>
-      </c>
-      <c r="E62" s="10" t="s">
+      <c r="B63" s="25" t="s">
+        <v>159</v>
+      </c>
+      <c r="C63" s="25" t="s">
+        <v>163</v>
+      </c>
+      <c r="D63" s="25" t="s">
+        <v>164</v>
+      </c>
+      <c r="E63" s="25" t="s">
+        <v>61</v>
+      </c>
+      <c r="F63" s="25" t="s">
+        <v>165</v>
+      </c>
+      <c r="G63" s="26">
         <v>12</v>
       </c>
-      <c r="F62" s="9" t="s">
-        <v>163</v>
-      </c>
-      <c r="G62" s="11">
-        <v>11</v>
-      </c>
-      <c r="H62" s="11"/>
-    </row>
-    <row r="63" ht="19.5" customHeight="1">
-      <c r="A63" s="26" t="s">
-        <v>164</v>
-      </c>
-      <c r="B63" s="26" t="s">
-        <v>161</v>
-      </c>
-      <c r="C63" s="26" t="s">
-        <v>165</v>
-      </c>
-      <c r="D63" s="26" t="s">
-        <v>166</v>
-      </c>
-      <c r="E63" s="26" t="s">
-        <v>62</v>
-      </c>
-      <c r="F63" s="26" t="s">
-        <v>167</v>
-      </c>
-      <c r="G63" s="27">
-        <v>12</v>
-      </c>
-      <c r="H63" s="27"/>
+      <c r="H63" s="26"/>
     </row>
     <row r="64" ht="19.5" customHeight="1">
       <c r="A64" s="9" t="s">
-        <v>168</v>
+        <v>166</v>
       </c>
       <c r="B64" s="9" t="s">
-        <v>161</v>
+        <v>159</v>
       </c>
       <c r="C64" s="9" t="s">
-        <v>169</v>
+        <v>167</v>
       </c>
       <c r="D64" s="9" t="s">
-        <v>67</v>
+        <v>65</v>
       </c>
       <c r="E64" s="10" t="s">
         <v>12</v>
       </c>
       <c r="F64" s="9" t="s">
-        <v>170</v>
+        <v>168</v>
       </c>
       <c r="G64" s="11">
         <v>11</v>
@@ -3148,38 +4401,38 @@
       <c r="H65" s="11"/>
     </row>
     <row r="66" ht="19.5" customHeight="1">
-      <c r="A66" s="18" t="s">
+      <c r="A66" s="17" t="s">
+        <v>169</v>
+      </c>
+      <c r="B66" s="19" t="s">
+        <v>169</v>
+      </c>
+      <c r="C66" s="17" t="s">
+        <v>170</v>
+      </c>
+      <c r="D66" s="19" t="s">
+        <v>129</v>
+      </c>
+      <c r="E66" s="19" t="s">
+        <v>32</v>
+      </c>
+      <c r="F66" s="19" t="s">
         <v>171</v>
       </c>
-      <c r="B66" s="20" t="s">
-        <v>171</v>
-      </c>
-      <c r="C66" s="18" t="s">
+      <c r="G66" s="18">
+        <v>21</v>
+      </c>
+      <c r="H66" s="18"/>
+    </row>
+    <row r="67" ht="19.5" customHeight="1">
+      <c r="A67" s="34" t="s">
         <v>172</v>
       </c>
-      <c r="D66" s="20" t="s">
-        <v>131</v>
-      </c>
-      <c r="E66" s="20" t="s">
-        <v>32</v>
-      </c>
-      <c r="F66" s="20" t="s">
-        <v>173</v>
-      </c>
-      <c r="G66" s="19">
-        <v>21</v>
-      </c>
-      <c r="H66" s="19"/>
-    </row>
-    <row r="67" ht="19.5" customHeight="1">
-      <c r="A67" s="35" t="s">
-        <v>174</v>
-      </c>
-      <c r="B67" s="36"/>
-      <c r="C67" s="36"/>
-      <c r="D67" s="36"/>
-      <c r="E67" s="36"/>
-      <c r="F67" s="37"/>
+      <c r="B67" s="35"/>
+      <c r="C67" s="35"/>
+      <c r="D67" s="35"/>
+      <c r="E67" s="35"/>
+      <c r="F67" s="36"/>
       <c r="G67" s="11">
         <f>SUM(G2,G3,G5,G6,G8,G14,G16,G18,G20,G24,G25,G26,G27,G28,G29,G30,G31,G32,G33,G34,G35,G36,G37,G38,G39,G41,G46,G48,G50,G52,G54,G58,G62,G63,G64,G66)</f>
         <v>508</v>
@@ -3227,6 +4480,7 @@
   <pageMargins left="0.511811024" right="0.511811024" top="0.78740157500000008" bottom="0.78740157500000008" header="0.31496062000000014" footer="0.31496062000000014"/>
   <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" usePrinterDefaults="1" blackAndWhite="0" draft="0" cellComments="none" useFirstPageNumber="0" errors="displayed" horizontalDpi="600" verticalDpi="600" copies="1"/>
   <headerFooter/>
+  <drawing r:id="rId1"/>
 </worksheet>
 </file>
 
@@ -3244,62 +4498,62 @@
   </cols>
   <sheetData>
     <row r="1" ht="23.25">
-      <c r="A1" s="38" t="s">
+      <c r="A1" s="37" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="38" t="s">
+      <c r="B1" s="37" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="39" t="s">
+      <c r="C1" s="38" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="38" t="s">
+      <c r="D1" s="37" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="38" t="s">
+      <c r="E1" s="37" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="38" t="s">
+      <c r="F1" s="37" t="s">
         <v>5</v>
       </c>
-      <c r="G1" s="40" t="s">
+      <c r="G1" s="39" t="s">
         <v>6</v>
       </c>
-      <c r="H1" s="41"/>
+      <c r="H1" s="40"/>
     </row>
     <row r="2" ht="37.5">
-      <c r="A2" s="42" t="s">
+      <c r="A2" s="41" t="s">
+        <v>173</v>
+      </c>
+      <c r="B2" s="42" t="s">
+        <v>173</v>
+      </c>
+      <c r="C2" s="43" t="s">
+        <v>174</v>
+      </c>
+      <c r="D2" s="42" t="s">
+        <v>147</v>
+      </c>
+      <c r="E2" s="44" t="s">
+        <v>12</v>
+      </c>
+      <c r="F2" s="42" t="s">
         <v>175</v>
       </c>
-      <c r="B2" s="43" t="s">
-        <v>175</v>
-      </c>
-      <c r="C2" s="44" t="s">
-        <v>176</v>
-      </c>
-      <c r="D2" s="43" t="s">
-        <v>149</v>
-      </c>
-      <c r="E2" s="45" t="s">
-        <v>12</v>
-      </c>
-      <c r="F2" s="43" t="s">
-        <v>177</v>
-      </c>
-      <c r="G2" s="46">
+      <c r="G2" s="45">
         <v>21</v>
       </c>
-      <c r="H2" s="47"/>
+      <c r="H2" s="46"/>
     </row>
     <row r="3" ht="18.75">
-      <c r="A3" s="46"/>
-      <c r="B3" s="46"/>
-      <c r="C3" s="44"/>
-      <c r="D3" s="46"/>
-      <c r="E3" s="46"/>
-      <c r="F3" s="46"/>
-      <c r="G3" s="46"/>
-      <c r="H3" s="47"/>
+      <c r="A3" s="45"/>
+      <c r="B3" s="45"/>
+      <c r="C3" s="43"/>
+      <c r="D3" s="45"/>
+      <c r="E3" s="45"/>
+      <c r="F3" s="45"/>
+      <c r="G3" s="45"/>
+      <c r="H3" s="46"/>
     </row>
   </sheetData>
   <printOptions headings="0" gridLines="0"/>

</xml_diff>

<commit_message>
Alteração no Burndown da Sprint 2, Inserção da planilha de tasks da Sprint 3 e Documento de Teste do Produto
</commit_message>
<xml_diff>
--- a/DOCS/sprints/sprint-02/TasksSprint2.xlsx
+++ b/DOCS/sprints/sprint-02/TasksSprint2.xlsx
@@ -16,7 +16,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="160" uniqueCount="160">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="149" uniqueCount="149">
   <si>
     <t>ID</t>
   </si>
@@ -39,34 +39,40 @@
     <t>Pontuação</t>
   </si>
   <si>
-    <t>DT-CONCLUSÂO</t>
-  </si>
-  <si>
-    <t>BD01.1</t>
-  </si>
-  <si>
-    <t>BD01</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Estruturar documentos</t>
+    <t xml:space="preserve">Dt. Fechamento</t>
+  </si>
+  <si>
+    <t>BD03.1</t>
+  </si>
+  <si>
+    <t>BD03</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Revisar modelagem relacional do dominio</t>
   </si>
   <si>
     <t xml:space="preserve">William, Lucas</t>
   </si>
   <si>
-    <t>EXCLUIDO</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Respostas com vinculo persistido a evidencias documentais.</t>
+    <t>Concluido</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Modelo cobrindo navegacao, respostas, usuarios, duvidas, logs, documentos e metadados.</t>
   </si>
   <si>
     <t>BURNDOWN</t>
   </si>
   <si>
-    <t>BD01.2</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Estruturar metadados</t>
+    <t>BD03.2</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Ampliar seed do banco com base no Desafio.pdf</t>
+  </si>
+  <si>
+    <t>William</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Seed suficiente para demonstrar o fluxo publico real.</t>
   </si>
   <si>
     <t>Data</t>
@@ -78,33 +84,6 @@
     <t xml:space="preserve">Esforço Real</t>
   </si>
   <si>
-    <t>BD03.1</t>
-  </si>
-  <si>
-    <t>BD03</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Revisar modelagem relacional do dominio</t>
-  </si>
-  <si>
-    <t>Validação</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Modelo cobrindo navegacao, respostas, usuarios, duvidas, logs, documentos e metadados.</t>
-  </si>
-  <si>
-    <t>BD03.2</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Ampliar seed do banco com base no Desafio.pdf</t>
-  </si>
-  <si>
-    <t>William</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Seed suficiente para demonstrar o fluxo publico real.</t>
-  </si>
-  <si>
     <t>DW01.1.1</t>
   </si>
   <si>
@@ -117,9 +96,6 @@
     <t>Pedro</t>
   </si>
   <si>
-    <t>Concluido</t>
-  </si>
-  <si>
     <t>DW01.1.2</t>
   </si>
   <si>
@@ -300,18 +276,12 @@
     <t>ES01.12</t>
   </si>
   <si>
-    <t xml:space="preserve">Definir convencao minima de branches e commits</t>
+    <t xml:space="preserve">Quebrar backlog da Sprint 2 em tasks rastreaveis</t>
   </si>
   <si>
     <t>Felipe</t>
   </si>
   <si>
-    <t xml:space="preserve">Time usando main, develop, feature/*, fix/* e docs/* com mensagens de commit claras.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Quebrar backlog da Sprint 2 em tasks rastreaveis</t>
-  </si>
-  <si>
     <t xml:space="preserve">Cada item da sprint com responsavel, status e vinculo ao backlog do produto.</t>
   </si>
   <si>
@@ -319,9 +289,6 @@
   </si>
   <si>
     <t xml:space="preserve">Consolidar burndown e evidencias de colaboracao da Sprint 2</t>
-  </si>
-  <si>
-    <t>Andamento</t>
   </si>
   <si>
     <t xml:space="preserve">Burndown e evidencias preparados para a avaliacao final da sprint.</t>
@@ -502,15 +469,21 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
-  <numFmts count="4">
-    <numFmt numFmtId="164" formatCode="dd/mm;@"/>
-    <numFmt numFmtId="165" formatCode="0.0"/>
-    <numFmt numFmtId="166" formatCode="dd-mmm"/>
-    <numFmt numFmtId="167" formatCode="[$-416]d\-mmm;@"/>
+  <numFmts count="3">
+    <numFmt numFmtId="164" formatCode="dd-mmm"/>
+    <numFmt numFmtId="165" formatCode="dd/mm;@"/>
+    <numFmt numFmtId="166" formatCode="0.0"/>
   </numFmts>
   <fonts count="13">
     <font>
       <sz val="11.000000"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="14.000000"/>
       <color theme="1"/>
       <name val="Calibri"/>
       <scheme val="minor"/>
@@ -548,12 +521,16 @@
     </font>
     <font>
       <sz val="14.000000"/>
-      <color indexed="2"/>
+      <color theme="1"/>
       <name val="Calibri"/>
     </font>
     <font>
       <sz val="14.000000"/>
-      <color indexed="2"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="16.000000"/>
       <name val="Calibri"/>
       <scheme val="minor"/>
     </font>
@@ -565,27 +542,21 @@
       <scheme val="minor"/>
     </font>
     <font>
-      <sz val="14.000000"/>
-      <name val="Calibri"/>
-    </font>
-    <font>
-      <sz val="14.000000"/>
+      <b/>
+      <sz val="16.000000"/>
       <color theme="1"/>
-      <name val="Calibri"/>
-    </font>
-    <font>
-      <sz val="14.000000"/>
-      <color theme="0" tint="0"/>
       <name val="Calibri"/>
       <scheme val="minor"/>
     </font>
     <font>
-      <sz val="14.000000"/>
+      <b/>
+      <sz val="18.000000"/>
+      <color theme="1"/>
       <name val="Calibri"/>
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="13">
+  <fills count="7">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -605,6 +576,12 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
+        <fgColor rgb="FFD1FAE5"/>
+        <bgColor rgb="FFD1FAE5"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
         <fgColor rgb="FFE5E7EB"/>
         <bgColor rgb="FFE5E7EB"/>
       </patternFill>
@@ -615,50 +592,8 @@
         <bgColor indexed="5"/>
       </patternFill>
     </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFB3C6E7"/>
-        <bgColor rgb="FFB3C6E7"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FF00B0F0"/>
-        <bgColor rgb="FF00B0F0"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFD1FAE5"/>
-        <bgColor rgb="FFD1FAE5"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFFFC000"/>
-        <bgColor rgb="FFFFC000"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor indexed="2"/>
-        <bgColor indexed="2"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="0" tint="-0.049989318521683403"/>
-        <bgColor theme="0" tint="-0.049989318521683403"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFFFE597"/>
-        <bgColor rgb="FFFFE597"/>
-      </patternFill>
-    </fill>
   </fills>
-  <borders count="6">
+  <borders count="9">
     <border>
       <left style="none"/>
       <right style="none"/>
@@ -673,6 +608,32 @@
       <right style="thin">
         <color theme="1"/>
       </right>
+      <top style="thin">
+        <color theme="1"/>
+      </top>
+      <bottom style="thin">
+        <color theme="1"/>
+      </bottom>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="thin">
+        <color theme="1"/>
+      </left>
+      <right style="thin">
+        <color theme="1"/>
+      </right>
+      <top style="thin">
+        <color theme="1"/>
+      </top>
+      <bottom style="none"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="thin">
+        <color theme="1"/>
+      </left>
+      <right style="none"/>
       <top style="thin">
         <color theme="1"/>
       </top>
@@ -700,13 +661,24 @@
       <left style="thin">
         <color theme="1"/>
       </left>
-      <right style="none"/>
-      <top style="thin">
+      <right style="thin">
         <color theme="1"/>
-      </top>
+      </right>
+      <top style="none"/>
       <bottom style="thin">
         <color theme="1"/>
       </bottom>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="thin">
+        <color theme="1"/>
+      </left>
+      <right style="thin">
+        <color theme="1"/>
+      </right>
+      <top style="none"/>
+      <bottom style="none"/>
       <diagonal style="none"/>
     </border>
     <border>
@@ -737,148 +709,166 @@
   <cellStyleXfs count="1">
     <xf fontId="0" fillId="0" borderId="0" numFmtId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
   </cellStyleXfs>
-  <cellXfs count="47">
+  <cellXfs count="41">
     <xf fontId="0" fillId="0" borderId="0" numFmtId="0" xfId="0"/>
     <xf fontId="0" fillId="0" borderId="0" numFmtId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
+      <protection locked="0"/>
     </xf>
     <xf fontId="1" fillId="0" borderId="0" numFmtId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
+      <protection locked="0"/>
     </xf>
     <xf fontId="2" fillId="0" borderId="0" numFmtId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
+      <protection locked="0"/>
     </xf>
-    <xf fontId="3" fillId="2" borderId="1" numFmtId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf fontId="3" fillId="0" borderId="0" numFmtId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf fontId="4" fillId="2" borderId="1" numFmtId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf fontId="3" fillId="3" borderId="1" numFmtId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection locked="0"/>
     </xf>
     <xf fontId="4" fillId="3" borderId="1" numFmtId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection locked="0"/>
     </xf>
-    <xf fontId="5" fillId="2" borderId="1" numFmtId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf fontId="5" fillId="3" borderId="1" numFmtId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf fontId="6" fillId="2" borderId="1" numFmtId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
+      <protection locked="0"/>
     </xf>
-    <xf fontId="6" fillId="4" borderId="1" numFmtId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    <xf fontId="6" fillId="2" borderId="2" numFmtId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection locked="0"/>
     </xf>
     <xf fontId="7" fillId="4" borderId="1" numFmtId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf fontId="8" fillId="4" borderId="3" numFmtId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf fontId="9" fillId="5" borderId="4" numFmtId="164" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf fontId="10" fillId="6" borderId="1" numFmtId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf fontId="2" fillId="4" borderId="3" numFmtId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf fontId="2" fillId="0" borderId="1" numFmtId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf fontId="11" fillId="0" borderId="5" numFmtId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf fontId="2" fillId="0" borderId="1" numFmtId="165" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf fontId="8" fillId="4" borderId="1" numFmtId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf fontId="2" fillId="4" borderId="1" numFmtId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf fontId="11" fillId="5" borderId="1" numFmtId="164" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf fontId="2" fillId="0" borderId="1" numFmtId="166" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf fontId="9" fillId="5" borderId="1" numFmtId="164" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf fontId="9" fillId="0" borderId="1" numFmtId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection locked="0"/>
     </xf>
     <xf fontId="7" fillId="0" borderId="1" numFmtId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf fontId="9" fillId="0" borderId="2" numFmtId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
+      <protection locked="0"/>
     </xf>
-    <xf fontId="8" fillId="5" borderId="1" numFmtId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf fontId="2" fillId="4" borderId="0" numFmtId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
+      <protection locked="0"/>
     </xf>
-    <xf fontId="9" fillId="0" borderId="1" numFmtId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    <xf fontId="9" fillId="5" borderId="5" numFmtId="164" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection locked="0"/>
     </xf>
     <xf fontId="0" fillId="0" borderId="1" numFmtId="0" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
+      <protection locked="0"/>
     </xf>
-    <xf fontId="1" fillId="0" borderId="1" numFmtId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf fontId="9" fillId="5" borderId="1" numFmtId="16" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
+      <protection locked="0"/>
     </xf>
-    <xf fontId="1" fillId="0" borderId="1" numFmtId="164" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf fontId="2" fillId="4" borderId="1" numFmtId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
+      <protection hidden="0" locked="0"/>
     </xf>
-    <xf fontId="10" fillId="6" borderId="1" numFmtId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    <xf fontId="0" fillId="0" borderId="0" numFmtId="0" xfId="0">
+      <protection locked="0"/>
     </xf>
-    <xf fontId="9" fillId="6" borderId="1" numFmtId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf fontId="9" fillId="5" borderId="2" numFmtId="16" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
+      <protection locked="0"/>
     </xf>
-    <xf fontId="11" fillId="7" borderId="1" numFmtId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf fontId="9" fillId="5" borderId="6" numFmtId="164" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
+      <protection locked="0"/>
     </xf>
-    <xf fontId="1" fillId="0" borderId="1" numFmtId="165" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf fontId="9" fillId="0" borderId="5" numFmtId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
+      <protection locked="0"/>
     </xf>
-    <xf fontId="1" fillId="6" borderId="1" numFmtId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf fontId="8" fillId="4" borderId="1" numFmtId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
+      <protection locked="0"/>
     </xf>
-    <xf fontId="9" fillId="8" borderId="1" numFmtId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    <xf fontId="8" fillId="0" borderId="1" numFmtId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection locked="0"/>
     </xf>
-    <xf fontId="1" fillId="8" borderId="1" numFmtId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf fontId="10" fillId="0" borderId="3" numFmtId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf fontId="10" fillId="0" borderId="7" numFmtId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf fontId="10" fillId="0" borderId="8" numFmtId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf fontId="12" fillId="0" borderId="1" numFmtId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf fontId="10" fillId="8" borderId="1" numFmtId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf fontId="1" fillId="5" borderId="1" numFmtId="166" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf fontId="12" fillId="9" borderId="1" numFmtId="166" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf fontId="10" fillId="0" borderId="1" numFmtId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf fontId="1" fillId="6" borderId="0" numFmtId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf fontId="11" fillId="10" borderId="1" numFmtId="16" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf fontId="11" fillId="10" borderId="1" numFmtId="166" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf fontId="1" fillId="8" borderId="1" numFmtId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-      <protection hidden="0" locked="1"/>
-    </xf>
-    <xf fontId="11" fillId="10" borderId="2" numFmtId="167" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf fontId="12" fillId="11" borderId="2" numFmtId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf fontId="12" fillId="9" borderId="2" numFmtId="16" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf fontId="12" fillId="5" borderId="2" numFmtId="16" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf fontId="11" fillId="7" borderId="2" numFmtId="16" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf fontId="7" fillId="4" borderId="1" numFmtId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-      <protection hidden="0" locked="1"/>
-    </xf>
-    <xf fontId="12" fillId="9" borderId="1" numFmtId="16" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf fontId="9" fillId="12" borderId="1" numFmtId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf fontId="1" fillId="12" borderId="1" numFmtId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-      <protection hidden="0" locked="1"/>
-    </xf>
-    <xf fontId="10" fillId="12" borderId="1" numFmtId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf fontId="1" fillId="12" borderId="1" numFmtId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf fontId="9" fillId="8" borderId="1" numFmtId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf fontId="9" fillId="0" borderId="1" numFmtId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf fontId="8" fillId="0" borderId="3" numFmtId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf fontId="8" fillId="0" borderId="4" numFmtId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf fontId="8" fillId="0" borderId="5" numFmtId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
+      <protection locked="0"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -917,7 +907,7 @@
           <a:bodyPr/>
           <a:p>
             <a:pPr>
-              <a:defRPr sz="1400" b="0" spc="0">
+              <a:defRPr sz="1400" b="1" spc="0">
                 <a:solidFill>
                   <a:schemeClr val="tx1">
                     <a:lumMod val="65000"/>
@@ -930,10 +920,10 @@
               </a:defRPr>
             </a:pPr>
             <a:r>
-              <a:rPr/>
+              <a:rPr sz="1600" b="1"/>
               <a:t>Sprint 2</a:t>
             </a:r>
-            <a:endParaRPr/>
+            <a:endParaRPr sz="1600" b="1"/>
           </a:p>
         </c:rich>
       </c:tx>
@@ -952,7 +942,7 @@
         <a:bodyPr/>
         <a:p>
           <a:pPr>
-            <a:defRPr sz="1400" b="0" spc="0">
+            <a:defRPr sz="1600" b="1" spc="0">
               <a:solidFill>
                 <a:schemeClr val="tx1">
                   <a:lumMod val="65000"/>
@@ -1285,58 +1275,58 @@
                   <c:v>419</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>419</c:v>
+                  <c:v>399</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>419</c:v>
+                  <c:v>397</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>419</c:v>
+                  <c:v>395</c:v>
                 </c:pt>
                 <c:pt idx="4">
-                  <c:v>419</c:v>
+                  <c:v>385</c:v>
                 </c:pt>
                 <c:pt idx="5">
-                  <c:v>419</c:v>
+                  <c:v>368</c:v>
                 </c:pt>
                 <c:pt idx="6">
-                  <c:v>419</c:v>
+                  <c:v>363</c:v>
                 </c:pt>
                 <c:pt idx="7">
-                  <c:v>419</c:v>
+                  <c:v>358</c:v>
                 </c:pt>
                 <c:pt idx="8">
-                  <c:v>419</c:v>
+                  <c:v>333</c:v>
                 </c:pt>
                 <c:pt idx="9">
-                  <c:v>419</c:v>
+                  <c:v>306</c:v>
                 </c:pt>
                 <c:pt idx="10">
-                  <c:v>419</c:v>
+                  <c:v>281</c:v>
                 </c:pt>
                 <c:pt idx="11">
-                  <c:v>419</c:v>
+                  <c:v>256</c:v>
                 </c:pt>
                 <c:pt idx="12">
-                  <c:v>405</c:v>
+                  <c:v>221</c:v>
                 </c:pt>
                 <c:pt idx="13">
-                  <c:v>388</c:v>
+                  <c:v>196</c:v>
                 </c:pt>
                 <c:pt idx="14">
-                  <c:v>388</c:v>
+                  <c:v>171</c:v>
                 </c:pt>
                 <c:pt idx="15">
-                  <c:v>388</c:v>
+                  <c:v>136</c:v>
                 </c:pt>
                 <c:pt idx="16">
-                  <c:v>388</c:v>
+                  <c:v>111</c:v>
                 </c:pt>
                 <c:pt idx="17">
-                  <c:v>388</c:v>
+                  <c:v>86</c:v>
                 </c:pt>
                 <c:pt idx="18">
-                  <c:v>129</c:v>
+                  <c:v>43</c:v>
                 </c:pt>
                 <c:pt idx="19">
                   <c:v>0</c:v>
@@ -1349,6 +1339,7 @@
         <c:dLbls>
           <c:showBubbleSize val="0"/>
           <c:showCatName val="0"/>
+          <c:showLeaderLines val="0"/>
           <c:showLegendKey val="0"/>
           <c:showPercent val="0"/>
           <c:showSerName val="0"/>
@@ -1522,8 +1513,8 @@
   </c:chart>
   <c:spPr bwMode="auto">
     <a:xfrm rot="0" flipH="0" flipV="0">
-      <a:off x="28908374" y="257174"/>
-      <a:ext cx="9315450" cy="4543424"/>
+      <a:off x="29194124" y="495298"/>
+      <a:ext cx="7924799" cy="3705225"/>
     </a:xfrm>
     <a:prstGeom prst="rect">
       <a:avLst/>
@@ -2158,15 +2149,15 @@
   <xdr:twoCellAnchor editAs="twoCell">
     <xdr:from>
       <xdr:col>12</xdr:col>
-      <xdr:colOff>323849</xdr:colOff>
+      <xdr:colOff>609599</xdr:colOff>
       <xdr:row>1</xdr:row>
-      <xdr:rowOff>9524</xdr:rowOff>
+      <xdr:rowOff>247648</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>27</xdr:col>
-      <xdr:colOff>495299</xdr:colOff>
-      <xdr:row>19</xdr:row>
-      <xdr:rowOff>95249</xdr:rowOff>
+      <xdr:col>25</xdr:col>
+      <xdr:colOff>609599</xdr:colOff>
+      <xdr:row>16</xdr:row>
+      <xdr:rowOff>238124</xdr:rowOff>
     </xdr:to>
     <xdr:graphicFrame>
       <xdr:nvGraphicFramePr>
@@ -2176,8 +2167,8 @@
         </xdr:cNvGraphicFramePr>
       </xdr:nvGraphicFramePr>
       <xdr:xfrm rot="0" flipH="0" flipV="0">
-        <a:off x="28908374" y="257174"/>
-        <a:ext cx="9315450" cy="4543424"/>
+        <a:off x="29194124" y="495298"/>
+        <a:ext cx="7924799" cy="3705225"/>
       </xdr:xfrm>
       <a:graphic>
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
@@ -2680,1738 +2671,1883 @@
     <col customWidth="1" min="6" max="6" style="1" width="162.7109375"/>
     <col customWidth="1" min="7" max="7" style="1" width="20.7109375"/>
     <col customWidth="1" min="8" max="8" style="2" width="35.00390625"/>
-    <col bestFit="1" customWidth="1" min="9" max="9" style="2" width="9.140625"/>
+    <col bestFit="1" customWidth="1" min="9" max="9" style="3" width="9.140625"/>
     <col customWidth="1" min="10" max="10" style="1" width="14.8515625"/>
     <col customWidth="1" min="11" max="11" style="1" width="23.00390625"/>
     <col customWidth="1" min="12" max="12" style="1" width="23.7109375"/>
-    <col min="13" max="16384" style="1" width="9.140625"/>
+    <col min="13" max="13" style="1" width="9.140625"/>
+    <col min="14" max="26" style="1" width="9.140625"/>
+    <col customWidth="1" min="27" max="27" style="1" width="10.421875"/>
+    <col customWidth="1" min="28" max="28" style="1" width="21.8515625"/>
+    <col customWidth="1" min="29" max="29" style="1" width="22.00390625"/>
+    <col min="30" max="30" style="1" width="9.140625"/>
+    <col min="31" max="16384" style="1" width="9.140625"/>
   </cols>
   <sheetData>
-    <row r="1" s="3" customFormat="1" ht="19.5" customHeight="1">
-      <c r="A1" s="4" t="s">
+    <row r="1" s="4" customFormat="1" ht="19.5" customHeight="1">
+      <c r="A1" s="5" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="5" t="s">
+      <c r="B1" s="6" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="6" t="s">
+      <c r="C1" s="7" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="5" t="s">
+      <c r="D1" s="6" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="5" t="s">
+      <c r="E1" s="6" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="5" t="s">
+      <c r="F1" s="6" t="s">
         <v>5</v>
       </c>
-      <c r="G1" s="7" t="s">
+      <c r="G1" s="8" t="s">
         <v>6</v>
       </c>
-      <c r="H1" s="7" t="s">
+      <c r="H1" s="9" t="s">
         <v>7</v>
       </c>
-      <c r="I1" s="2"/>
+      <c r="I1" s="3"/>
+      <c r="J1" s="4"/>
+      <c r="K1" s="4"/>
+      <c r="L1" s="4"/>
+      <c r="M1" s="4"/>
+      <c r="N1" s="4"/>
+      <c r="AA1" s="4"/>
+      <c r="AB1" s="4"/>
+      <c r="AC1" s="4"/>
+      <c r="AD1" s="4"/>
     </row>
     <row r="2" ht="19.5" customHeight="1">
-      <c r="A2" s="8" t="s">
+      <c r="A2" s="10" t="s">
         <v>8</v>
       </c>
-      <c r="B2" s="8" t="s">
+      <c r="B2" s="10" t="s">
         <v>9</v>
       </c>
-      <c r="C2" s="8" t="s">
+      <c r="C2" s="10" t="s">
         <v>10</v>
       </c>
-      <c r="D2" s="8" t="s">
+      <c r="D2" s="10" t="s">
         <v>11</v>
       </c>
-      <c r="E2" s="8" t="s">
+      <c r="E2" s="10" t="s">
         <v>12</v>
       </c>
-      <c r="F2" s="8" t="s">
+      <c r="F2" s="10" t="s">
         <v>13</v>
       </c>
-      <c r="G2" s="9">
+      <c r="G2" s="11">
         <v>27</v>
       </c>
-      <c r="H2" s="10"/>
-      <c r="I2" s="2"/>
-      <c r="J2" s="11" t="s">
+      <c r="H2" s="12">
+        <v>46167</v>
+      </c>
+      <c r="I2" s="3"/>
+      <c r="J2" s="13" t="s">
         <v>14</v>
       </c>
-      <c r="K2" s="11"/>
-      <c r="L2" s="11"/>
+      <c r="K2" s="13"/>
+      <c r="L2" s="13"/>
+      <c r="M2" s="1"/>
+      <c r="N2" s="1"/>
+      <c r="O2" s="1"/>
+      <c r="P2" s="1"/>
+      <c r="Q2" s="1"/>
     </row>
     <row r="3" ht="19.5" customHeight="1">
-      <c r="A3" s="8" t="s">
+      <c r="A3" s="10" t="s">
         <v>15</v>
       </c>
-      <c r="B3" s="8" t="s">
+      <c r="B3" s="10" t="s">
         <v>9</v>
       </c>
-      <c r="C3" s="8" t="s">
+      <c r="C3" s="10" t="s">
         <v>16</v>
       </c>
-      <c r="D3" s="8" t="s">
+      <c r="D3" s="10" t="s">
+        <v>17</v>
+      </c>
+      <c r="E3" s="10" t="s">
+        <v>12</v>
+      </c>
+      <c r="F3" s="10" t="s">
+        <v>18</v>
+      </c>
+      <c r="G3" s="14">
+        <v>28</v>
+      </c>
+      <c r="H3" s="12">
+        <v>46167</v>
+      </c>
+      <c r="I3" s="3"/>
+      <c r="J3" s="8" t="s">
+        <v>19</v>
+      </c>
+      <c r="K3" s="8" t="s">
+        <v>20</v>
+      </c>
+      <c r="L3" s="8" t="s">
+        <v>21</v>
+      </c>
+      <c r="M3" s="1"/>
+      <c r="N3" s="1"/>
+      <c r="O3" s="1"/>
+      <c r="P3" s="1"/>
+      <c r="AE3" s="1"/>
+      <c r="AF3" s="1"/>
+      <c r="AG3" s="1"/>
+    </row>
+    <row r="4" ht="19.5" customHeight="1">
+      <c r="A4" s="15"/>
+      <c r="B4" s="15"/>
+      <c r="C4" s="15"/>
+      <c r="D4" s="15"/>
+      <c r="E4" s="15"/>
+      <c r="F4" s="15"/>
+      <c r="G4" s="15"/>
+      <c r="H4" s="16"/>
+      <c r="J4" s="17">
+        <v>46148</v>
+      </c>
+      <c r="K4" s="15">
+        <f>G56</f>
+        <v>419</v>
+      </c>
+      <c r="L4" s="15">
+        <v>419</v>
+      </c>
+      <c r="M4" s="1"/>
+      <c r="N4" s="1"/>
+      <c r="O4" s="1"/>
+      <c r="P4" s="1"/>
+      <c r="AE4" s="1"/>
+      <c r="AF4" s="1"/>
+      <c r="AG4" s="1"/>
+    </row>
+    <row r="5" ht="19.5" customHeight="1">
+      <c r="A5" s="18" t="s">
+        <v>22</v>
+      </c>
+      <c r="B5" s="18" t="s">
+        <v>23</v>
+      </c>
+      <c r="C5" s="18" t="s">
+        <v>24</v>
+      </c>
+      <c r="D5" s="19" t="s">
+        <v>25</v>
+      </c>
+      <c r="E5" s="10" t="s">
+        <v>12</v>
+      </c>
+      <c r="F5" s="18" t="s">
+        <v>24</v>
+      </c>
+      <c r="G5" s="19">
+        <v>21</v>
+      </c>
+      <c r="H5" s="20">
+        <v>46166</v>
+      </c>
+      <c r="I5" s="3"/>
+      <c r="J5" s="17">
+        <v>46149</v>
+      </c>
+      <c r="K5" s="21">
+        <f t="shared" ref="K5:K10" si="0">K4-22.052</f>
+        <v>396.94799999999998</v>
+      </c>
+      <c r="L5" s="15">
+        <v>399</v>
+      </c>
+      <c r="M5" s="1"/>
+      <c r="N5" s="1"/>
+      <c r="O5" s="1"/>
+      <c r="P5" s="1"/>
+      <c r="Q5" s="1"/>
+      <c r="AE5" s="1"/>
+      <c r="AF5" s="1"/>
+      <c r="AG5" s="1"/>
+    </row>
+    <row r="6" ht="19.5" customHeight="1">
+      <c r="A6" s="18" t="s">
+        <v>26</v>
+      </c>
+      <c r="B6" s="18" t="s">
+        <v>23</v>
+      </c>
+      <c r="C6" s="18" t="s">
+        <v>27</v>
+      </c>
+      <c r="D6" s="19" t="s">
+        <v>25</v>
+      </c>
+      <c r="E6" s="10" t="s">
+        <v>12</v>
+      </c>
+      <c r="F6" s="18" t="s">
+        <v>24</v>
+      </c>
+      <c r="G6" s="19">
+        <v>5</v>
+      </c>
+      <c r="H6" s="22">
+        <v>46161</v>
+      </c>
+      <c r="I6" s="3"/>
+      <c r="J6" s="17">
+        <v>46150</v>
+      </c>
+      <c r="K6" s="21">
+        <f t="shared" si="0"/>
+        <v>374.89599999999996</v>
+      </c>
+      <c r="L6" s="15">
+        <v>397</v>
+      </c>
+      <c r="M6" s="1"/>
+      <c r="N6" s="1"/>
+      <c r="O6" s="1"/>
+      <c r="P6" s="1"/>
+      <c r="Q6" s="1"/>
+      <c r="AB6" s="1"/>
+      <c r="AE6" s="1"/>
+      <c r="AF6" s="1"/>
+      <c r="AG6" s="1"/>
+    </row>
+    <row r="7" ht="19.5" customHeight="1">
+      <c r="A7" s="18" t="s">
+        <v>28</v>
+      </c>
+      <c r="B7" s="18" t="s">
+        <v>23</v>
+      </c>
+      <c r="C7" s="18" t="s">
+        <v>29</v>
+      </c>
+      <c r="D7" s="19" t="s">
+        <v>25</v>
+      </c>
+      <c r="E7" s="10" t="s">
+        <v>12</v>
+      </c>
+      <c r="F7" s="18" t="s">
+        <v>24</v>
+      </c>
+      <c r="G7" s="19">
+        <v>5</v>
+      </c>
+      <c r="H7" s="22">
+        <v>46161</v>
+      </c>
+      <c r="I7" s="3"/>
+      <c r="J7" s="17">
+        <v>46151</v>
+      </c>
+      <c r="K7" s="21">
+        <f t="shared" si="0"/>
+        <v>352.84399999999994</v>
+      </c>
+      <c r="L7" s="15">
+        <v>395</v>
+      </c>
+      <c r="M7" s="1"/>
+      <c r="N7" s="1"/>
+      <c r="O7" s="1"/>
+      <c r="P7" s="1"/>
+      <c r="Q7" s="1"/>
+      <c r="AB7" s="1"/>
+      <c r="AE7" s="1"/>
+      <c r="AF7" s="1"/>
+      <c r="AG7" s="1"/>
+    </row>
+    <row r="8" ht="19.5" customHeight="1">
+      <c r="A8" s="18" t="s">
+        <v>30</v>
+      </c>
+      <c r="B8" s="18" t="s">
+        <v>23</v>
+      </c>
+      <c r="C8" s="18" t="s">
+        <v>31</v>
+      </c>
+      <c r="D8" s="19" t="s">
+        <v>25</v>
+      </c>
+      <c r="E8" s="10" t="s">
+        <v>12</v>
+      </c>
+      <c r="F8" s="18" t="s">
+        <v>24</v>
+      </c>
+      <c r="G8" s="19">
+        <v>6</v>
+      </c>
+      <c r="H8" s="22">
+        <v>46166</v>
+      </c>
+      <c r="I8" s="3"/>
+      <c r="J8" s="17">
+        <v>46152</v>
+      </c>
+      <c r="K8" s="21">
+        <f t="shared" si="0"/>
+        <v>330.79199999999992</v>
+      </c>
+      <c r="L8" s="15">
+        <v>385</v>
+      </c>
+      <c r="M8" s="1"/>
+      <c r="N8" s="1"/>
+      <c r="O8" s="1"/>
+      <c r="P8" s="1"/>
+      <c r="Q8" s="1"/>
+      <c r="AB8" s="1"/>
+      <c r="AE8" s="1"/>
+      <c r="AF8" s="1"/>
+      <c r="AG8" s="1"/>
+    </row>
+    <row r="9" ht="19.5" customHeight="1">
+      <c r="A9" s="18" t="s">
+        <v>32</v>
+      </c>
+      <c r="B9" s="18" t="s">
+        <v>23</v>
+      </c>
+      <c r="C9" s="18" t="s">
+        <v>33</v>
+      </c>
+      <c r="D9" s="19" t="s">
+        <v>25</v>
+      </c>
+      <c r="E9" s="10" t="s">
+        <v>12</v>
+      </c>
+      <c r="F9" s="18" t="s">
+        <v>24</v>
+      </c>
+      <c r="G9" s="19">
+        <v>5</v>
+      </c>
+      <c r="H9" s="22">
+        <v>46161</v>
+      </c>
+      <c r="I9" s="3"/>
+      <c r="J9" s="17">
+        <v>46153</v>
+      </c>
+      <c r="K9" s="21">
+        <f t="shared" si="0"/>
+        <v>308.7399999999999</v>
+      </c>
+      <c r="L9" s="15">
+        <v>368</v>
+      </c>
+      <c r="M9" s="1"/>
+      <c r="N9" s="1"/>
+      <c r="O9" s="1"/>
+      <c r="P9" s="1"/>
+      <c r="Q9" s="1"/>
+      <c r="AB9" s="1"/>
+      <c r="AE9" s="1"/>
+      <c r="AF9" s="1"/>
+      <c r="AG9" s="1"/>
+    </row>
+    <row r="10" ht="19.5" customHeight="1">
+      <c r="A10" s="15"/>
+      <c r="B10" s="15"/>
+      <c r="C10" s="15"/>
+      <c r="D10" s="15"/>
+      <c r="E10" s="15"/>
+      <c r="F10" s="15"/>
+      <c r="G10" s="15"/>
+      <c r="H10" s="23"/>
+      <c r="I10" s="3"/>
+      <c r="J10" s="17">
+        <v>46154</v>
+      </c>
+      <c r="K10" s="21">
+        <f t="shared" si="0"/>
+        <v>286.68799999999987</v>
+      </c>
+      <c r="L10" s="15">
+        <v>363</v>
+      </c>
+      <c r="M10" s="1"/>
+      <c r="N10" s="1"/>
+      <c r="O10" s="1"/>
+      <c r="P10" s="1"/>
+      <c r="Q10" s="1"/>
+      <c r="AB10" s="1"/>
+      <c r="AE10" s="1"/>
+      <c r="AF10" s="1"/>
+      <c r="AG10" s="1"/>
+    </row>
+    <row r="11" ht="19.5" customHeight="1">
+      <c r="A11" s="10" t="s">
+        <v>34</v>
+      </c>
+      <c r="B11" s="10" t="s">
+        <v>34</v>
+      </c>
+      <c r="C11" s="10" t="s">
+        <v>35</v>
+      </c>
+      <c r="D11" s="10" t="s">
+        <v>36</v>
+      </c>
+      <c r="E11" s="10" t="s">
+        <v>12</v>
+      </c>
+      <c r="F11" s="10" t="s">
+        <v>37</v>
+      </c>
+      <c r="G11" s="19">
+        <v>34</v>
+      </c>
+      <c r="H11" s="22">
+        <v>46166</v>
+      </c>
+      <c r="I11" s="3"/>
+      <c r="J11" s="17">
+        <v>46155</v>
+      </c>
+      <c r="K11" s="21">
+        <f t="shared" ref="K11:K23" si="1">K10-22.052</f>
+        <v>264.63599999999985</v>
+      </c>
+      <c r="L11" s="15">
+        <v>358</v>
+      </c>
+      <c r="M11" s="1"/>
+      <c r="N11" s="1"/>
+      <c r="O11" s="1"/>
+      <c r="P11" s="1"/>
+      <c r="Q11" s="1"/>
+      <c r="AB11" s="1"/>
+      <c r="AE11" s="1"/>
+      <c r="AF11" s="1"/>
+      <c r="AG11" s="1"/>
+    </row>
+    <row r="12" ht="19.5" customHeight="1">
+      <c r="A12" s="15"/>
+      <c r="B12" s="15"/>
+      <c r="C12" s="15"/>
+      <c r="D12" s="15"/>
+      <c r="E12" s="15"/>
+      <c r="F12" s="15"/>
+      <c r="G12" s="15"/>
+      <c r="H12" s="23"/>
+      <c r="I12" s="3"/>
+      <c r="J12" s="17">
+        <v>46156</v>
+      </c>
+      <c r="K12" s="21">
+        <f t="shared" si="1"/>
+        <v>242.58399999999986</v>
+      </c>
+      <c r="L12" s="15">
+        <v>333</v>
+      </c>
+      <c r="M12" s="1"/>
+      <c r="N12" s="1"/>
+      <c r="O12" s="1"/>
+      <c r="P12" s="1"/>
+      <c r="Q12" s="1"/>
+      <c r="AB12" s="1"/>
+      <c r="AE12" s="1"/>
+      <c r="AF12" s="1"/>
+      <c r="AG12" s="1"/>
+    </row>
+    <row r="13" ht="19.5" customHeight="1">
+      <c r="A13" s="10" t="s">
+        <v>38</v>
+      </c>
+      <c r="B13" s="10" t="s">
+        <v>38</v>
+      </c>
+      <c r="C13" s="10" t="s">
+        <v>39</v>
+      </c>
+      <c r="D13" s="10" t="s">
+        <v>40</v>
+      </c>
+      <c r="E13" s="10" t="s">
+        <v>12</v>
+      </c>
+      <c r="F13" s="10" t="s">
+        <v>41</v>
+      </c>
+      <c r="G13" s="19">
+        <v>55</v>
+      </c>
+      <c r="H13" s="22">
+        <v>46166</v>
+      </c>
+      <c r="I13" s="3"/>
+      <c r="J13" s="17">
+        <v>46157</v>
+      </c>
+      <c r="K13" s="21">
+        <f t="shared" si="1"/>
+        <v>220.53199999999987</v>
+      </c>
+      <c r="L13" s="15">
+        <v>306</v>
+      </c>
+      <c r="M13" s="1"/>
+      <c r="N13" s="1"/>
+      <c r="O13" s="1"/>
+      <c r="P13" s="1"/>
+      <c r="Q13" s="1"/>
+      <c r="AB13" s="1"/>
+      <c r="AE13" s="1"/>
+      <c r="AF13" s="1"/>
+      <c r="AG13" s="1"/>
+    </row>
+    <row r="14" ht="19.5" customHeight="1">
+      <c r="A14" s="24"/>
+      <c r="B14" s="24"/>
+      <c r="C14" s="24"/>
+      <c r="D14" s="24"/>
+      <c r="E14" s="24"/>
+      <c r="F14" s="24"/>
+      <c r="G14" s="15"/>
+      <c r="H14" s="25"/>
+      <c r="I14" s="3"/>
+      <c r="J14" s="17">
+        <v>46158</v>
+      </c>
+      <c r="K14" s="21">
+        <f t="shared" si="1"/>
+        <v>198.47999999999988</v>
+      </c>
+      <c r="L14" s="15">
+        <v>281</v>
+      </c>
+      <c r="M14" s="1"/>
+      <c r="N14" s="1"/>
+      <c r="O14" s="1"/>
+      <c r="P14" s="1"/>
+      <c r="Q14" s="1"/>
+      <c r="AB14" s="1"/>
+      <c r="AE14" s="1"/>
+      <c r="AF14" s="1"/>
+      <c r="AG14" s="1"/>
+    </row>
+    <row r="15" ht="19.5" customHeight="1">
+      <c r="A15" s="10" t="s">
+        <v>42</v>
+      </c>
+      <c r="B15" s="10" t="s">
+        <v>43</v>
+      </c>
+      <c r="C15" s="19" t="s">
+        <v>44</v>
+      </c>
+      <c r="D15" s="10" t="s">
+        <v>36</v>
+      </c>
+      <c r="E15" s="10" t="s">
+        <v>12</v>
+      </c>
+      <c r="F15" s="26" t="s">
+        <v>45</v>
+      </c>
+      <c r="G15" s="14">
+        <v>21</v>
+      </c>
+      <c r="H15" s="12">
+        <v>46167</v>
+      </c>
+      <c r="I15" s="3"/>
+      <c r="J15" s="17">
+        <v>46159</v>
+      </c>
+      <c r="K15" s="21">
+        <f t="shared" si="1"/>
+        <v>176.42799999999988</v>
+      </c>
+      <c r="L15" s="15">
+        <v>256</v>
+      </c>
+      <c r="M15" s="1"/>
+      <c r="N15" s="1"/>
+      <c r="O15" s="1"/>
+      <c r="P15" s="1"/>
+      <c r="Q15" s="1"/>
+      <c r="AB15" s="1"/>
+      <c r="AE15" s="1"/>
+      <c r="AF15" s="1"/>
+      <c r="AG15" s="1"/>
+    </row>
+    <row r="16" ht="19.5" customHeight="1">
+      <c r="A16" s="10" t="s">
+        <v>46</v>
+      </c>
+      <c r="B16" s="10" t="s">
+        <v>43</v>
+      </c>
+      <c r="C16" s="19" t="s">
+        <v>47</v>
+      </c>
+      <c r="D16" s="10" t="s">
+        <v>40</v>
+      </c>
+      <c r="E16" s="10" t="s">
+        <v>12</v>
+      </c>
+      <c r="F16" s="19" t="s">
+        <v>45</v>
+      </c>
+      <c r="G16" s="14">
+        <v>10</v>
+      </c>
+      <c r="H16" s="12">
+        <v>46167</v>
+      </c>
+      <c r="I16" s="3"/>
+      <c r="J16" s="17">
+        <v>46160</v>
+      </c>
+      <c r="K16" s="21">
+        <f t="shared" si="1"/>
+        <v>154.37599999999989</v>
+      </c>
+      <c r="L16" s="15">
+        <v>221</v>
+      </c>
+      <c r="M16" s="1"/>
+      <c r="N16" s="1"/>
+      <c r="O16" s="1"/>
+      <c r="P16" s="1"/>
+      <c r="Q16" s="1"/>
+      <c r="AB16" s="1"/>
+      <c r="AE16" s="1"/>
+      <c r="AF16" s="1"/>
+      <c r="AG16" s="1"/>
+    </row>
+    <row r="17" ht="19.5" customHeight="1">
+      <c r="A17" s="10" t="s">
+        <v>48</v>
+      </c>
+      <c r="B17" s="10" t="s">
+        <v>43</v>
+      </c>
+      <c r="C17" s="19" t="s">
+        <v>49</v>
+      </c>
+      <c r="D17" s="10" t="s">
+        <v>17</v>
+      </c>
+      <c r="E17" s="10" t="s">
+        <v>12</v>
+      </c>
+      <c r="F17" s="19" t="s">
+        <v>45</v>
+      </c>
+      <c r="G17" s="19">
         <v>11</v>
       </c>
-      <c r="E3" s="8" t="s">
+      <c r="H17" s="27">
+        <v>46166</v>
+      </c>
+      <c r="I17" s="3"/>
+      <c r="J17" s="17">
+        <v>46161</v>
+      </c>
+      <c r="K17" s="21">
+        <f t="shared" si="1"/>
+        <v>132.3239999999999</v>
+      </c>
+      <c r="L17" s="15">
+        <v>196</v>
+      </c>
+      <c r="M17" s="1"/>
+      <c r="N17" s="1"/>
+      <c r="O17" s="1"/>
+      <c r="P17" s="1"/>
+      <c r="Q17" s="1"/>
+      <c r="AB17" s="1"/>
+      <c r="AE17" s="1"/>
+      <c r="AF17" s="1"/>
+      <c r="AG17" s="1"/>
+    </row>
+    <row r="18" ht="19.5" customHeight="1">
+      <c r="A18" s="24"/>
+      <c r="B18" s="24"/>
+      <c r="C18" s="15"/>
+      <c r="D18" s="24"/>
+      <c r="E18" s="24"/>
+      <c r="F18" s="28"/>
+      <c r="G18" s="15"/>
+      <c r="H18" s="23"/>
+      <c r="I18" s="3"/>
+      <c r="J18" s="17">
+        <v>46162</v>
+      </c>
+      <c r="K18" s="21">
+        <f t="shared" si="1"/>
+        <v>110.27199999999991</v>
+      </c>
+      <c r="L18" s="15">
+        <v>171</v>
+      </c>
+      <c r="M18" s="1"/>
+      <c r="N18" s="1"/>
+      <c r="O18" s="1"/>
+      <c r="P18" s="1"/>
+      <c r="Q18" s="1"/>
+      <c r="AB18" s="1"/>
+      <c r="AE18" s="1"/>
+      <c r="AF18" s="1"/>
+      <c r="AG18" s="1"/>
+    </row>
+    <row r="19" ht="19.5" customHeight="1">
+      <c r="A19" s="10" t="s">
+        <v>50</v>
+      </c>
+      <c r="B19" s="10" t="s">
+        <v>51</v>
+      </c>
+      <c r="C19" s="10" t="s">
+        <v>52</v>
+      </c>
+      <c r="D19" s="10" t="s">
+        <v>53</v>
+      </c>
+      <c r="E19" s="10" t="s">
         <v>12</v>
       </c>
-      <c r="F3" s="8" t="s">
-        <v>13</v>
-      </c>
-      <c r="G3" s="9">
-        <v>28</v>
-      </c>
-      <c r="H3" s="10"/>
-      <c r="I3" s="2"/>
-      <c r="J3" s="7" t="s">
-        <v>17</v>
-      </c>
-      <c r="K3" s="7" t="s">
-        <v>18</v>
-      </c>
-      <c r="L3" s="7" t="s">
-        <v>19</v>
-      </c>
-    </row>
-    <row r="4" ht="19.5" customHeight="1">
-      <c r="A4" s="12"/>
-      <c r="B4" s="13"/>
-      <c r="C4" s="13"/>
-      <c r="D4" s="13"/>
-      <c r="E4" s="13"/>
-      <c r="F4" s="13"/>
-      <c r="G4" s="13"/>
-      <c r="H4" s="14"/>
-      <c r="J4" s="15">
-        <v>46148</v>
-      </c>
-      <c r="K4" s="14">
-        <f>G60</f>
-        <v>419</v>
-      </c>
-      <c r="L4" s="14">
-        <f>G60</f>
-        <v>419</v>
-      </c>
-    </row>
-    <row r="5" ht="19.5" customHeight="1">
-      <c r="A5" s="16" t="s">
-        <v>20</v>
-      </c>
-      <c r="B5" s="16" t="s">
-        <v>21</v>
-      </c>
-      <c r="C5" s="16" t="s">
-        <v>22</v>
-      </c>
-      <c r="D5" s="16" t="s">
-        <v>11</v>
-      </c>
-      <c r="E5" s="16" t="s">
-        <v>23</v>
-      </c>
-      <c r="F5" s="16" t="s">
-        <v>24</v>
-      </c>
-      <c r="G5" s="17">
-        <v>27</v>
-      </c>
-      <c r="H5" s="18"/>
-      <c r="I5" s="2"/>
-      <c r="J5" s="15">
-        <v>46149</v>
-      </c>
-      <c r="K5" s="19">
-        <f>K4-22.052</f>
-        <v>396.94799999999998</v>
-      </c>
-      <c r="L5" s="14">
-        <v>419</v>
-      </c>
-    </row>
-    <row r="6" ht="19.5" customHeight="1">
-      <c r="A6" s="16" t="s">
-        <v>25</v>
-      </c>
-      <c r="B6" s="16" t="s">
-        <v>21</v>
-      </c>
-      <c r="C6" s="16" t="s">
-        <v>26</v>
-      </c>
-      <c r="D6" s="16" t="s">
-        <v>27</v>
-      </c>
-      <c r="E6" s="16" t="s">
-        <v>23</v>
-      </c>
-      <c r="F6" s="16" t="s">
-        <v>28</v>
-      </c>
-      <c r="G6" s="20">
-        <v>28</v>
-      </c>
-      <c r="H6" s="18"/>
-      <c r="I6" s="2"/>
-      <c r="J6" s="15">
-        <v>46150</v>
-      </c>
-      <c r="K6" s="19">
-        <f>K5-22.052</f>
-        <v>374.89599999999996</v>
-      </c>
-      <c r="L6" s="14">
-        <v>419</v>
-      </c>
-    </row>
-    <row r="7" ht="19.5" customHeight="1">
-      <c r="A7" s="14"/>
-      <c r="B7" s="14"/>
-      <c r="C7" s="14"/>
-      <c r="D7" s="14"/>
-      <c r="E7" s="14"/>
-      <c r="F7" s="14"/>
-      <c r="G7" s="14"/>
-      <c r="H7" s="14"/>
-      <c r="I7" s="2"/>
-      <c r="J7" s="15">
-        <v>46151</v>
-      </c>
-      <c r="K7" s="19">
-        <f>K6-22.052</f>
-        <v>352.84399999999994</v>
-      </c>
-      <c r="L7" s="14">
-        <v>419</v>
-      </c>
-    </row>
-    <row r="8" ht="19.5" customHeight="1">
-      <c r="A8" s="21" t="s">
-        <v>29</v>
-      </c>
-      <c r="B8" s="21" t="s">
-        <v>30</v>
-      </c>
-      <c r="C8" s="21" t="s">
-        <v>31</v>
-      </c>
-      <c r="D8" s="22" t="s">
-        <v>32</v>
-      </c>
-      <c r="E8" s="23" t="s">
-        <v>33</v>
-      </c>
-      <c r="F8" s="21" t="s">
-        <v>31</v>
-      </c>
-      <c r="G8" s="22">
-        <v>21</v>
-      </c>
-      <c r="H8" s="24">
+      <c r="F19" s="10" t="s">
+        <v>54</v>
+      </c>
+      <c r="G19" s="19">
+        <v>2</v>
+      </c>
+      <c r="H19" s="29">
+        <v>46160</v>
+      </c>
+      <c r="I19" s="3"/>
+      <c r="J19" s="17">
+        <v>46163</v>
+      </c>
+      <c r="K19" s="21">
+        <f t="shared" si="1"/>
+        <v>88.219999999999914</v>
+      </c>
+      <c r="L19" s="15">
+        <v>136</v>
+      </c>
+      <c r="M19" s="1"/>
+      <c r="N19" s="1"/>
+      <c r="O19" s="1"/>
+      <c r="P19" s="1"/>
+      <c r="Q19" s="1"/>
+      <c r="AB19" s="1"/>
+      <c r="AE19" s="1"/>
+      <c r="AF19" s="1"/>
+      <c r="AG19" s="1"/>
+    </row>
+    <row r="20" ht="19.5" customHeight="1">
+      <c r="A20" s="10" t="s">
+        <v>55</v>
+      </c>
+      <c r="B20" s="10" t="s">
+        <v>51</v>
+      </c>
+      <c r="C20" s="10" t="s">
+        <v>56</v>
+      </c>
+      <c r="D20" s="10" t="s">
+        <v>53</v>
+      </c>
+      <c r="E20" s="10" t="s">
+        <v>12</v>
+      </c>
+      <c r="F20" s="10" t="s">
+        <v>57</v>
+      </c>
+      <c r="G20" s="19">
+        <v>2</v>
+      </c>
+      <c r="H20" s="22">
+        <v>46160</v>
+      </c>
+      <c r="I20" s="3"/>
+      <c r="J20" s="17">
+        <v>46164</v>
+      </c>
+      <c r="K20" s="21">
+        <f t="shared" si="1"/>
+        <v>66.167999999999921</v>
+      </c>
+      <c r="L20" s="15">
+        <v>111</v>
+      </c>
+      <c r="M20" s="1"/>
+      <c r="N20" s="1"/>
+      <c r="O20" s="1"/>
+      <c r="P20" s="1"/>
+      <c r="Q20" s="1"/>
+      <c r="AB20" s="1"/>
+      <c r="AE20" s="1"/>
+      <c r="AF20" s="1"/>
+      <c r="AG20" s="1"/>
+    </row>
+    <row r="21" ht="19.5" customHeight="1">
+      <c r="A21" s="10" t="s">
+        <v>58</v>
+      </c>
+      <c r="B21" s="10" t="s">
+        <v>51</v>
+      </c>
+      <c r="C21" s="10" t="s">
+        <v>59</v>
+      </c>
+      <c r="D21" s="10" t="s">
+        <v>53</v>
+      </c>
+      <c r="E21" s="10" t="s">
+        <v>12</v>
+      </c>
+      <c r="F21" s="10" t="s">
+        <v>60</v>
+      </c>
+      <c r="G21" s="19">
+        <v>2</v>
+      </c>
+      <c r="H21" s="22">
+        <v>46160</v>
+      </c>
+      <c r="I21" s="3"/>
+      <c r="J21" s="17">
+        <v>46165</v>
+      </c>
+      <c r="K21" s="21">
+        <f t="shared" si="1"/>
+        <v>44.115999999999921</v>
+      </c>
+      <c r="L21" s="15">
+        <v>86</v>
+      </c>
+      <c r="M21" s="1"/>
+      <c r="N21" s="1"/>
+      <c r="O21" s="1"/>
+      <c r="P21" s="1"/>
+      <c r="Q21" s="1"/>
+      <c r="AB21" s="1"/>
+      <c r="AE21" s="1"/>
+      <c r="AF21" s="1"/>
+      <c r="AG21" s="1"/>
+    </row>
+    <row r="22" ht="19.5" customHeight="1">
+      <c r="A22" s="10" t="s">
+        <v>61</v>
+      </c>
+      <c r="B22" s="10" t="s">
+        <v>51</v>
+      </c>
+      <c r="C22" s="10" t="s">
+        <v>62</v>
+      </c>
+      <c r="D22" s="10" t="s">
+        <v>53</v>
+      </c>
+      <c r="E22" s="10" t="s">
+        <v>12</v>
+      </c>
+      <c r="F22" s="10" t="s">
+        <v>63</v>
+      </c>
+      <c r="G22" s="19">
+        <v>2</v>
+      </c>
+      <c r="H22" s="22">
         <v>46166</v>
       </c>
-      <c r="I8" s="2"/>
-      <c r="J8" s="15">
-        <v>46152</v>
-      </c>
-      <c r="K8" s="19">
-        <f>K7-22.052</f>
-        <v>330.79199999999992</v>
-      </c>
-      <c r="L8" s="14">
-        <v>419</v>
-      </c>
-    </row>
-    <row r="9" ht="19.5" customHeight="1">
-      <c r="A9" s="21" t="s">
-        <v>34</v>
-      </c>
-      <c r="B9" s="21" t="s">
-        <v>30</v>
-      </c>
-      <c r="C9" s="21" t="s">
-        <v>35</v>
-      </c>
-      <c r="D9" s="22" t="s">
-        <v>32</v>
-      </c>
-      <c r="E9" s="23" t="s">
-        <v>33</v>
-      </c>
-      <c r="F9" s="21" t="s">
-        <v>31</v>
-      </c>
-      <c r="G9" s="22">
-        <v>5</v>
-      </c>
-      <c r="H9" s="25">
-        <v>46161</v>
-      </c>
-      <c r="I9" s="2"/>
-      <c r="J9" s="15">
-        <v>46153</v>
-      </c>
-      <c r="K9" s="19">
-        <f>K8-22.052</f>
-        <v>308.7399999999999</v>
-      </c>
-      <c r="L9" s="14">
-        <v>419</v>
-      </c>
-    </row>
-    <row r="10" ht="19.5" customHeight="1">
-      <c r="A10" s="21" t="s">
-        <v>36</v>
-      </c>
-      <c r="B10" s="21" t="s">
-        <v>30</v>
-      </c>
-      <c r="C10" s="21" t="s">
-        <v>37</v>
-      </c>
-      <c r="D10" s="22" t="s">
-        <v>32</v>
-      </c>
-      <c r="E10" s="23" t="s">
-        <v>33</v>
-      </c>
-      <c r="F10" s="21" t="s">
-        <v>31</v>
-      </c>
-      <c r="G10" s="22">
-        <v>5</v>
-      </c>
-      <c r="H10" s="25">
-        <v>46161</v>
-      </c>
-      <c r="I10" s="2"/>
-      <c r="J10" s="15">
-        <v>46154</v>
-      </c>
-      <c r="K10" s="19">
-        <f>K9-22.052</f>
-        <v>286.68799999999987</v>
-      </c>
-      <c r="L10" s="14">
-        <v>419</v>
-      </c>
-    </row>
-    <row r="11" ht="19.5" customHeight="1">
-      <c r="A11" s="21" t="s">
-        <v>38</v>
-      </c>
-      <c r="B11" s="21" t="s">
-        <v>30</v>
-      </c>
-      <c r="C11" s="21" t="s">
-        <v>39</v>
-      </c>
-      <c r="D11" s="22" t="s">
-        <v>32</v>
-      </c>
-      <c r="E11" s="23" t="s">
-        <v>33</v>
-      </c>
-      <c r="F11" s="21" t="s">
-        <v>31</v>
-      </c>
-      <c r="G11" s="22">
-        <v>6</v>
-      </c>
-      <c r="H11" s="24">
+      <c r="I22" s="3"/>
+      <c r="J22" s="17">
         <v>46166</v>
       </c>
-      <c r="I11" s="2"/>
-      <c r="J11" s="15">
-        <v>46155</v>
-      </c>
-      <c r="K11" s="19">
-        <f>K10-22.052</f>
-        <v>264.63599999999985</v>
-      </c>
-      <c r="L11" s="14">
-        <v>419</v>
-      </c>
-    </row>
-    <row r="12" ht="19.5" customHeight="1">
-      <c r="A12" s="21" t="s">
-        <v>40</v>
-      </c>
-      <c r="B12" s="21" t="s">
-        <v>30</v>
-      </c>
-      <c r="C12" s="21" t="s">
-        <v>41</v>
-      </c>
-      <c r="D12" s="22" t="s">
-        <v>32</v>
-      </c>
-      <c r="E12" s="23" t="s">
-        <v>33</v>
-      </c>
-      <c r="F12" s="21" t="s">
-        <v>31</v>
-      </c>
-      <c r="G12" s="22">
-        <v>5</v>
-      </c>
-      <c r="H12" s="25">
-        <v>46161</v>
-      </c>
-      <c r="I12" s="2"/>
-      <c r="J12" s="15">
-        <v>46156</v>
-      </c>
-      <c r="K12" s="19">
-        <f>K11-22.052</f>
-        <v>242.58399999999986</v>
-      </c>
-      <c r="L12" s="14">
-        <v>419</v>
-      </c>
-    </row>
-    <row r="13" ht="19.5" customHeight="1">
-      <c r="A13" s="14"/>
-      <c r="B13" s="14"/>
-      <c r="C13" s="14"/>
-      <c r="D13" s="14"/>
-      <c r="E13" s="14"/>
-      <c r="F13" s="14"/>
-      <c r="G13" s="14"/>
-      <c r="H13" s="14"/>
-      <c r="I13" s="2"/>
-      <c r="J13" s="15">
-        <v>46157</v>
-      </c>
-      <c r="K13" s="19">
-        <f>K12-22.052</f>
-        <v>220.53199999999987</v>
-      </c>
-      <c r="L13" s="14">
-        <v>419</v>
-      </c>
-    </row>
-    <row r="14" ht="19.5" customHeight="1">
-      <c r="A14" s="23" t="s">
-        <v>42</v>
-      </c>
-      <c r="B14" s="23" t="s">
-        <v>42</v>
-      </c>
-      <c r="C14" s="23" t="s">
+      <c r="K22" s="21">
+        <f t="shared" si="1"/>
+        <v>22.063999999999922</v>
+      </c>
+      <c r="L22" s="15">
         <v>43</v>
       </c>
-      <c r="D14" s="23" t="s">
-        <v>44</v>
-      </c>
-      <c r="E14" s="23" t="s">
-        <v>33</v>
-      </c>
-      <c r="F14" s="23" t="s">
-        <v>45</v>
-      </c>
-      <c r="G14" s="22">
-        <v>34</v>
-      </c>
-      <c r="H14" s="24">
+      <c r="M22" s="1"/>
+      <c r="N22" s="1"/>
+      <c r="O22" s="1"/>
+      <c r="P22" s="1"/>
+      <c r="AB22" s="1"/>
+      <c r="AE22" s="1"/>
+      <c r="AF22" s="1"/>
+      <c r="AG22" s="1"/>
+    </row>
+    <row r="23" ht="19.5" customHeight="1">
+      <c r="A23" s="10" t="s">
+        <v>64</v>
+      </c>
+      <c r="B23" s="30" t="s">
+        <v>51</v>
+      </c>
+      <c r="C23" s="10" t="s">
+        <v>65</v>
+      </c>
+      <c r="D23" s="10" t="s">
+        <v>53</v>
+      </c>
+      <c r="E23" s="10" t="s">
+        <v>12</v>
+      </c>
+      <c r="F23" s="10" t="s">
+        <v>66</v>
+      </c>
+      <c r="G23" s="19">
+        <v>2</v>
+      </c>
+      <c r="H23" s="22">
         <v>46166</v>
       </c>
-      <c r="I14" s="2"/>
-      <c r="J14" s="15">
-        <v>46158</v>
-      </c>
-      <c r="K14" s="19">
-        <f>K13-22.052</f>
-        <v>198.47999999999988</v>
-      </c>
-      <c r="L14" s="14">
-        <v>419</v>
-      </c>
-      <c r="M14" s="1"/>
-    </row>
-    <row r="15" ht="19.5" customHeight="1">
-      <c r="A15" s="14"/>
-      <c r="B15" s="14"/>
-      <c r="C15" s="14"/>
-      <c r="D15" s="14"/>
-      <c r="E15" s="14"/>
-      <c r="F15" s="14"/>
-      <c r="G15" s="14"/>
-      <c r="H15" s="14"/>
-      <c r="I15" s="2"/>
-      <c r="J15" s="15">
-        <v>46159</v>
-      </c>
-      <c r="K15" s="19">
-        <f>K14-22.052</f>
-        <v>176.42799999999988</v>
-      </c>
-      <c r="L15" s="14">
-        <v>419</v>
-      </c>
-      <c r="M15" s="1"/>
-    </row>
-    <row r="16" ht="19.5" customHeight="1">
-      <c r="A16" s="23" t="s">
-        <v>46</v>
-      </c>
-      <c r="B16" s="23" t="s">
-        <v>46</v>
-      </c>
-      <c r="C16" s="23" t="s">
-        <v>47</v>
-      </c>
-      <c r="D16" s="23" t="s">
-        <v>48</v>
-      </c>
-      <c r="E16" s="23" t="s">
-        <v>33</v>
-      </c>
-      <c r="F16" s="23" t="s">
-        <v>49</v>
-      </c>
-      <c r="G16" s="22">
-        <v>55</v>
-      </c>
-      <c r="H16" s="24">
+      <c r="I23" s="3"/>
+      <c r="J23" s="17">
+        <v>46167</v>
+      </c>
+      <c r="K23" s="21">
+        <f t="shared" si="1"/>
+        <v>0.011999999999922295</v>
+      </c>
+      <c r="L23" s="15">
+        <v>0</v>
+      </c>
+      <c r="M23" s="1"/>
+      <c r="N23" s="1"/>
+      <c r="O23" s="1"/>
+      <c r="P23" s="1"/>
+      <c r="AB23" s="1"/>
+      <c r="AE23" s="1"/>
+      <c r="AF23" s="1"/>
+      <c r="AG23" s="1"/>
+    </row>
+    <row r="24" ht="19.5" customHeight="1">
+      <c r="A24" s="10" t="s">
+        <v>67</v>
+      </c>
+      <c r="B24" s="30" t="s">
+        <v>51</v>
+      </c>
+      <c r="C24" s="10" t="s">
+        <v>68</v>
+      </c>
+      <c r="D24" s="10" t="s">
+        <v>53</v>
+      </c>
+      <c r="E24" s="10" t="s">
+        <v>12</v>
+      </c>
+      <c r="F24" s="10" t="s">
+        <v>69</v>
+      </c>
+      <c r="G24" s="19">
+        <v>2</v>
+      </c>
+      <c r="H24" s="22">
         <v>46166</v>
       </c>
-      <c r="I16" s="2"/>
-      <c r="J16" s="15">
-        <v>46160</v>
-      </c>
-      <c r="K16" s="19">
-        <f>K15-22.052</f>
-        <v>154.37599999999989</v>
-      </c>
-      <c r="L16" s="14">
-        <f>L15-K27</f>
-        <v>405</v>
-      </c>
-      <c r="M16" s="1"/>
-    </row>
-    <row r="17" ht="19.5" customHeight="1">
-      <c r="A17" s="26"/>
-      <c r="B17" s="26"/>
-      <c r="C17" s="26"/>
-      <c r="D17" s="26"/>
-      <c r="E17" s="26"/>
-      <c r="F17" s="26"/>
-      <c r="G17" s="14"/>
-      <c r="H17" s="14"/>
-      <c r="I17" s="2"/>
-      <c r="J17" s="15">
-        <v>46161</v>
-      </c>
-      <c r="K17" s="19">
-        <f>K16-22.052</f>
-        <v>132.3239999999999</v>
-      </c>
-      <c r="L17" s="14">
-        <f>L16-K28</f>
-        <v>388</v>
-      </c>
-      <c r="M17" s="1"/>
-    </row>
-    <row r="18" ht="19.5" customHeight="1">
-      <c r="A18" s="16" t="s">
-        <v>50</v>
-      </c>
-      <c r="B18" s="16" t="s">
-        <v>51</v>
-      </c>
-      <c r="C18" s="20" t="s">
-        <v>52</v>
-      </c>
-      <c r="D18" s="16" t="s">
-        <v>44</v>
-      </c>
-      <c r="E18" s="16" t="s">
-        <v>23</v>
-      </c>
-      <c r="F18" s="27" t="s">
-        <v>53</v>
-      </c>
-      <c r="G18" s="20">
-        <v>21</v>
-      </c>
-      <c r="H18" s="18"/>
-      <c r="I18" s="2"/>
-      <c r="J18" s="15">
-        <v>46162</v>
-      </c>
-      <c r="K18" s="19">
-        <f>K17-22.052</f>
-        <v>110.27199999999991</v>
-      </c>
-      <c r="L18" s="14">
-        <v>388</v>
-      </c>
-      <c r="M18" s="1"/>
-    </row>
-    <row r="19" ht="19.5" customHeight="1">
-      <c r="A19" s="16" t="s">
-        <v>54</v>
-      </c>
-      <c r="B19" s="16" t="s">
-        <v>51</v>
-      </c>
-      <c r="C19" s="20" t="s">
-        <v>55</v>
-      </c>
-      <c r="D19" s="16" t="s">
-        <v>48</v>
-      </c>
-      <c r="E19" s="16" t="s">
-        <v>23</v>
-      </c>
-      <c r="F19" s="20" t="s">
-        <v>53</v>
-      </c>
-      <c r="G19" s="20">
-        <v>10</v>
-      </c>
-      <c r="H19" s="18"/>
-      <c r="I19" s="2"/>
-      <c r="J19" s="15">
-        <v>46163</v>
-      </c>
-      <c r="K19" s="19">
-        <f>K18-22.052</f>
-        <v>88.219999999999914</v>
-      </c>
-      <c r="L19" s="14">
-        <v>388</v>
-      </c>
-      <c r="M19" s="1"/>
-    </row>
-    <row r="20" ht="19.5" customHeight="1">
-      <c r="A20" s="23" t="s">
-        <v>56</v>
-      </c>
-      <c r="B20" s="23" t="s">
-        <v>51</v>
-      </c>
-      <c r="C20" s="22" t="s">
-        <v>57</v>
-      </c>
-      <c r="D20" s="23" t="s">
-        <v>27</v>
-      </c>
-      <c r="E20" s="23" t="s">
-        <v>33</v>
-      </c>
-      <c r="F20" s="22" t="s">
-        <v>53</v>
-      </c>
-      <c r="G20" s="22">
-        <v>11</v>
-      </c>
-      <c r="H20" s="24">
-        <v>46166</v>
-      </c>
-      <c r="I20" s="2"/>
-      <c r="J20" s="15">
-        <v>46164</v>
-      </c>
-      <c r="K20" s="19">
-        <f>K19-22.052</f>
-        <v>66.167999999999921</v>
-      </c>
-      <c r="L20" s="14">
-        <v>388</v>
-      </c>
-      <c r="M20" s="1"/>
-    </row>
-    <row r="21" ht="19.5" customHeight="1">
-      <c r="A21" s="26"/>
-      <c r="B21" s="26"/>
-      <c r="C21" s="14"/>
-      <c r="D21" s="26"/>
-      <c r="E21" s="26"/>
-      <c r="F21" s="13"/>
-      <c r="G21" s="14"/>
-      <c r="H21" s="14"/>
-      <c r="I21" s="2"/>
-      <c r="J21" s="15">
-        <v>46165</v>
-      </c>
-      <c r="K21" s="19">
-        <f>K20-22.052</f>
-        <v>44.115999999999921</v>
-      </c>
-      <c r="L21" s="14">
-        <v>388</v>
-      </c>
-      <c r="M21" s="1"/>
-    </row>
-    <row r="22" ht="19.5" customHeight="1">
-      <c r="A22" s="23" t="s">
-        <v>58</v>
-      </c>
-      <c r="B22" s="23" t="s">
-        <v>59</v>
-      </c>
-      <c r="C22" s="23" t="s">
-        <v>60</v>
-      </c>
-      <c r="D22" s="23" t="s">
-        <v>61</v>
-      </c>
-      <c r="E22" s="23" t="s">
-        <v>33</v>
-      </c>
-      <c r="F22" s="23" t="s">
-        <v>62</v>
-      </c>
-      <c r="G22" s="22">
-        <v>2</v>
-      </c>
-      <c r="H22" s="28">
-        <v>46160</v>
-      </c>
-      <c r="I22" s="2"/>
-      <c r="J22" s="15">
-        <v>46166</v>
-      </c>
-      <c r="K22" s="19">
-        <f>K21-22.052</f>
-        <v>22.063999999999922</v>
-      </c>
-      <c r="L22" s="14">
-        <f>L21-K29</f>
-        <v>129</v>
-      </c>
-      <c r="M22" s="1"/>
-    </row>
-    <row r="23" ht="19.5" customHeight="1">
-      <c r="A23" s="23" t="s">
-        <v>63</v>
-      </c>
-      <c r="B23" s="23" t="s">
-        <v>59</v>
-      </c>
-      <c r="C23" s="23" t="s">
-        <v>64</v>
-      </c>
-      <c r="D23" s="23" t="s">
-        <v>61</v>
-      </c>
-      <c r="E23" s="23" t="s">
-        <v>33</v>
-      </c>
-      <c r="F23" s="23" t="s">
-        <v>65</v>
-      </c>
-      <c r="G23" s="22">
-        <v>2</v>
-      </c>
-      <c r="H23" s="29">
-        <v>46160</v>
-      </c>
-      <c r="I23" s="2"/>
-      <c r="J23" s="15">
-        <v>46167</v>
-      </c>
-      <c r="K23" s="19">
-        <f>K22-22.052</f>
-        <v>0.011999999999922295</v>
-      </c>
-      <c r="L23" s="14">
-        <f>L22-K30</f>
-        <v>0</v>
-      </c>
-      <c r="M23" s="1"/>
-    </row>
-    <row r="24" ht="19.5" customHeight="1">
-      <c r="A24" s="23" t="s">
-        <v>66</v>
-      </c>
-      <c r="B24" s="23" t="s">
-        <v>59</v>
-      </c>
-      <c r="C24" s="23" t="s">
-        <v>67</v>
-      </c>
-      <c r="D24" s="23" t="s">
-        <v>61</v>
-      </c>
-      <c r="E24" s="23" t="s">
-        <v>33</v>
-      </c>
-      <c r="F24" s="23" t="s">
-        <v>68</v>
-      </c>
-      <c r="G24" s="22">
-        <v>2</v>
-      </c>
-      <c r="H24" s="29">
-        <v>46160</v>
-      </c>
-      <c r="I24" s="2"/>
+      <c r="I24" s="3"/>
       <c r="J24" s="1"/>
-      <c r="K24" s="3"/>
+      <c r="K24" s="4"/>
       <c r="L24" s="1"/>
       <c r="M24" s="1"/>
+      <c r="N24" s="1"/>
+      <c r="O24" s="1"/>
+      <c r="P24" s="1"/>
+      <c r="AB24" s="1"/>
+      <c r="AE24" s="1"/>
+      <c r="AF24" s="1"/>
+      <c r="AG24" s="1"/>
     </row>
     <row r="25" ht="19.5" customHeight="1">
-      <c r="A25" s="23" t="s">
-        <v>69</v>
-      </c>
-      <c r="B25" s="23" t="s">
-        <v>59</v>
-      </c>
-      <c r="C25" s="23" t="s">
+      <c r="A25" s="10" t="s">
         <v>70</v>
       </c>
-      <c r="D25" s="23" t="s">
-        <v>61</v>
-      </c>
-      <c r="E25" s="23" t="s">
-        <v>33</v>
-      </c>
-      <c r="F25" s="23" t="s">
+      <c r="B25" s="30" t="s">
+        <v>51</v>
+      </c>
+      <c r="C25" s="10" t="s">
         <v>71</v>
       </c>
-      <c r="G25" s="22">
+      <c r="D25" s="10" t="s">
+        <v>53</v>
+      </c>
+      <c r="E25" s="10" t="s">
+        <v>12</v>
+      </c>
+      <c r="F25" s="10" t="s">
+        <v>72</v>
+      </c>
+      <c r="G25" s="19">
         <v>2</v>
       </c>
-      <c r="H25" s="24">
+      <c r="H25" s="22">
         <v>46166</v>
       </c>
-      <c r="I25" s="2"/>
+      <c r="I25" s="3"/>
       <c r="J25" s="1"/>
       <c r="K25" s="1"/>
       <c r="L25" s="1"/>
       <c r="M25" s="1"/>
+      <c r="N25" s="1"/>
     </row>
     <row r="26" ht="19.5" customHeight="1">
-      <c r="A26" s="23" t="s">
-        <v>72</v>
+      <c r="A26" s="10" t="s">
+        <v>73</v>
       </c>
       <c r="B26" s="30" t="s">
-        <v>59</v>
-      </c>
-      <c r="C26" s="23" t="s">
-        <v>73</v>
-      </c>
-      <c r="D26" s="23" t="s">
-        <v>61</v>
-      </c>
-      <c r="E26" s="23" t="s">
-        <v>33</v>
-      </c>
-      <c r="F26" s="23" t="s">
+        <v>51</v>
+      </c>
+      <c r="C26" s="10" t="s">
         <v>74</v>
       </c>
-      <c r="G26" s="22">
+      <c r="D26" s="10" t="s">
+        <v>53</v>
+      </c>
+      <c r="E26" s="10" t="s">
+        <v>12</v>
+      </c>
+      <c r="F26" s="10" t="s">
+        <v>75</v>
+      </c>
+      <c r="G26" s="19">
         <v>2</v>
       </c>
-      <c r="H26" s="24">
-        <v>46166</v>
-      </c>
-      <c r="I26" s="2"/>
-      <c r="J26" s="2"/>
-      <c r="K26" s="2"/>
+      <c r="H26" s="22">
+        <v>46160</v>
+      </c>
+      <c r="I26" s="3"/>
+      <c r="J26" s="3"/>
+      <c r="K26" s="3"/>
       <c r="L26" s="1"/>
       <c r="M26" s="1"/>
+      <c r="N26" s="1"/>
     </row>
     <row r="27" ht="19.5" customHeight="1">
-      <c r="A27" s="23" t="s">
-        <v>75</v>
+      <c r="A27" s="10" t="s">
+        <v>76</v>
       </c>
       <c r="B27" s="30" t="s">
-        <v>59</v>
-      </c>
-      <c r="C27" s="23" t="s">
-        <v>76</v>
-      </c>
-      <c r="D27" s="23" t="s">
-        <v>61</v>
-      </c>
-      <c r="E27" s="23" t="s">
-        <v>33</v>
-      </c>
-      <c r="F27" s="23" t="s">
+        <v>51</v>
+      </c>
+      <c r="C27" s="10" t="s">
         <v>77</v>
       </c>
-      <c r="G27" s="22">
+      <c r="D27" s="10" t="s">
+        <v>53</v>
+      </c>
+      <c r="E27" s="10" t="s">
+        <v>12</v>
+      </c>
+      <c r="F27" s="10" t="s">
+        <v>78</v>
+      </c>
+      <c r="G27" s="19">
         <v>2</v>
       </c>
-      <c r="H27" s="24">
-        <v>46166</v>
-      </c>
-      <c r="I27" s="2"/>
-      <c r="J27" s="31">
+      <c r="H27" s="22">
         <v>46160</v>
       </c>
-      <c r="K27" s="32">
-        <f>SUM(G22,G23,G24,G29,G30,G31,G32)</f>
-        <v>14</v>
-      </c>
+      <c r="I27" s="3"/>
+      <c r="J27" s="31"/>
+      <c r="K27" s="31"/>
       <c r="L27" s="1"/>
       <c r="M27" s="1"/>
+      <c r="N27" s="1"/>
     </row>
     <row r="28" ht="19.5" customHeight="1">
-      <c r="A28" s="23" t="s">
-        <v>78</v>
+      <c r="A28" s="10" t="s">
+        <v>79</v>
       </c>
       <c r="B28" s="30" t="s">
-        <v>59</v>
-      </c>
-      <c r="C28" s="23" t="s">
-        <v>79</v>
-      </c>
-      <c r="D28" s="23" t="s">
-        <v>61</v>
-      </c>
-      <c r="E28" s="23" t="s">
-        <v>33</v>
-      </c>
-      <c r="F28" s="23" t="s">
+        <v>51</v>
+      </c>
+      <c r="C28" s="10" t="s">
         <v>80</v>
       </c>
-      <c r="G28" s="22">
+      <c r="D28" s="10" t="s">
+        <v>53</v>
+      </c>
+      <c r="E28" s="10" t="s">
+        <v>12</v>
+      </c>
+      <c r="F28" s="10" t="s">
+        <v>81</v>
+      </c>
+      <c r="G28" s="19">
         <v>2</v>
       </c>
-      <c r="H28" s="24">
-        <v>46166</v>
-      </c>
-      <c r="I28" s="2"/>
-      <c r="J28" s="33">
-        <v>46161</v>
-      </c>
-      <c r="K28" s="32">
-        <f>SUM(G9,G10,G12,G34)</f>
-        <v>17</v>
-      </c>
-      <c r="L28" s="2"/>
+      <c r="H28" s="22">
+        <v>46160</v>
+      </c>
+      <c r="I28" s="3"/>
+      <c r="J28" s="31"/>
+      <c r="K28" s="31"/>
+      <c r="L28" s="3"/>
       <c r="M28" s="1"/>
+      <c r="N28" s="1"/>
     </row>
     <row r="29" ht="19.5" customHeight="1">
-      <c r="A29" s="23" t="s">
-        <v>81</v>
-      </c>
-      <c r="B29" s="30" t="s">
-        <v>59</v>
-      </c>
-      <c r="C29" s="23" t="s">
+      <c r="A29" s="10" t="s">
         <v>82</v>
       </c>
-      <c r="D29" s="23" t="s">
-        <v>61</v>
-      </c>
-      <c r="E29" s="23" t="s">
-        <v>33</v>
-      </c>
-      <c r="F29" s="23" t="s">
+      <c r="B29" s="10" t="s">
+        <v>51</v>
+      </c>
+      <c r="C29" s="10" t="s">
         <v>83</v>
       </c>
-      <c r="G29" s="22">
+      <c r="D29" s="10" t="s">
+        <v>53</v>
+      </c>
+      <c r="E29" s="10" t="s">
+        <v>12</v>
+      </c>
+      <c r="F29" s="10" t="s">
+        <v>84</v>
+      </c>
+      <c r="G29" s="19">
         <v>2</v>
       </c>
       <c r="H29" s="29">
         <v>46160</v>
       </c>
-      <c r="I29" s="2"/>
-      <c r="J29" s="34">
+      <c r="I29" s="3"/>
+      <c r="J29" s="31"/>
+      <c r="K29" s="31"/>
+      <c r="L29" s="3"/>
+      <c r="M29" s="1"/>
+      <c r="N29" s="1"/>
+    </row>
+    <row r="30" ht="19.5" customHeight="1">
+      <c r="A30" s="18" t="s">
+        <v>85</v>
+      </c>
+      <c r="B30" s="30" t="s">
+        <v>51</v>
+      </c>
+      <c r="C30" s="10" t="s">
+        <v>86</v>
+      </c>
+      <c r="D30" s="10" t="s">
+        <v>87</v>
+      </c>
+      <c r="E30" s="10" t="s">
+        <v>12</v>
+      </c>
+      <c r="F30" s="10" t="s">
+        <v>88</v>
+      </c>
+      <c r="G30" s="19">
+        <v>2</v>
+      </c>
+      <c r="H30" s="32">
+        <v>46161</v>
+      </c>
+      <c r="I30" s="3"/>
+      <c r="J30" s="31"/>
+      <c r="K30" s="31"/>
+      <c r="L30" s="3"/>
+      <c r="M30" s="1"/>
+      <c r="N30" s="1"/>
+    </row>
+    <row r="31" ht="19.5" customHeight="1">
+      <c r="A31" s="18" t="s">
+        <v>89</v>
+      </c>
+      <c r="B31" s="30" t="s">
+        <v>51</v>
+      </c>
+      <c r="C31" s="10" t="s">
+        <v>90</v>
+      </c>
+      <c r="D31" s="10" t="s">
+        <v>87</v>
+      </c>
+      <c r="E31" s="10" t="s">
+        <v>12</v>
+      </c>
+      <c r="F31" s="10" t="s">
+        <v>91</v>
+      </c>
+      <c r="G31" s="14">
+        <v>2</v>
+      </c>
+      <c r="H31" s="12">
+        <v>46167</v>
+      </c>
+      <c r="I31" s="3"/>
+      <c r="J31" s="3"/>
+      <c r="K31" s="3"/>
+      <c r="L31" s="3"/>
+      <c r="M31" s="1"/>
+      <c r="N31" s="1"/>
+    </row>
+    <row r="32" ht="19.5" customHeight="1">
+      <c r="A32" s="18" t="s">
+        <v>92</v>
+      </c>
+      <c r="B32" s="30" t="s">
+        <v>51</v>
+      </c>
+      <c r="C32" s="10" t="s">
+        <v>93</v>
+      </c>
+      <c r="D32" s="10" t="s">
+        <v>94</v>
+      </c>
+      <c r="E32" s="10" t="s">
+        <v>12</v>
+      </c>
+      <c r="F32" s="10" t="s">
+        <v>95</v>
+      </c>
+      <c r="G32" s="14">
+        <v>4</v>
+      </c>
+      <c r="H32" s="12">
+        <v>46167</v>
+      </c>
+      <c r="I32" s="3"/>
+      <c r="J32" s="1"/>
+      <c r="K32" s="3"/>
+      <c r="L32" s="3"/>
+      <c r="M32" s="1"/>
+      <c r="N32" s="1"/>
+    </row>
+    <row r="33" ht="19.5" customHeight="1">
+      <c r="A33" s="18" t="s">
+        <v>96</v>
+      </c>
+      <c r="B33" s="10" t="s">
+        <v>51</v>
+      </c>
+      <c r="C33" s="10" t="s">
+        <v>97</v>
+      </c>
+      <c r="D33" s="10" t="s">
+        <v>98</v>
+      </c>
+      <c r="E33" s="10" t="s">
+        <v>12</v>
+      </c>
+      <c r="F33" s="10" t="s">
+        <v>99</v>
+      </c>
+      <c r="G33" s="19">
+        <v>2</v>
+      </c>
+      <c r="H33" s="33">
         <v>46166</v>
       </c>
-      <c r="K29" s="32">
-        <f>SUM(G11,G14,G16,G20,G25,G26,G27,G28,G37,G40,G45,G46,G49,G50,G52,G53,G56,G59)</f>
-        <v>259</v>
-      </c>
-      <c r="L29" s="2"/>
-      <c r="M29" s="1"/>
-    </row>
-    <row r="30" ht="19.5" customHeight="1">
-      <c r="A30" s="23" t="s">
-        <v>84</v>
-      </c>
-      <c r="B30" s="30" t="s">
-        <v>59</v>
-      </c>
-      <c r="C30" s="23" t="s">
-        <v>85</v>
-      </c>
-      <c r="D30" s="23" t="s">
-        <v>61</v>
-      </c>
-      <c r="E30" s="23" t="s">
-        <v>33</v>
-      </c>
-      <c r="F30" s="23" t="s">
-        <v>86</v>
-      </c>
-      <c r="G30" s="22">
+      <c r="I33" s="3"/>
+      <c r="J33" s="1"/>
+      <c r="K33" s="3"/>
+      <c r="L33" s="3"/>
+      <c r="M33" s="1"/>
+      <c r="N33" s="1"/>
+    </row>
+    <row r="34" ht="19.5" customHeight="1">
+      <c r="A34" s="18" t="s">
+        <v>100</v>
+      </c>
+      <c r="B34" s="10" t="s">
+        <v>51</v>
+      </c>
+      <c r="C34" s="10" t="s">
+        <v>101</v>
+      </c>
+      <c r="D34" s="10" t="s">
+        <v>98</v>
+      </c>
+      <c r="E34" s="10" t="s">
+        <v>12</v>
+      </c>
+      <c r="F34" s="10" t="s">
+        <v>102</v>
+      </c>
+      <c r="G34" s="14">
         <v>2</v>
       </c>
-      <c r="H30" s="29">
-        <v>46160</v>
-      </c>
-      <c r="I30" s="2"/>
-      <c r="J30" s="35">
+      <c r="H34" s="12">
         <v>46167</v>
       </c>
-      <c r="K30" s="32">
-        <f>SUM(G5,G6,G19,G35,G36,G38,G42,G55,G57)</f>
-        <v>129</v>
-      </c>
-      <c r="L30" s="2"/>
-      <c r="M30" s="1"/>
-    </row>
-    <row r="31" ht="19.5" customHeight="1">
-      <c r="A31" s="23" t="s">
-        <v>87</v>
-      </c>
-      <c r="B31" s="30" t="s">
-        <v>59</v>
-      </c>
-      <c r="C31" s="23" t="s">
-        <v>88</v>
-      </c>
-      <c r="D31" s="23" t="s">
-        <v>61</v>
-      </c>
-      <c r="E31" s="23" t="s">
-        <v>33</v>
-      </c>
-      <c r="F31" s="23" t="s">
-        <v>89</v>
-      </c>
-      <c r="G31" s="22">
-        <v>2</v>
-      </c>
-      <c r="H31" s="29">
-        <v>46160</v>
-      </c>
-      <c r="I31" s="2"/>
-      <c r="J31" s="2"/>
-      <c r="K31" s="2"/>
-      <c r="L31" s="2"/>
-      <c r="M31" s="1"/>
-    </row>
-    <row r="32" ht="19.5" customHeight="1">
-      <c r="A32" s="23" t="s">
-        <v>90</v>
-      </c>
-      <c r="B32" s="23" t="s">
-        <v>59</v>
-      </c>
-      <c r="C32" s="23" t="s">
-        <v>91</v>
-      </c>
-      <c r="D32" s="23" t="s">
-        <v>61</v>
-      </c>
-      <c r="E32" s="23" t="s">
-        <v>33</v>
-      </c>
-      <c r="F32" s="23" t="s">
-        <v>92</v>
-      </c>
-      <c r="G32" s="22">
-        <v>2</v>
-      </c>
-      <c r="H32" s="28">
-        <v>46160</v>
-      </c>
-      <c r="I32" s="2"/>
-      <c r="J32" s="1"/>
-      <c r="K32" s="2"/>
-      <c r="L32" s="2"/>
-      <c r="M32" s="1"/>
-    </row>
-    <row r="33" ht="19.5" customHeight="1">
-      <c r="A33" s="8" t="s">
-        <v>93</v>
-      </c>
-      <c r="B33" s="36" t="s">
-        <v>59</v>
-      </c>
-      <c r="C33" s="8" t="s">
-        <v>94</v>
-      </c>
-      <c r="D33" s="8" t="s">
-        <v>95</v>
-      </c>
-      <c r="E33" s="8" t="s">
+      <c r="I34" s="3"/>
+      <c r="J34" s="3"/>
+      <c r="K34" s="3"/>
+      <c r="L34" s="3"/>
+      <c r="M34" s="1"/>
+      <c r="N34" s="1"/>
+    </row>
+    <row r="35" ht="19.5" customHeight="1">
+      <c r="A35" s="24"/>
+      <c r="B35" s="24"/>
+      <c r="C35" s="24"/>
+      <c r="D35" s="24"/>
+      <c r="E35" s="24"/>
+      <c r="F35" s="24"/>
+      <c r="G35" s="15"/>
+      <c r="H35" s="34"/>
+      <c r="I35" s="3"/>
+      <c r="J35" s="3"/>
+      <c r="K35" s="3"/>
+      <c r="L35" s="3"/>
+      <c r="M35" s="1"/>
+      <c r="N35" s="1"/>
+    </row>
+    <row r="36" ht="19.5" customHeight="1">
+      <c r="A36" s="19" t="s">
+        <v>103</v>
+      </c>
+      <c r="B36" s="19" t="s">
+        <v>103</v>
+      </c>
+      <c r="C36" s="35" t="s">
+        <v>104</v>
+      </c>
+      <c r="D36" s="10" t="s">
+        <v>105</v>
+      </c>
+      <c r="E36" s="10" t="s">
         <v>12</v>
       </c>
-      <c r="F33" s="8" t="s">
-        <v>96</v>
-      </c>
-      <c r="G33" s="9">
-        <v>2</v>
-      </c>
-      <c r="H33" s="10"/>
-      <c r="I33" s="2"/>
-      <c r="J33" s="1"/>
-      <c r="K33" s="2"/>
-      <c r="L33" s="2"/>
-      <c r="M33" s="1"/>
-    </row>
-    <row r="34" ht="19.5" customHeight="1">
-      <c r="A34" s="21" t="s">
-        <v>93</v>
-      </c>
-      <c r="B34" s="30" t="s">
-        <v>59</v>
-      </c>
-      <c r="C34" s="23" t="s">
-        <v>97</v>
-      </c>
-      <c r="D34" s="23" t="s">
-        <v>95</v>
-      </c>
-      <c r="E34" s="23" t="s">
-        <v>33</v>
-      </c>
-      <c r="F34" s="23" t="s">
-        <v>98</v>
-      </c>
-      <c r="G34" s="22">
-        <v>2</v>
-      </c>
-      <c r="H34" s="37">
-        <v>46161</v>
-      </c>
-      <c r="I34" s="2"/>
-      <c r="J34" s="2"/>
-      <c r="K34" s="2"/>
-      <c r="L34" s="2"/>
-      <c r="M34" s="1"/>
-    </row>
-    <row r="35" ht="19.5" customHeight="1">
-      <c r="A35" s="38" t="s">
-        <v>99</v>
-      </c>
-      <c r="B35" s="39" t="s">
-        <v>59</v>
-      </c>
-      <c r="C35" s="40" t="s">
-        <v>100</v>
-      </c>
-      <c r="D35" s="40" t="s">
-        <v>95</v>
-      </c>
-      <c r="E35" s="40" t="s">
-        <v>101</v>
-      </c>
-      <c r="F35" s="40" t="s">
-        <v>102</v>
-      </c>
-      <c r="G35" s="41">
-        <v>2</v>
-      </c>
-      <c r="H35" s="18"/>
-      <c r="I35" s="2"/>
-      <c r="J35" s="2"/>
-      <c r="K35" s="2"/>
-      <c r="L35" s="2"/>
-      <c r="M35" s="1"/>
-    </row>
-    <row r="36" ht="19.5" customHeight="1">
-      <c r="A36" s="38" t="s">
-        <v>103</v>
-      </c>
-      <c r="B36" s="39" t="s">
-        <v>59</v>
-      </c>
-      <c r="C36" s="40" t="s">
-        <v>104</v>
-      </c>
-      <c r="D36" s="40" t="s">
+      <c r="F36" s="35" t="s">
+        <v>106</v>
+      </c>
+      <c r="G36" s="19">
+        <v>21</v>
+      </c>
+      <c r="H36" s="22">
+        <v>46166</v>
+      </c>
+      <c r="I36" s="3"/>
+      <c r="J36" s="3"/>
+      <c r="K36" s="3"/>
+      <c r="L36" s="3"/>
+      <c r="M36" s="1"/>
+      <c r="N36" s="1"/>
+    </row>
+    <row r="37" ht="19.5" customHeight="1">
+      <c r="A37" s="15"/>
+      <c r="B37" s="15"/>
+      <c r="C37" s="36"/>
+      <c r="D37" s="15"/>
+      <c r="E37" s="24"/>
+      <c r="F37" s="36"/>
+      <c r="G37" s="15"/>
+      <c r="H37" s="25"/>
+      <c r="I37" s="3"/>
+      <c r="J37" s="3"/>
+      <c r="K37" s="3"/>
+      <c r="L37" s="3"/>
+      <c r="M37" s="1"/>
+      <c r="N37" s="1"/>
+    </row>
+    <row r="38" ht="19.5" customHeight="1">
+      <c r="A38" s="10" t="s">
+        <v>107</v>
+      </c>
+      <c r="B38" s="10" t="s">
+        <v>107</v>
+      </c>
+      <c r="C38" s="10" t="s">
+        <v>108</v>
+      </c>
+      <c r="D38" s="10" t="s">
+        <v>36</v>
+      </c>
+      <c r="E38" s="10" t="s">
+        <v>12</v>
+      </c>
+      <c r="F38" s="10" t="s">
+        <v>109</v>
+      </c>
+      <c r="G38" s="14">
+        <v>34</v>
+      </c>
+      <c r="H38" s="12">
+        <v>46167</v>
+      </c>
+      <c r="I38" s="3"/>
+      <c r="J38" s="3"/>
+      <c r="K38" s="3"/>
+      <c r="L38" s="3"/>
+      <c r="M38" s="1"/>
+      <c r="N38" s="1"/>
+    </row>
+    <row r="39" ht="19.5" customHeight="1">
+      <c r="A39" s="15"/>
+      <c r="B39" s="15"/>
+      <c r="C39" s="15"/>
+      <c r="D39" s="15"/>
+      <c r="E39" s="15"/>
+      <c r="F39" s="15"/>
+      <c r="G39" s="15"/>
+      <c r="H39" s="34"/>
+      <c r="I39" s="3"/>
+      <c r="J39" s="3"/>
+      <c r="K39" s="3"/>
+      <c r="L39" s="3"/>
+      <c r="M39" s="1"/>
+      <c r="N39" s="1"/>
+    </row>
+    <row r="40" ht="19.5" customHeight="1">
+      <c r="A40" s="10" t="s">
+        <v>110</v>
+      </c>
+      <c r="B40" s="10" t="s">
+        <v>111</v>
+      </c>
+      <c r="C40" s="10" t="s">
+        <v>112</v>
+      </c>
+      <c r="D40" s="10" t="s">
         <v>105</v>
       </c>
-      <c r="E36" s="40" t="s">
-        <v>101</v>
-      </c>
-      <c r="F36" s="40" t="s">
-        <v>106</v>
-      </c>
-      <c r="G36" s="41">
-        <v>4</v>
-      </c>
-      <c r="H36" s="18"/>
-      <c r="I36" s="2"/>
-      <c r="J36" s="2"/>
-      <c r="K36" s="2"/>
-      <c r="L36" s="2"/>
-      <c r="M36" s="1"/>
-    </row>
-    <row r="37" ht="19.5" customHeight="1">
-      <c r="A37" s="21" t="s">
-        <v>107</v>
-      </c>
-      <c r="B37" s="23" t="s">
-        <v>59</v>
-      </c>
-      <c r="C37" s="23" t="s">
-        <v>108</v>
-      </c>
-      <c r="D37" s="23" t="s">
-        <v>109</v>
-      </c>
-      <c r="E37" s="23" t="s">
-        <v>33</v>
-      </c>
-      <c r="F37" s="23" t="s">
-        <v>110</v>
-      </c>
-      <c r="G37" s="22">
-        <v>2</v>
-      </c>
-      <c r="H37" s="24">
+      <c r="E40" s="10" t="s">
+        <v>12</v>
+      </c>
+      <c r="F40" s="10" t="s">
+        <v>113</v>
+      </c>
+      <c r="G40" s="19">
+        <v>17</v>
+      </c>
+      <c r="H40" s="22">
         <v>46166</v>
       </c>
-      <c r="I37" s="2"/>
-      <c r="J37" s="2"/>
-      <c r="K37" s="2"/>
-      <c r="L37" s="2"/>
-      <c r="M37" s="1"/>
-    </row>
-    <row r="38" ht="19.5" customHeight="1">
-      <c r="A38" s="38" t="s">
-        <v>111</v>
-      </c>
-      <c r="B38" s="40" t="s">
-        <v>59</v>
-      </c>
-      <c r="C38" s="40" t="s">
-        <v>112</v>
-      </c>
-      <c r="D38" s="40" t="s">
-        <v>109</v>
-      </c>
-      <c r="E38" s="40" t="s">
-        <v>101</v>
-      </c>
-      <c r="F38" s="40" t="s">
-        <v>113</v>
-      </c>
-      <c r="G38" s="41">
-        <v>2</v>
-      </c>
-      <c r="H38" s="18"/>
-      <c r="I38" s="2"/>
-      <c r="J38" s="2"/>
-      <c r="K38" s="2"/>
-      <c r="L38" s="2"/>
-      <c r="M38" s="1"/>
-    </row>
-    <row r="39" ht="19.5" customHeight="1">
-      <c r="A39" s="26"/>
-      <c r="B39" s="26"/>
-      <c r="C39" s="26"/>
-      <c r="D39" s="26"/>
-      <c r="E39" s="26"/>
-      <c r="F39" s="26"/>
-      <c r="G39" s="14"/>
-      <c r="H39" s="14"/>
-      <c r="I39" s="2"/>
-      <c r="J39" s="2"/>
-      <c r="K39" s="2"/>
-      <c r="L39" s="2"/>
-      <c r="M39" s="1"/>
-    </row>
-    <row r="40" ht="19.5" customHeight="1">
-      <c r="A40" s="22" t="s">
-        <v>114</v>
-      </c>
-      <c r="B40" s="22" t="s">
-        <v>114</v>
-      </c>
-      <c r="C40" s="42" t="s">
-        <v>115</v>
-      </c>
-      <c r="D40" s="23" t="s">
-        <v>116</v>
-      </c>
-      <c r="E40" s="23" t="s">
-        <v>33</v>
-      </c>
-      <c r="F40" s="42" t="s">
-        <v>117</v>
-      </c>
-      <c r="G40" s="22">
-        <v>21</v>
-      </c>
-      <c r="H40" s="24">
-        <v>46166</v>
-      </c>
-      <c r="I40" s="2"/>
+      <c r="I40" s="3"/>
       <c r="J40" s="1"/>
       <c r="K40" s="1"/>
       <c r="L40" s="1"/>
       <c r="M40" s="1"/>
+      <c r="N40" s="1"/>
     </row>
     <row r="41" ht="19.5" customHeight="1">
-      <c r="A41" s="14"/>
-      <c r="B41" s="14"/>
-      <c r="C41" s="43"/>
-      <c r="D41" s="14"/>
-      <c r="E41" s="26"/>
-      <c r="F41" s="43"/>
-      <c r="G41" s="14"/>
-      <c r="H41" s="14"/>
-      <c r="I41" s="2"/>
+      <c r="A41" s="10" t="s">
+        <v>114</v>
+      </c>
+      <c r="B41" s="10" t="s">
+        <v>111</v>
+      </c>
+      <c r="C41" s="10" t="s">
+        <v>115</v>
+      </c>
+      <c r="D41" s="10" t="s">
+        <v>105</v>
+      </c>
+      <c r="E41" s="10" t="s">
+        <v>12</v>
+      </c>
+      <c r="F41" s="10" t="s">
+        <v>116</v>
+      </c>
+      <c r="G41" s="19">
+        <v>17</v>
+      </c>
+      <c r="H41" s="22">
+        <v>46166</v>
+      </c>
+      <c r="I41" s="3"/>
       <c r="J41" s="1"/>
       <c r="K41" s="1"/>
       <c r="L41" s="1"/>
       <c r="M41" s="1"/>
+      <c r="N41" s="1"/>
     </row>
     <row r="42" ht="19.5" customHeight="1">
-      <c r="A42" s="16" t="s">
+      <c r="A42" s="10" t="s">
+        <v>117</v>
+      </c>
+      <c r="B42" s="10" t="s">
+        <v>111</v>
+      </c>
+      <c r="C42" s="10" t="s">
         <v>118</v>
       </c>
-      <c r="B42" s="16" t="s">
-        <v>118</v>
-      </c>
-      <c r="C42" s="16" t="s">
+      <c r="D42" s="10" t="s">
+        <v>17</v>
+      </c>
+      <c r="E42" s="10" t="s">
+        <v>12</v>
+      </c>
+      <c r="F42" s="10" t="s">
         <v>119</v>
       </c>
-      <c r="D42" s="16" t="s">
-        <v>44</v>
-      </c>
-      <c r="E42" s="16" t="s">
-        <v>23</v>
-      </c>
-      <c r="F42" s="16" t="s">
-        <v>120</v>
-      </c>
-      <c r="G42" s="20">
-        <v>34</v>
-      </c>
-      <c r="H42" s="18"/>
-      <c r="I42" s="2"/>
+      <c r="G42" s="19">
+        <v>17</v>
+      </c>
+      <c r="H42" s="22">
+        <v>46166</v>
+      </c>
+      <c r="I42" s="3"/>
       <c r="J42" s="1"/>
       <c r="K42" s="1"/>
       <c r="L42" s="1"/>
       <c r="M42" s="1"/>
+      <c r="N42" s="1"/>
     </row>
     <row r="43" ht="19.5" customHeight="1">
-      <c r="A43" s="14"/>
-      <c r="B43" s="14"/>
-      <c r="C43" s="14"/>
-      <c r="D43" s="14"/>
-      <c r="E43" s="14"/>
-      <c r="F43" s="14"/>
-      <c r="G43" s="14"/>
-      <c r="H43" s="14"/>
-      <c r="I43" s="2"/>
+      <c r="A43" s="15"/>
+      <c r="B43" s="15"/>
+      <c r="C43" s="15"/>
+      <c r="D43" s="15"/>
+      <c r="E43" s="15"/>
+      <c r="F43" s="15"/>
+      <c r="G43" s="15"/>
+      <c r="H43" s="23"/>
+      <c r="I43" s="3"/>
       <c r="J43" s="1"/>
       <c r="K43" s="1"/>
       <c r="L43" s="1"/>
       <c r="M43" s="1"/>
+      <c r="N43" s="1"/>
     </row>
     <row r="44" ht="19.5" customHeight="1">
-      <c r="A44" s="23" t="s">
+      <c r="A44" s="18" t="s">
+        <v>120</v>
+      </c>
+      <c r="B44" s="10" t="s">
         <v>121</v>
       </c>
-      <c r="B44" s="23" t="s">
+      <c r="C44" s="10" t="s">
         <v>122</v>
       </c>
-      <c r="C44" s="23" t="s">
+      <c r="D44" s="10" t="s">
         <v>123</v>
       </c>
-      <c r="D44" s="23" t="s">
-        <v>116</v>
-      </c>
-      <c r="E44" s="23" t="s">
-        <v>33</v>
-      </c>
-      <c r="F44" s="23" t="s">
+      <c r="E44" s="10" t="s">
+        <v>12</v>
+      </c>
+      <c r="F44" s="10" t="s">
         <v>124</v>
       </c>
-      <c r="G44" s="22">
-        <v>17</v>
-      </c>
-      <c r="H44" s="24">
+      <c r="G44" s="19">
+        <v>28</v>
+      </c>
+      <c r="H44" s="22">
         <v>46166</v>
       </c>
-      <c r="I44" s="2"/>
+      <c r="I44" s="3"/>
       <c r="J44" s="1"/>
       <c r="K44" s="1"/>
       <c r="L44" s="1"/>
       <c r="M44" s="1"/>
+      <c r="N44" s="1"/>
     </row>
     <row r="45" ht="19.5" customHeight="1">
-      <c r="A45" s="23" t="s">
+      <c r="A45" s="18" t="s">
         <v>125</v>
       </c>
-      <c r="B45" s="23" t="s">
-        <v>122</v>
-      </c>
-      <c r="C45" s="23" t="s">
+      <c r="B45" s="10" t="s">
+        <v>121</v>
+      </c>
+      <c r="C45" s="10" t="s">
         <v>126</v>
       </c>
-      <c r="D45" s="23" t="s">
-        <v>116</v>
-      </c>
-      <c r="E45" s="23" t="s">
-        <v>33</v>
-      </c>
-      <c r="F45" s="23" t="s">
-        <v>127</v>
-      </c>
-      <c r="G45" s="22">
-        <v>17</v>
-      </c>
-      <c r="H45" s="24">
+      <c r="D45" s="10" t="s">
+        <v>105</v>
+      </c>
+      <c r="E45" s="10" t="s">
+        <v>12</v>
+      </c>
+      <c r="F45" s="10" t="s">
+        <v>124</v>
+      </c>
+      <c r="G45" s="19">
+        <v>10</v>
+      </c>
+      <c r="H45" s="22">
         <v>46166</v>
       </c>
-      <c r="I45" s="2"/>
+      <c r="I45" s="3"/>
       <c r="J45" s="1"/>
       <c r="K45" s="1"/>
       <c r="L45" s="1"/>
       <c r="M45" s="1"/>
+      <c r="N45" s="1"/>
     </row>
     <row r="46" ht="19.5" customHeight="1">
-      <c r="A46" s="23" t="s">
+      <c r="A46" s="18" t="s">
+        <v>127</v>
+      </c>
+      <c r="B46" s="10" t="s">
+        <v>121</v>
+      </c>
+      <c r="C46" s="10" t="s">
         <v>128</v>
       </c>
-      <c r="B46" s="23" t="s">
-        <v>122</v>
-      </c>
-      <c r="C46" s="23" t="s">
-        <v>129</v>
-      </c>
-      <c r="D46" s="23" t="s">
-        <v>27</v>
-      </c>
-      <c r="E46" s="23" t="s">
-        <v>33</v>
-      </c>
-      <c r="F46" s="23" t="s">
-        <v>130</v>
-      </c>
-      <c r="G46" s="22">
+      <c r="D46" s="10" t="s">
         <v>17</v>
       </c>
-      <c r="H46" s="24">
+      <c r="E46" s="10" t="s">
+        <v>12</v>
+      </c>
+      <c r="F46" s="10" t="s">
+        <v>124</v>
+      </c>
+      <c r="G46" s="19">
+        <v>18</v>
+      </c>
+      <c r="H46" s="22">
         <v>46166</v>
       </c>
-      <c r="I46" s="2"/>
+      <c r="I46" s="3"/>
       <c r="J46" s="1"/>
       <c r="K46" s="1"/>
       <c r="L46" s="1"/>
       <c r="M46" s="1"/>
+      <c r="N46" s="1"/>
     </row>
     <row r="47" ht="19.5" customHeight="1">
-      <c r="A47" s="14"/>
-      <c r="B47" s="14"/>
-      <c r="C47" s="14"/>
-      <c r="D47" s="14"/>
-      <c r="E47" s="14"/>
-      <c r="F47" s="14"/>
-      <c r="G47" s="14"/>
-      <c r="H47" s="14"/>
-      <c r="I47" s="2"/>
+      <c r="A47" s="18" t="s">
+        <v>129</v>
+      </c>
+      <c r="B47" s="10" t="s">
+        <v>121</v>
+      </c>
+      <c r="C47" s="10" t="s">
+        <v>130</v>
+      </c>
+      <c r="D47" s="10" t="s">
+        <v>123</v>
+      </c>
+      <c r="E47" s="10" t="s">
+        <v>12</v>
+      </c>
+      <c r="F47" s="10" t="s">
+        <v>131</v>
+      </c>
+      <c r="G47" s="19">
+        <v>27</v>
+      </c>
+      <c r="H47" s="22">
+        <v>46166</v>
+      </c>
+      <c r="I47" s="3"/>
       <c r="J47" s="1"/>
       <c r="K47" s="1"/>
       <c r="L47" s="1"/>
       <c r="M47" s="1"/>
+      <c r="N47" s="1"/>
     </row>
     <row r="48" ht="19.5" customHeight="1">
-      <c r="A48" s="21" t="s">
+      <c r="A48" s="18" t="s">
+        <v>132</v>
+      </c>
+      <c r="B48" s="10" t="s">
+        <v>121</v>
+      </c>
+      <c r="C48" s="10" t="s">
+        <v>126</v>
+      </c>
+      <c r="D48" s="10" t="s">
+        <v>105</v>
+      </c>
+      <c r="E48" s="10" t="s">
+        <v>12</v>
+      </c>
+      <c r="F48" s="10" t="s">
         <v>131</v>
       </c>
-      <c r="B48" s="23" t="s">
-        <v>132</v>
-      </c>
-      <c r="C48" s="23" t="s">
-        <v>133</v>
-      </c>
-      <c r="D48" s="23" t="s">
-        <v>134</v>
-      </c>
-      <c r="E48" s="23" t="s">
-        <v>33</v>
-      </c>
-      <c r="F48" s="23" t="s">
-        <v>135</v>
-      </c>
-      <c r="G48" s="22">
-        <v>28</v>
-      </c>
-      <c r="H48" s="24">
+      <c r="G48" s="19">
+        <v>10</v>
+      </c>
+      <c r="H48" s="22">
         <v>46166</v>
       </c>
-      <c r="I48" s="2"/>
+      <c r="I48" s="3"/>
       <c r="J48" s="1"/>
       <c r="K48" s="1"/>
       <c r="L48" s="1"/>
       <c r="M48" s="1"/>
+      <c r="N48" s="1"/>
     </row>
     <row r="49" ht="19.5" customHeight="1">
-      <c r="A49" s="21" t="s">
+      <c r="A49" s="18" t="s">
+        <v>133</v>
+      </c>
+      <c r="B49" s="10" t="s">
+        <v>121</v>
+      </c>
+      <c r="C49" s="10" t="s">
+        <v>128</v>
+      </c>
+      <c r="D49" s="10" t="s">
+        <v>17</v>
+      </c>
+      <c r="E49" s="10" t="s">
+        <v>12</v>
+      </c>
+      <c r="F49" s="10" t="s">
+        <v>131</v>
+      </c>
+      <c r="G49" s="19">
+        <v>17</v>
+      </c>
+      <c r="H49" s="22">
+        <v>46166</v>
+      </c>
+    </row>
+    <row r="50" ht="19.5" customHeight="1">
+      <c r="A50" s="28"/>
+      <c r="B50" s="15"/>
+      <c r="C50" s="15"/>
+      <c r="D50" s="15"/>
+      <c r="E50" s="15"/>
+      <c r="F50" s="15"/>
+      <c r="G50" s="15"/>
+      <c r="H50" s="25"/>
+    </row>
+    <row r="51" ht="19.5" customHeight="1">
+      <c r="A51" s="10" t="s">
+        <v>134</v>
+      </c>
+      <c r="B51" s="10" t="s">
+        <v>135</v>
+      </c>
+      <c r="C51" s="10" t="s">
         <v>136</v>
       </c>
-      <c r="B49" s="23" t="s">
-        <v>132</v>
-      </c>
-      <c r="C49" s="23" t="s">
+      <c r="D51" s="10" t="s">
+        <v>17</v>
+      </c>
+      <c r="E51" s="10" t="s">
+        <v>12</v>
+      </c>
+      <c r="F51" s="10" t="s">
         <v>137</v>
       </c>
-      <c r="D49" s="23" t="s">
-        <v>116</v>
-      </c>
-      <c r="E49" s="23" t="s">
-        <v>33</v>
-      </c>
-      <c r="F49" s="23" t="s">
+      <c r="G51" s="14">
+        <v>11</v>
+      </c>
+      <c r="H51" s="12">
+        <v>46167</v>
+      </c>
+    </row>
+    <row r="52" ht="19.5" customHeight="1">
+      <c r="A52" s="10" t="s">
+        <v>138</v>
+      </c>
+      <c r="B52" s="10" t="s">
         <v>135</v>
       </c>
-      <c r="G49" s="22">
-        <v>10</v>
-      </c>
-      <c r="H49" s="24">
+      <c r="C52" s="10" t="s">
+        <v>139</v>
+      </c>
+      <c r="D52" s="10" t="s">
+        <v>140</v>
+      </c>
+      <c r="E52" s="10" t="s">
+        <v>12</v>
+      </c>
+      <c r="F52" s="10" t="s">
+        <v>141</v>
+      </c>
+      <c r="G52" s="19">
+        <v>12</v>
+      </c>
+      <c r="H52" s="33">
         <v>46166</v>
       </c>
     </row>
-    <row r="50" ht="19.5" customHeight="1">
-      <c r="A50" s="21" t="s">
-        <v>138</v>
-      </c>
-      <c r="B50" s="23" t="s">
-        <v>132</v>
-      </c>
-      <c r="C50" s="23" t="s">
-        <v>139</v>
-      </c>
-      <c r="D50" s="23" t="s">
-        <v>27</v>
-      </c>
-      <c r="E50" s="23" t="s">
-        <v>33</v>
-      </c>
-      <c r="F50" s="23" t="s">
+    <row r="53" ht="19.5" customHeight="1">
+      <c r="A53" s="10" t="s">
+        <v>142</v>
+      </c>
+      <c r="B53" s="10" t="s">
         <v>135</v>
       </c>
-      <c r="G50" s="22">
-        <v>18</v>
-      </c>
-      <c r="H50" s="24">
+      <c r="C53" s="10" t="s">
+        <v>143</v>
+      </c>
+      <c r="D53" s="10" t="s">
+        <v>53</v>
+      </c>
+      <c r="E53" s="10" t="s">
+        <v>12</v>
+      </c>
+      <c r="F53" s="10" t="s">
+        <v>144</v>
+      </c>
+      <c r="G53" s="14">
+        <v>11</v>
+      </c>
+      <c r="H53" s="12">
+        <v>46167</v>
+      </c>
+    </row>
+    <row r="54" ht="19.5" customHeight="1">
+      <c r="A54" s="15"/>
+      <c r="B54" s="15"/>
+      <c r="C54" s="15"/>
+      <c r="D54" s="15"/>
+      <c r="E54" s="15"/>
+      <c r="F54" s="15"/>
+      <c r="G54" s="15"/>
+      <c r="H54" s="34"/>
+    </row>
+    <row r="55" ht="19.5" customHeight="1">
+      <c r="A55" s="18" t="s">
+        <v>145</v>
+      </c>
+      <c r="B55" s="10" t="s">
+        <v>145</v>
+      </c>
+      <c r="C55" s="18" t="s">
+        <v>146</v>
+      </c>
+      <c r="D55" s="10" t="s">
+        <v>105</v>
+      </c>
+      <c r="E55" s="10" t="s">
+        <v>12</v>
+      </c>
+      <c r="F55" s="10" t="s">
+        <v>147</v>
+      </c>
+      <c r="G55" s="19">
+        <v>21</v>
+      </c>
+      <c r="H55" s="22">
         <v>46166</v>
       </c>
     </row>
-    <row r="51" ht="19.5" customHeight="1">
-      <c r="A51" s="21" t="s">
-        <v>140</v>
-      </c>
-      <c r="B51" s="23" t="s">
-        <v>132</v>
-      </c>
-      <c r="C51" s="23" t="s">
-        <v>141</v>
-      </c>
-      <c r="D51" s="23" t="s">
-        <v>134</v>
-      </c>
-      <c r="E51" s="23" t="s">
-        <v>33</v>
-      </c>
-      <c r="F51" s="23" t="s">
-        <v>142</v>
-      </c>
-      <c r="G51" s="22">
-        <v>27</v>
-      </c>
-      <c r="H51" s="24">
-        <v>46166</v>
-      </c>
-    </row>
-    <row r="52" ht="19.5" customHeight="1">
-      <c r="A52" s="21" t="s">
-        <v>143</v>
-      </c>
-      <c r="B52" s="23" t="s">
-        <v>132</v>
-      </c>
-      <c r="C52" s="23" t="s">
-        <v>137</v>
-      </c>
-      <c r="D52" s="23" t="s">
-        <v>116</v>
-      </c>
-      <c r="E52" s="23" t="s">
-        <v>33</v>
-      </c>
-      <c r="F52" s="23" t="s">
-        <v>142</v>
-      </c>
-      <c r="G52" s="22">
-        <v>10</v>
-      </c>
-      <c r="H52" s="24">
-        <v>46166</v>
-      </c>
-    </row>
-    <row r="53" ht="19.5" customHeight="1">
-      <c r="A53" s="21" t="s">
-        <v>144</v>
-      </c>
-      <c r="B53" s="23" t="s">
-        <v>132</v>
-      </c>
-      <c r="C53" s="23" t="s">
-        <v>139</v>
-      </c>
-      <c r="D53" s="23" t="s">
-        <v>27</v>
-      </c>
-      <c r="E53" s="23" t="s">
-        <v>33</v>
-      </c>
-      <c r="F53" s="23" t="s">
-        <v>142</v>
-      </c>
-      <c r="G53" s="22">
-        <v>17</v>
-      </c>
-      <c r="H53" s="24">
-        <v>46166</v>
-      </c>
-    </row>
-    <row r="54" ht="19.5" customHeight="1">
-      <c r="A54" s="13"/>
-      <c r="B54" s="14"/>
-      <c r="C54" s="14"/>
-      <c r="D54" s="14"/>
-      <c r="E54" s="14"/>
-      <c r="F54" s="14"/>
-      <c r="G54" s="14"/>
-      <c r="H54" s="14"/>
-    </row>
-    <row r="55" ht="19.5" customHeight="1">
-      <c r="A55" s="16" t="s">
-        <v>145</v>
-      </c>
-      <c r="B55" s="16" t="s">
-        <v>146</v>
-      </c>
-      <c r="C55" s="16" t="s">
-        <v>147</v>
-      </c>
-      <c r="D55" s="16" t="s">
-        <v>27</v>
-      </c>
-      <c r="E55" s="16" t="s">
-        <v>23</v>
-      </c>
-      <c r="F55" s="16" t="s">
+    <row r="56" ht="19.5" customHeight="1">
+      <c r="A56" s="37" t="s">
         <v>148</v>
       </c>
-      <c r="G55" s="20">
-        <v>11</v>
-      </c>
-      <c r="H55" s="18"/>
-    </row>
-    <row r="56" ht="19.5" customHeight="1">
-      <c r="A56" s="23" t="s">
-        <v>149</v>
-      </c>
-      <c r="B56" s="23" t="s">
-        <v>146</v>
-      </c>
-      <c r="C56" s="23" t="s">
-        <v>150</v>
-      </c>
-      <c r="D56" s="23" t="s">
-        <v>151</v>
-      </c>
-      <c r="E56" s="23" t="s">
-        <v>33</v>
-      </c>
-      <c r="F56" s="23" t="s">
-        <v>152</v>
-      </c>
-      <c r="G56" s="22">
-        <v>12</v>
-      </c>
-      <c r="H56" s="24">
-        <v>46166</v>
+      <c r="B56" s="38"/>
+      <c r="C56" s="38"/>
+      <c r="D56" s="38"/>
+      <c r="E56" s="38"/>
+      <c r="F56" s="39"/>
+      <c r="G56" s="40">
+        <f>SUM(G2,G3,G5,G11,G13,G15,G19,G20,G21,G22,G23,G24,G25,G26,G27,G28,G29,G30,G31,G32,G33,G34,G36,G38,G40,G42,G44,G47,G51,G52,G53,G55)</f>
+        <v>419</v>
       </c>
     </row>
     <row r="57" ht="19.5" customHeight="1">
-      <c r="A57" s="16" t="s">
-        <v>153</v>
-      </c>
-      <c r="B57" s="16" t="s">
-        <v>146</v>
-      </c>
-      <c r="C57" s="16" t="s">
-        <v>154</v>
-      </c>
-      <c r="D57" s="16" t="s">
-        <v>61</v>
-      </c>
-      <c r="E57" s="16" t="s">
-        <v>23</v>
-      </c>
-      <c r="F57" s="16" t="s">
-        <v>155</v>
-      </c>
-      <c r="G57" s="20">
-        <v>11</v>
-      </c>
-      <c r="H57" s="18"/>
+      <c r="G57" s="1"/>
     </row>
     <row r="58" ht="19.5" customHeight="1">
-      <c r="A58" s="14"/>
-      <c r="B58" s="14"/>
-      <c r="C58" s="14"/>
-      <c r="D58" s="14"/>
-      <c r="E58" s="14"/>
-      <c r="F58" s="14"/>
-      <c r="G58" s="14"/>
-      <c r="H58" s="14"/>
-    </row>
-    <row r="59" ht="19.5" customHeight="1">
-      <c r="A59" s="21" t="s">
-        <v>156</v>
-      </c>
-      <c r="B59" s="23" t="s">
-        <v>156</v>
-      </c>
-      <c r="C59" s="21" t="s">
-        <v>157</v>
-      </c>
-      <c r="D59" s="23" t="s">
-        <v>116</v>
-      </c>
-      <c r="E59" s="23" t="s">
-        <v>33</v>
-      </c>
-      <c r="F59" s="23" t="s">
-        <v>158</v>
-      </c>
-      <c r="G59" s="22">
-        <v>21</v>
-      </c>
-      <c r="H59" s="24">
-        <v>46166</v>
-      </c>
+      <c r="G58" s="1"/>
     </row>
     <row r="60" ht="19.5" customHeight="1">
-      <c r="A60" s="44" t="s">
-        <v>159</v>
-      </c>
-      <c r="B60" s="45"/>
-      <c r="C60" s="45"/>
-      <c r="D60" s="45"/>
-      <c r="E60" s="45"/>
-      <c r="F60" s="46"/>
-      <c r="G60" s="14">
-        <f>SUM(G5,G6,G8,G14,G16,G18,G22,G23,G24,G25,G26,G27,G28,G29,G30,G31,G32,G34,G35,G36,G37,G38,G40,G42,G44,G46,G48,G51,G55,G56,G57,G59)</f>
-        <v>419</v>
-      </c>
+      <c r="G60" s="1"/>
       <c r="H60" s="2"/>
     </row>
     <row r="61" ht="19.5" customHeight="1">
@@ -4427,45 +4563,45 @@
       <c r="H63" s="2"/>
     </row>
     <row r="64" ht="19.5" customHeight="1">
-      <c r="A64" s="2"/>
-      <c r="B64" s="2"/>
-      <c r="C64" s="2"/>
-      <c r="D64" s="2"/>
-      <c r="E64" s="2"/>
-      <c r="F64" s="2"/>
-      <c r="G64" s="2"/>
+      <c r="A64" s="3"/>
+      <c r="B64" s="3"/>
+      <c r="C64" s="3"/>
+      <c r="D64" s="3"/>
+      <c r="E64" s="3"/>
+      <c r="F64" s="3"/>
+      <c r="G64" s="3"/>
     </row>
     <row r="65" ht="19.5" customHeight="1">
-      <c r="A65" s="2"/>
-      <c r="B65" s="2"/>
-      <c r="C65" s="2"/>
-      <c r="D65" s="2"/>
-      <c r="E65" s="2"/>
-      <c r="F65" s="2"/>
+      <c r="A65" s="3"/>
+      <c r="B65" s="3"/>
+      <c r="C65" s="3"/>
+      <c r="D65" s="3"/>
+      <c r="E65" s="3"/>
+      <c r="F65" s="3"/>
       <c r="G65" s="1"/>
     </row>
     <row r="66" ht="19.5" customHeight="1">
-      <c r="A66" s="2"/>
-      <c r="B66" s="2"/>
-      <c r="C66" s="2"/>
-      <c r="D66" s="2"/>
-      <c r="E66" s="2"/>
-      <c r="F66" s="2"/>
+      <c r="A66" s="3"/>
+      <c r="B66" s="3"/>
+      <c r="C66" s="3"/>
+      <c r="D66" s="3"/>
+      <c r="E66" s="3"/>
+      <c r="F66" s="3"/>
       <c r="H66" s="2"/>
     </row>
     <row r="67" ht="19.5" customHeight="1">
-      <c r="A67" s="2"/>
-      <c r="B67" s="2"/>
-      <c r="C67" s="2"/>
-      <c r="D67" s="2"/>
-      <c r="E67" s="2"/>
-      <c r="F67" s="2"/>
+      <c r="A67" s="3"/>
+      <c r="B67" s="3"/>
+      <c r="C67" s="3"/>
+      <c r="D67" s="3"/>
+      <c r="E67" s="3"/>
+      <c r="F67" s="3"/>
       <c r="G67" s="1"/>
     </row>
   </sheetData>
   <mergeCells count="2">
     <mergeCell ref="J2:L2"/>
-    <mergeCell ref="A60:F60"/>
+    <mergeCell ref="A56:F56"/>
   </mergeCells>
   <printOptions headings="0" gridLines="0"/>
   <pageMargins left="0.511811024" right="0.511811024" top="0.78740157500000008" bottom="0.78740157500000008" header="0.31496062000000014" footer="0.31496062000000014"/>

</xml_diff>